<commit_message>
fix(ch10): display LaTeX formatting in solutions, exact homework 10 numerical calibration, KaTeX copy-paste scrambling fix, and search bar card ID support
</commit_message>
<xml_diff>
--- a/FunE_Master_Exam_Flashcards_Ch6_10_Master.xlsx
+++ b/FunE_Master_Exam_Flashcards_Ch6_10_Master.xlsx
@@ -1739,26 +1739,28 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Right-hand solenoid rule:
-Fingers = Current curl, Thumb = North Pole (N)</t>
+          <t>$$\text{Right-Hand Solenoid Rule: Fingers} \rightarrow \vec{I}_{\text{curl}}, \quad \text{Thumb} \rightarrow \text{North Pole (N)}$$
+$$\vec{F} = I (\vec{L} \times \vec{B})$$</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>1. The two essential parts are:
-- Stator (ส่วนที่อยู่กับที่ - stationary field frame)
-- Rotor / Armature (ส่วนที่หมุนเคลื่อนที่ - rotating part)
+- Stator (ส่วนที่อยู่กับที่): Stationary field frame providing magnetic flux $\vec{B}$.
+- Rotor / Armature (ส่วนที่หมุนเคลื่อนที่): Rotating shaft carrying current coils that generate torque $\vec{\tau}$.
 2. Solenoid Pole Identification:
-Using the right-hand coil rule, curl four fingers in the direction current wraps around the iron pole pieces. The thumb points toward the North pole (where magnetic flux emerges).</t>
+Using the right-hand coil rule, curl four fingers in the direction current wraps around the iron pole pieces. The thumb points toward the North pole (N) where magnetic flux emerges:
+$$\text{Current direction: } \vec{I} \implies \text{Magnetic dipole: } \vec{m} \parallel \text{Thumb (N)}$$</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>1. โครงสร้างหลัก 2 ส่วนของมอเตอร์:
-- Stator (ส่วนที่อยู่กับที่ สร้างสนามแม่เหล็กหลัก)
-- Rotor หรือ Armature (ส่วนที่หมุน ตัดกับเส้นแรงแม่เหล็ก)
+- Stator (ส่วนที่อยู่กับที่): สร้างสนามแม่เหล็กหลัก $\vec{B}$
+- Rotor หรือ Armature (ส่วนที่หมุน): ตัดกับเส้นแรงแม่เหล็กเพื่อสร้างแรงบิดหมุน $\vec{\tau}$
 2. การระบุขั้วแม่เหล็ก N-S:
-ใช้กฎมือขวาสำหรับโซเลนอยด์ (กำมือขวานิ้วทั้งสี่ตามทิศทางกระแสที่พันรอบแกนเหล็ก) นิ้วหัวแม่มือจะชี้ไปยังทิศทางของขั้วเหนือ (N Pole) เสมอ</t>
+ใช้กฎมือขวาสำหรับโซเลนอยด์ (กำมือนิ้วทั้งสี่ตามทิศทางกระแส $\vec{I}$ ที่พันรอบแกนเหล็ก) นิ้วหัวแม่มือจะชี้ไปยังทิศทางของขั้วเหนือ (N Pole) ที่เส้นแรงแม่เหล็กพุ่งออกเสมอ:
+$$\text{ทิศทางกระแส: } \vec{I} \implies \text{ขั้วเหนือ (N Pole): ตามทิศนิ้วหัวแม่มือ}$$</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -3883,7 +3885,7 @@
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>$$\frac{S_{\text{auto}}}{S_{\text{2-w}}} = \frac{1}{1 - 1/a_{\text{auto}}}$$
-Conducted power + Transformed power</t>
+$$S_{\text{auto}} = S_{\text{conducted}} + S_{\text{transformed}}$$</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -3892,9 +3894,11 @@
 An auto-transformer has a SINGLE continuous winding shared partly by both primary and secondary circuits (tapped common winding).
 2. Higher Rating &amp; Efficiency:
 Power is transferred via two mechanisms simultaneously:
-- By electromagnetic induction (transformed power)
-- By direct electrical conduction (conducted power)
-Because part of the energy flows conductively through the shared copper, magnetic core and windings can be much smaller and lighter, with lower $I^2 R$ and core losses.
+- By direct electrical conduction ($S_{\text{conducted}} = V_2 I_1$)
+- By electromagnetic induction ($S_{\text{transformed}} = V_2 (I_2 - I_1)$)
+Because a large fraction of power flows conductively without transforming through magnetic flux:
+$$\frac{S_{\text{auto}}}{S_{\text{2-w}}} = \frac{1}{1 - 1/a} &gt; 1$$
+Core and windings are much smaller, dramatically lowering $I^2 R$ heat loss and core losses.
 3. Safety Drawback:
 NO ELECTRICAL ISOLATION between primary (HV) and secondary (LV)! If the common ground connection opens, the full high voltage appears directly on the low voltage terminals, risking electrocution.</t>
         </is>
@@ -3904,7 +3908,10 @@
           <t>1. โครงสร้างและหลักการ:
 หม้อแปลงออโต้มี 'ขดลวดเพียงขดเดียว' พันบนแกนเหล็ก โดยขดลวดปฐมภูมิและทุติยภูมิจะใช้เนื้อขดลวดส่วนหนึ่งร่วมกัน (Common Winding)
 2. พิกัดและประสิทธิภาพที่สูงกว่า:
-ส่งถ่ายพลังงานได้ 2 ทางพร้อมกัน คือ ทางการเหนี่ยวนำแม่เหล็ก และ ทางการนำไฟฟ้าโดยตรง (Conduction) ทำให้ประหยัดขนาดแกนเหล็กและทองแดง มีการสูญเสียต่ำกว่ามาก
+ส่งถ่ายพลังงานได้ 2 ทางพร้อมกัน คือ ทางการนำไฟฟ้าโดยตรง ($S_{\text{conducted}}$) และทางการเหนี่ยวนำแม่เหล็ก ($S_{\text{transformed}}$):
+$$S_{\text{auto}} = S_{\text{conducted}} + S_{\text{transformed}}$$
+$$\frac{S_{\text{auto}}}{S_{\text{2-w}}} = \frac{1}{1 - 1/a} &gt; 1$$
+ทำให้ประหยัดขนาดแกนเหล็กและทองแดง มีการสูญเสียความร้อน $I^2 R$ และการสูญเสียในแกนเหล็กต่ำกว่ามาก
 3. ข้อเสียร้ายแรงด้านความปลอดภัย:
 'ไม่มีการแยกทางไฟฟ้าระหว่างขดลวด (No Galvanic Isolation)' ด้านแรงดันสูงและแรงดันต่ำเชื่อมถึงกันโดยตรง หากขดลวดร่วมขาด แรงดันสูงจากฝั่งปฐมภูมิจะรั่วข้ามไปยังฝั่งทุติยภูมิทันที</t>
         </is>
@@ -3972,40 +3979,46 @@
         <is>
           <t>$$\text{Stages: Generation } \rightarrow \text{ Transmission } \rightarrow \text{ Distribution } \rightarrow \text{ Utilization}$$
 $$P = \sqrt{3} V_L I_L \cos\theta \implies I_L = \frac{P}{\sqrt{3} V_L \cos\theta}$$
-$$P_{\text{loss}} = 3 I_L^2 R_{\text{line}} \propto \frac{1}{V_L^2}$$</t>
+$$P_{\text{loss}} = 3 I_L^2 R_{\text{line}} = \frac{P^2 R_{\text{line}}}{V_L^2 \cos^2\theta} \propto \frac{1}{V_L^2}$$</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
           <t>1. Four Stages of Power System:
-- Generation: 10 - 20 kV (alternator output terminals)
-- Transmission: 115 kV, 230 kV, 500 kV (long-distance bulk power transfer)
-- Distribution: 22 kV, 24 kV, 33 kV (medium voltage to substations and streets)
-- Utilization: 380 V (3-phase) / 220 V (1-phase) (end consumers)
-2. Voltage Classifications for Exam:
-- 500 kV: Extra High Voltage (EHV)
-- 22 kV: Medium Voltage (MV) - standard PEA/MEA primary distribution
-- 380 V: Low Voltage (LV) - standard 3-phase line-to-line utilization
-- Household: 220 V (or modern 230 V) - single-phase line-to-neutral utilization.</t>
+- Generation (การผลิต): $10\text{ kV} - 20\text{ kV}$ at power station alternators.
+- Transmission (สายส่งไฟฟ้า): $115\text{ kV}, 230\text{ kV}, 500\text{ kV}$ bulk long-distance power wheeling.
+- Distribution (สายจำหน่าย): $22\text{ kV}$ (PEA), $24\text{ kV} / 12\text{ kV}$ (MEA), $33\text{ kV}$ primary street feeders.
+- Utilization (การใช้ไฟฟ้า): $380\text{ V}$ (3-phase) / $220\text{ V}$ (single-phase) end customers.
+2. Voltage Level Classifications:
+- $500\text{ kV}$: Extra High Voltage (EHV)
+- $22\text{ kV}$: Medium Voltage (MV) - standard PEA distribution
+- $380\text{ V}$: Low Voltage (LV) - standard 3-phase line-to-line
+- Household: $220\text{ V}$ (or modern $230\text{ V}$) - single-phase line-to-neutral.
+3. Line Loss Scaling:
+$$P_{\text{loss}} = 3 I_L^2 R_{\text{line}} \propto \frac{1}{V_L^2}$$
+Stepping up voltage by a factor of 10 reduces line current by 10 and line losses by a factor of 100.</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
           <t>1. 4 ขั้นตอนหลักของระบบไฟฟ้ากำลัง:
-- การผลิต (Generation): 10 - 20 kV (แรงดันออกจากเครื่องกำเนิดไฟฟ้า)
-- สายส่งไฟฟ้า (Transmission): 115 kV, 230 kV, 500 kV (ส่งพลังงานระยะไกลข้ามภาค)
-- สายจำหน่าย (Distribution): 22 kV (กฟภ.), 24 kV / 12 kV (กฟน.), 33 kV (จ่ายเข้าเสาไฟหน้าบ้าน/หม้อแปลงชุมชน)
-- การใช้ไฟฟ้า (Utilization): 380 V (3 เฟส) / 220 V (1 เฟส) (จ่ายเข้าอุปกรณ์ไฟฟ้าผู้ใช้)
+- การผลิต (Generation): แรงดัน $10\text{ kV} - 20\text{ kV}$ ผลิตจากเครื่องกำเนิดไฟฟ้าในโรงไฟฟ้า
+- สายส่งไฟฟ้า (Transmission): แรงดัน $115\text{ kV}, 230\text{ kV}, 500\text{ kV}$ ส่งพลังงานระยะไกลข้ามภาค
+- สายจำหน่าย (Distribution): แรงดัน $22\text{ kV}$ (กฟภ.), $24\text{ kV} / 12\text{ kV}$ (กฟน.), $33\text{ kV}$ จ่ายตามแนวถนนเข้าสู่หม้อแปลงชุมชน
+- การใช้ไฟฟ้า (Utilization): แรงดัน $380\text{ V}$ (3 เฟส) / $220\text{ V}$ (1 เฟส) จ่ายเข้าอุปกรณ์ไฟฟ้าผู้ใช้
 2. จัดกลุ่มระดับแรงดันตามโจทย์ข้อสอบ:
-- 500 kV: แรงดันสูงพิเศษ (Extra High Voltage: EHV)
-- 22 kV: แรงดันปานกลาง (Medium Voltage: MV) - สายป้อนหลักของ กฟภ.
-- 380 V: แรงดันต่ำ (Low Voltage: LV) - ไฟฟ้า 3 เฟสในโรงงาน/อาคาร
-- แรงดันไฟบ้าน: 220 V (หรือมาตรฐานใหม่ 230 V) - ไฟฟ้า 1 เฟสใช้งานทั่วไป</t>
+- $500\text{ kV}$: แรงดันสูงพิเศษ (Extra High Voltage: EHV)
+- $22\text{ kV}$: แรงดันปานกลาง (Medium Voltage: MV) - สายป้อนหลักของ กฟภ.
+- $380\text{ V}$: แรงดันต่ำ (Low Voltage: LV) - ไฟฟ้า 3 เฟสในโรงงานและอาคาร
+- แรงดันไฟบ้าน: $220\text{ V}$ (หรือ $230\text{ V}$) - ไฟฟ้า 1 เฟสใช้งานทั่วไป
+3. การลดการสูญเสียในสายส่ง:
+$$P_{\text{loss}} = 3 I_L^2 R_{\text{line}} \propto \frac{1}{V_L^2}$$
+เมื่อเพิ่มแรงดันส่ง $V_L$ กระแส $I_L$ จะลดลง ทำให้การสูญเสียความร้อนลดลงอย่างมหาศาลตามสัดส่วน $(1/V_L^2)$</t>
         </is>
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>Why transmit at Extra High Voltage (500 kV)? Because stepping up VL reduces line current IL proportionally, which decreases transmission line I^2 R loss by a factor of (1/V)^2.</t>
+          <t>Why transmit at 500 kV? Because stepping up VL reduces line current IL proportionally, which decreases I^2 R line loss by a factor of (1/V)^2.</t>
         </is>
       </c>
       <c r="M39" s="5" t="inlineStr">
@@ -4072,29 +4085,35 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>$$\text{EGAT: Generation + High-Voltage Grid (Nationwide)}$$
-$$\text{MEA: Distribution in 3 Provinces (BKK, Nonthaburi, Samut Prakan)}$$
-$$\text{PEA: Distribution in 74 Provinces (All other provinces)}$$</t>
+          <t>$$\text{EGAT: Generation + High-Voltage Transmission Grid (Nationwide)}$$
+$$\text{MEA: Retail Distribution in 3 Provinces (Bangkok, Nonthaburi, Samut Prakan)}$$
+$$\text{PEA: Retail Distribution in 74 Provinces (All other regions)}$$</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
           <t>1. EGAT (Electricity Generating Authority of Thailand / กฟผ.):
-Responsible for bulk power generation (hydro, thermal, combined cycle) and the nationwide high-voltage transmission grid (115 kV - 500 kV). Sells wholesale electricity to MEA, PEA, and large direct industrial customers.
+- Responsibilities: Bulk power generation and high-voltage transmission grid ($115\text{ kV} - 500\text{ kV}$) across the entire nation.
+- Sells wholesale electricity to MEA, PEA, and large direct industrial customers.
 2. MEA (Metropolitan Electricity Authority / กฟน.):
-Responsible for electricity distribution and retail customer service strictly across 3 provinces: Bangkok, Nonthaburi, and Samut Prakan.
+- Responsibilities: Retail electricity distribution and customer service.
+- Jurisdiction: Strictly 3 provinces: Bangkok, Nonthaburi, and Samut Prakan.
 3. PEA (Provincial Electricity Authority / กฟภ.):
-Responsible for electricity distribution and retail customer service across all remaining 74 provinces of Thailand.</t>
+- Responsibilities: Retail electricity distribution and customer service.
+- Jurisdiction: All remaining 74 provinces across Thailand.</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
           <t>1. กฟผ. (EGAT - การไฟฟ้าฝ่ายผลิตแห่งประเทศไทย):
-มีหน้าที่ผลิตพลังงานไฟฟ้า (เขื่อน, โรงไฟฟ้าถ่านหิน, ก๊าซธรรมชาติ) และบริหารโครงข่ายสายส่งไฟฟ้าแรงสูงทั่วประเทศ (115 kV - 500 kV) โดยขายส่งไฟฟ้าให้ กฟน., กฟภ. และผู้ใช้อุตสาหกรรมรายใหญ่ตรง
+- หน้าที่: ผลิตพลังงานไฟฟ้า (เขื่อน, โรงไฟฟ้าถ่านหิน, ก๊าซธรรมชาติ) และบริหารระบบโครงข่ายสายส่งไฟฟ้าแรงสูงทั่วประเทศ ($115\text{ kV} - 500\text{ kV}$)
+- ขายส่งไฟฟ้าให้แก่ กฟน., กฟภ. และผู้ใช้อุตสาหกรรมขนาดใหญ่โดยตรง
 2. กฟน. (MEA - การไฟฟ้านครหลวง):
-มีหน้าที่จัดจำหน่ายไฟฟ้าและให้บริการผู้ใช้ไฟในพื้นที่เฉพาะ 3 จังหวัด ได้แก่ กรุงเทพมหานคร, นนทบุรี และสมุทรปราการ
+- หน้าที่: จัดจำหน่ายไฟฟ้าและดูแลระบบสายจำหน่ายแก่ผู้ใช้ไฟ
+- พื้นที่รับผิดชอบ: เฉพาะ 3 จังหวัดเท่านั้น คือ กรุงเทพมหานคร, นนทบุรี และสมุทรปราการ
 3. กฟภ. (PEA - การไฟฟ้าส่วนภูมิภาค):
-มีหน้าที่จัดจำหน่ายไฟฟ้าและดูแลระบบสายจำหน่ายในพื้นที่ 74 จังหวัดที่เหลือทั่วประเทศ</t>
+- หน้าที่: จัดจำหน่ายไฟฟ้าและดูแลระบบสายจำหน่ายแก่ผู้ใช้ไฟ
+- พื้นที่รับผิดชอบ: 74 จังหวัดที่เหลือทั่วประเทศไทย</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
@@ -4159,28 +4178,28 @@
       <c r="I41" s="5" t="inlineStr">
         <is>
           <t>$$\text{Primary / Most Used: Natural Gas (ก๊าซธรรมชาติ) } \approx 55\% - 60\%$$
-$$\text{Second: Coal / Lignite (ถ่านหินลิกไนต์) } + \text{ Imported Hydro (สปป.ลาว)}$$
+$$\text{Second: Coal / Lignite (ถ่านหินลิกไนต์) } \approx 15\% - 18\% + \text{Imported Hydro } \approx 12\% - 15\%$$
 $$\text{Least Used: Heavy Fuel Oil / Diesel (น้ำมันเตา/ดีเซล) } &lt; 1\%$$</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>1. Most Used Fuel:
-Natural Gas (ก๊าซธรรมชาติ) generates over 55-60% of total electrical energy in Thailand, supplied from the Gulf of Thailand, Myanmar pipelines, and imported Liquefied Natural Gas (LNG).
-2. Secondary Sources:
-Coal / Lignite (ถ่านหินลิกไนต์ แม่เมาะ) and imported hydropower from Lao PDR.
+          <t>1. Most Heavily Used Fuel:
+Natural Gas (ก๊าซธรรมชาติ) accounts for over $55\% - 60\%$ of total electricity generation in Thailand, sourced from the Gulf of Thailand, Myanmar pipelines, and imported Liquefied Natural Gas (LNG).
+2. Secondary Fuels:
+Coal / Lignite (ถ่านหินลิกไนต์ที่แม่เมาะ) and imported hydropower from Lao PDR.
 3. Least Used Fuel:
-Heavy fuel oil (น้ำมันเตา) and diesel, utilized only as emergency backup during gas pipeline maintenance due to exceptionally high operating costs and particulate emissions.</t>
+Heavy fuel oil (น้ำมันเตา) and diesel ($&lt; 1\%$), used strictly as emergency standby when gas pipelines undergo planned maintenance due to extremely high operating costs.</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
           <t>1. เชื้อเพลิงที่ใช้มากที่สุด:
-ก๊าซธรรมชาติ (Natural Gas) ครองสัดส่วนมากกว่า 55-60% ของการผลิตไฟฟ้าทั้งหมดในไทย (มาจากอ่าวไทย, ท่อส่งพม่า และการนำเข้า LNG)
+ก๊าซธรรมชาติ (Natural Gas) ครองสัดส่วนมากกว่า $55\% - 60\%$ ของการผลิตไฟฟ้าทั้งหมดในไทย (มาจากอ่าวไทย, ท่อส่งพม่า และการนำเข้า LNG)
 2. เชื้อเพลิงรองลงมา:
-ถ่านหิน/ลิกไนต์ (Coal/Lignite ที่โรงไฟฟ้าแม่เมาะ) และการซื้อพลังน้ำนำเข้าจาก สปป.ลาว
+ถ่านหิน/ลิกไนต์ (Coal/Lignite ที่โรงไฟฟ้าแม่เมาะ $\approx 16\%$) และการซื้อพลังน้ำนำเข้าจาก สปป.ลาว ($\approx 13\%$)
 3. เชื้อเพลิงที่ใช้น้อยที่สุด:
-น้ำมันเตา (Heavy Fuel Oil) และน้ำมันดีเซล ซึ่งใช้ไม่ถึง 1% โดยจะเดินเครื่องเฉพาะช่วงฉุกเฉินหรือซ่อมบำรุงท่อก๊าซเท่านั้นเนื่องจากมีต้นทุนต่อหน่วยสูงมากและปล่อยมลพิษสูง</t>
+น้ำมันเตา (Heavy Fuel Oil) และน้ำมันดีเซล ซึ่งใช้ไม่ถึง $1\%$ โดยจะเดินเครื่องเฉพาะช่วงฉุกเฉินหรือซ่อมบำรุงท่อก๊าซเท่านั้นเนื่องจากมีต้นทุนต่อหน่วยสูงมาก</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -4244,20 +4263,22 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>$$\text{Base Load: Continuous 24/7 operation, High Capital Cost, Low Fuel/Operating Cost}$$
-$$\text{Peak Load: Fast Startup (minutes), Low Capital Cost, High Fuel/Operating Cost}$$</t>
+          <t>$$\text{Base Load: 24/7 continuous, High Capital Cost, Low Fuel Cost/kWh, Startup: Hours to Days}$$
+$$\text{Peak Load: Fast Startup (3-15 min), Lower Capital Cost, High Fuel Cost/kWh}$$</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
           <t>1. Base Load Power Plants:
-- Purpose: Run continuously 24 hours a day at rated constant capacity to meet baseline national demand.
+- Objective: Operate continuously 24 hours a day at rated steady capacity to supply baseline grid demand.
 - Plant Types: Coal/Lignite Thermal Plants (Mae Moh), Nuclear, Combined-Cycle Gas Turbine (CCGT).
-- Characteristics: Very high capital construction cost, low fuel/operating cost per kWh, very slow startup time (hours to days from cold start).
+- Economics: Very high capital cost, lowest operating cost per kWh.
+- Startup Time: Very slow (hours to days from cold condition).
 2. Peak Load Power Plants:
-- Purpose: Operated temporarily during peak demand hours (typically hot weekday afternoons and early evenings) and sudden grid disturbances.
+- Objective: Dispatched briefly during peak demand hours (hot afternoons, early evenings) and sudden grid disturbances.
 - Plant Types: Gas Turbines (Open Cycle), Pumped-Storage Hydro (เขื่อนลำตะคองชลภาวัฒนา), Conventional Hydro.
-- Characteristics: Lower capital investment, high fuel operating cost per kWh, extremely fast startup time (starts and synchronizes to grid in 3 - 15 minutes).</t>
+- Economics: Lower capital investment, high fuel cost per kWh.
+- Startup Time: Extremely fast ($3 - 15\text{ minutes}$ from stop to full synchronized generation).</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -4265,11 +4286,12 @@
           <t>1. โรงไฟฟ้าฐาน (Base Load Power Plant):
 - วัตถุประสงค์: เดินเครื่องผลิตไฟฟ้าคงที่ต่อเนื่องตลอด 24 ชั่วโมงเพื่อรองรับความต้องการไฟฟ้าขั้นต่ำของประเทศ
 - ประเภทโรงไฟฟ้า: โรงไฟฟ้าพลังความร้อนถ่านหิน (แม่เมาะ), นิวเคลียร์, โรงไฟฟ้าพลังความร้อนร่วม (Combined Cycle)
-- จุดเด่น: ค่าก่อสร้างสูงมาก (High Capital Cost) แต่ต้นทุนค่าเชื้อเพลิงต่อหน่วยต่ำมาก, สตาร์ทเครื่องช้า (ใช้เวลาหลายชั่วโมงถึงเป็นวัน)
+- จุดเด่น: ค่าก่อสร้างสูงมาก (High Capital Cost) แต่ต้นทุนค่าเชื้อเพลิงต่อหน่วยต่ำมาก
+- เวลาสตาร์ทเครื่อง: ช้ามาก (ใช้เวลาหลายชั่วโมงถึงเป็นวันจากสถานะเครื่องเย็น)
 2. โรงไฟฟ้ารับโหลดสูงสุด (Peak Load Power Plant):
-- วัตถุประสงค์: เดินเครื่องเฉพาะช่วงเวลาที่มีการใช้ไฟฟ้าสูงสุด (เช่น บ่ายวันทำงานที่อากาศร้อนจัด หรือช่วงค่ำ) และช่วงฉุกเฉิน
+- วัตถุประสงค์: เดินเครื่องเฉพาะช่วงเวลาที่มีการใช้ไฟฟ้าสูงสุด (Peak Hours) เช่น ช่วงบ่ายวันทำงาน หรือช่วงค่ำ
 - ประเภทโรงไฟฟ้า: กังหันก๊าซเดี่ยว (Gas Turbine), พลังน้ำสูบกลับ (เขื่อนลำตะคอง), โรงไฟฟ้าพลังน้ำ
-- จุดเด่น: สตาร์ทเครื่องได้เร็วมาก (Fast Startup ภายใน 3 - 15 นาที), ค่าก่อสร้างต่ำกว่า แต่ต้นทุนเชื้อเพลิงต่อหน่วยสูง</t>
+- จุดเด่น: สตาร์ทเครื่องได้เร็วมาก (Fast Startup ภายใน $3 - 15\text{ นาที}$), ค่าก่อสร้างต่ำกว่า แต่ต้นทุนเชื้อเพลิงต่อหน่วยสูง</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -4342,21 +4364,21 @@
       <c r="I43" s="5" t="inlineStr">
         <is>
           <t>$$\text{Suspension: Straight paths, supports vertical conductor weight}$$
-$$\text{Tension / Angle: Turns/corners, withstands directional pull tension}$$
-$$\text{Dead-end: Terminal stations, handles one-sided full mechanical tension}$$
-$$\text{Transposition: Balances mutual inductance } L_{12} = L_{23} = L_{31} \text{ and capacitance across 3 phases}$$</t>
+$$\text{Tension / Angle: Path turns, withstands directional pull tension}$$
+$$\text{Dead-end: Line termination at substations, handles full unilateral tension}$$
+$$\text{Transposition: Equalizes phase inductances } L_{12} = L_{23} = L_{31} \text{ and capacitances}$$</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
           <t>1. Suspension Towers (เสาแขวน):
-Used along straight line routes. Insulators hang vertically downwards to support only the physical downward weight of conductors without taking longitudinal line tension.
+Used along straight line routes. Insulator strings hang vertically downward to support only the physical downward weight of conductors without taking longitudinal line tension.
 2. Tension / Angle Towers (เสารั้ง / เสามุม):
-Installed where transmission line changes direction (curves/corners). Insulators are placed horizontally in tension to withstand the horizontal mechanical pulling vector.
+Installed where transmission line changes direction (curves/corners). Insulator strings are positioned horizontally under tension to withstand the horizontal resultant mechanical pulling force.
 3. Dead-end / Terminal Towers (เสาสิ้นสุด):
-Placed where the line terminates at a substation or crosses major obstacles (wide rivers, mountains). Engineered to withstand the full, unbalanced tension from one side.
-4. Transposition Towers (เสาสลับเฟส):
-Swaps physical conductor positions at regular 1/3 distance intervals to equalize line inductances and capacitances, balancing phase voltages.</t>
+Placed where the line terminates at a substation or crosses major obstacles (wide rivers, mountain passes). Engineered to withstand full, unbalanced mechanical tension from one side.
+4. Transposition Towers (เสาสลับตำแหน่งเฟส):
+Swaps conductor positions (A, B, C) at regular $1/3$ line distance intervals to equalize line mutual inductances and capacitances across all 3 phases, preventing voltage unbalance.</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
@@ -4368,7 +4390,7 @@
 3. เสาสิ้นสุด (Dead-end / Terminal Tower):
 ใช้บริเวณปลายสุดของสายส่งก่อนเข้าสถานีไฟฟ้าย่อย หรือจุดข้ามแม่น้ำกว้าง โครงสร้างแข็งแรงเป็นพิเศษเพื่อรับแรงดึงข้างเดียวทั้งหมดได้โดยไม่พัง
 4. เสาสลับตำแหน่งเฟส (Transposition Tower):
-สลับตำแหน่งสายตัวนำ (A, B, C) ทุกๆ 1/3 ของระยะทาง เพื่อให้ค่าความเหนี่ยวนำ (Inductance) และความจุไฟฟ้า (Capacitance) ของทั้ง 3 เฟสสมดุลเท่ากัน ลดปัญหาแรงดันไม่สมดุล</t>
+สลับตำแหน่งสายตัวนำ (A, B, C) ทุกๆ $1/3$ ของระยะทาง เพื่อให้ค่าความเหนี่ยวนำ ($L_{12} = L_{23} = L_{31}$) และความจุไฟฟ้าของทั้ง 3 เฟสสมดุลเท่ากัน ป้องกันแรงดันตกคร่อมไม่สมดุล</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -4410,12 +4432,12 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Customer Categories &amp; Supply Voltage Thresholds</t>
+          <t>Voltage Range Classifications &amp; Customer Types</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ประเภทผู้ใช้ไฟฟ้าตามเกณฑ์ กฟน./กฟภ. และระดับแรงดันที่ต้องจ่าย</t>
+          <t>การจำแนกระดับแรงดันไฟฟ้าและประเภทผู้ใช้ไฟฟ้าในประเทศไทย</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4425,58 +4447,59 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Final Exam ข้อ 5.4 (หน้า 25 - 4 คะแนน)</t>
+          <t>Final Exam ข้อ 5.3 &amp; 5.4 (หน้า 25 - 4 คะแนน)</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>State the standard customer categories used by MEA and PEA (Residential, Small General Service, Medium/Large General Service), and explain why large industrial customers must receive high voltage (22 kV - 115 kV) rather than low voltage (380 V).</t>
+          <t>Define Low Voltage (LV), Medium Voltage (MV), High Voltage (HV), and Extra High Voltage (EHV). Identify which customer tariff types connect to each voltage level.</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>จงระบุประเภทผู้ใช้ไฟฟ้ามาตรฐานตามข้อกำหนดของ กฟน./กฟภ. (บ้านอยู่อาศัย, กิจการขนาดเล็ก, กิจการขนาดกลาง/ใหญ่) และอธิบายเหตุผลทางวิศวกรรมว่าเหตุใดโรงงานอุตสาหกรรมขนาดใหญ่จึงต้องรับไฟฟ้าที่แรงดันสูง (22 kV - 115 kV) แทนที่จะรับที่แรงดันต่ำ 380 V</t>
+          <t>จงนิยามระดับแรงดัน: แรงดันต่ำ (LV), แรงดันปานกลาง (MV), แรงดันสูง (HV) และแรงดันสูงพิเศษ (EHV) พร้อมทั้งระบุว่าผู้ใช้ไฟฟ้าประเภทใดรับไฟที่ระดับแรงดันดังกล่าว</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>$$I = \frac{P}{\sqrt{3} V_L \cos\theta}$$
-$$\text{If } P = 10\text{ MW at } 380\text{ V: } I \approx 18,200\text{ A (Impossibly thick cables)}$$
-$$\text{If } P = 10\text{ MW at } 22\text{ kV: } I \approx 315\text{ A (Standard manageable cable)}$$</t>
+          <t>$$\text{EHV: } 500\text{ kV} \qquad \text{HV: } 115\text{ kV}, 230\text{ kV}$$
+$$\text{MV: } 22\text{ kV}, 24\text{ kV}, 33\text{ kV} \qquad \text{LV: } 380\text{ V } (3\phi), \; 220\text{ V } (1\phi)$$</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>1. Customer Categories (MEA/PEA):
-- Type 1: Residential (บ้านอยู่อาศัย) - Single-phase 220 V or 3-phase 380 V for large homes.
-- Type 2: Small General Service (ธุรกิจขนาดเล็ก) - Demand &lt; 30 kW (shops, small offices).
-- Type 3: Medium General Service (ธุรกิจขนาดกลาง) - Demand 30 kW - 999 kW.
-- Type 4: Large General Service (ธุรกิจขนาดใหญ่) - Demand &gt;= 1,000 kW (factories, malls).
-2. Why Large Customers Take High Voltage (22 kV - 115 kV):
-- Current Reduction: From P = sqrt(3)*V*I*cos(theta), supplying massive power at 380 V would require tens of thousands of amperes, needing impossibly thick copper busbars and incurring massive voltage drops (Delta V = I*Z).
-- Grid Reliability: Directly feeding from 22 kV or 115 kV keeps the customer's heavy fluctuating loads from distorting voltage quality for neighboring residential consumers on the low-voltage network.</t>
+          <t>1. Voltage Definitions in Thai System:
+- Extra High Voltage (EHV): $500\text{ kV}$ (inter-regional supergrid lines)
+- High Voltage (HV): $115\text{ kV}, 230\text{ kV}$ (regional transmission substations)
+- Medium Voltage (MV): $22\text{ kV}$ (PEA), $24\text{ kV} / 12\text{ kV}$ (MEA), $33\text{ kV}$ (distribution lines along roads)
+- Low Voltage (LV): $380\text{ V}$ (3-phase) / $220\text{ V}$ (single-phase).
+2. Customer Connections:
+- EHV / HV ($115 - 500\text{ kV}$): Heavy industrial plants (steel smelting, cement plants, chemical refineries).
+- MV ($22 - 33\text{ kV}$): Medium factories, department stores, universities, hospitals (having private step-down transformers).
+- LV ($220 / 380\text{ V}$): Residential homes, small commercial shops, residential buildings.</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>1. ประเภทผู้ใช้ไฟฟ้า (กฟน./กฟภ.):
-- ประเภท 1: บ้านอยู่อาศัย (Residential) - ใช้ไฟ 1 เฟส 220 V หรือ 3 เฟส 380 V
-- ประเภท 2: กิจการขนาดเล็ก (Small General Service) - ความต้องการพลังไฟฟ้า &lt; 30 kW
-- ประเภท 3: กิจการขนาดกลาง (Medium General Service) - ความต้องการ 30 kW - 999 kW
-- ประเภท 4: กิจการขนาดใหญ่ (Large General Service) - ความต้องการ &gt;= 1,000 kW ขึ้นไป (โรงงาน, ศูนย์การค้า)
-2. ทำไมกิจการขนาดใหญ่ต้องรับไฟที่แรงดันสูง (22 kV - 115 kV):
-- ลดขนาดกระแส: จากสูตร I = P / (sqrt(3)*V*cos(theta)) หากจ่ายโหลด 10 MW ที่ 380 V กระแสจะสูงถึง 18,000 แอมป์ สายไฟต้องมีขนาดมโหฬารและแรงดันตกมหาศาล แต่ถ้ารับที่ 22 kV กระแสเหลือเพียง 315 A
-- ป้องกันผลกระทบต่อผู้ใช้ไฟรายอื่น: การใช้ไฟกระชากของโรงงานจะไม่รบกวนแรงดันของผู้ใช้ไฟบ้านเรือนข้างเคียง</t>
+          <t>1. การแบ่งระดับแรงดันในระบบไฟฟ้าไทย:
+- แรงดันสูงพิเศษ (EHV): $500\text{ kV}$ (สายส่งสายหลักเชื่อมต่อระหว่างภาค)
+- แรงดันสูง (HV): $115\text{ kV}, 230\text{ kV}$ (สายส่งเชื่อมระหว่างสถานีไฟฟ้าย่อย)
+- แรงดันปานกลาง (MV): $22\text{ kV}$ (กฟภ.), $24\text{ kV} / 12\text{ kV}$ (กฟน.), $33\text{ kV}$ (สายป้อนบนเสาไฟริมถนน)
+- แรงดันต่ำ (LV): $380\text{ V}$ (3 เฟส) / $220\text{ V}$ (1 เฟสใช้งานทั่วไป)
+2. ประเภทผู้ใช้ไฟฟ้าที่ต่อรับไฟ:
+- EHV / HV ($115 - 500\text{ kV}$): โรงงานอุตสาหกรรมหนักขนาดใหญ่มาก (โรงถลุงเหล็ก, โรงปูนซีเมนต์, โรงกลั่นปิโตรเคมี)
+- MV ($22 - 33\text{ kV}$): โรงงานอุตสาหกรรมขนาดกลาง, ห้างสรรพสินค้า, มหาวิทยาลัย, โรงพยาบาล (มีหม้อแปลงของตนเอง)
+- LV ($220 / 380\text{ V}$): บ้านเรือนที่อยู่อาศัย, อาคารพาณิชย์ และร้านค้าทั่วไป</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>Supplying large loads at low voltage causes extreme copper loss I^2 R and severe voltage drop Delta V = I*Z.</t>
+          <t>Do not confuse MV (22 kV) with HV (115 kV). Normal street power lines on concrete poles are Medium Voltage (22 kV).</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>เหตุผลสำคัญ: ยิ่งกำลังไฟฟ้า P สูง ยิ่งต้องรับที่แรงดันสูง V เพื่อให้กระแส I ต่ำ ทำให้ประหยัดขนาดสายไฟ ลดแรงดันตก และลดการสูญเสีย I^2*R</t>
+          <t>ข้อระวัง: เสาไฟคอนกรีตริมถนนทั่วไปคือแรงดันปานกลาง (22 kV หรือ 24 kV) ไม่ใช่แรงดันสูง ส่วนสายไฟล่างสุดคือแรงดันต่ำ 220/380 V</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -4508,12 +4531,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Power Plant Specifics in Thailand (Bhumibol, Ubolratana, Mae Moh, Nam Pong)</t>
+          <t>Power Plant Types &amp; Fuel Sources in Thailand</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>โรงไฟฟ้าสำคัญในประเทศไทย (เขื่อนภูมิพล, เขื่อนอุบลรัตน์, โรงไฟฟ้าแม่เมาะ, โรงไฟฟ้าน้ำพอง)</t>
+          <t>ประเภทโรงไฟฟ้า แหล่งเชื้อเพลิง และโรงไฟฟ้าหลักในประเทศไทย</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -4523,58 +4546,53 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Final Exam ข้อ 5.2 (หน้า 25 - 2 คะแนน) &amp; Sheet ติว</t>
+          <t>Final Exam ข้อ 5.1 &amp; 5.2 (หน้า 25 - 4 คะแนน)</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Identify the power generation types and fuels of these major Thai power plants: Bhumibol Dam, Ubolratana Dam, Mae Moh Power Plant, and Nam Pong Power Plant.</t>
+          <t>Name the major power plant types in Thailand, list their fuel sources, and cite authentic plant examples for coal, combined cycle, and pumped storage hydro.</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>จงระบุประเภทของโรงไฟฟ้าและเชื้อเพลิงหลักของโรงไฟฟ้าสำคัญในประเทศไทยต่อไปนี้: เขื่อนภูมิพล, เขื่อนอุบลรัตน์, โรงไฟฟ้าแม่เมาะ และโรงไฟฟ้าน้ำพอง</t>
+          <t>จงระบุประเภทโรงไฟฟ้าหลักในประเทศไทย แหล่งเชื้อเพลิงที่ใช้ พร้อมยกตัวอย่างโรงไฟฟ้าของจริงสำหรับโรงไฟฟ้าถ่านหิน, โรงไฟฟ้าความร้อนร่วม และโรงไฟฟ้าพลังน้ำสูบกลับ</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>$$\text{Bhumibol / Ubolratana: Hydroelectric (พลังน้ำ)}$$
-$$\text{Mae Moh (Lampang): Lignite Coal Thermal (พลังความร้อนถ่านหินลิกไนต์)}$$
-$$\text{Nam Pong (Khon Kaen): Natural Gas Combined Cycle (พลังความร้อนร่วมก๊าซธรรมชาติ)}$$</t>
+          <t>$$\text{Thermal Coal / Lignite: Mae Moh (ลำปาง) } \rightarrow \text{Base Load}$$
+$$\text{Combined Cycle (Gas): Bang Pakong, South Bangkok, Wang Noi } \rightarrow \text{Base / Intermediate Load}$$
+$$\text{Pumped Storage Hydro: Lam Takhong (ลำตะคอง โคราช) } \rightarrow \text{Peak Load}$$
+$$\text{Conventional Hydro: Bhumibol, Sirikit, Srinagarind } \rightarrow \text{Peak / Quick Reserve}$$</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>1. Bhumibol Dam (เขื่อนภูมิพล - Tak):
-Hydroelectric power plant (พลังน้ำ); Thailand's largest concrete arch-gravity dam; also features pumped-storage units.
-2. Ubolratana Dam (เขื่อนอุบลรัตน์ - Khon Kaen):
-Hydroelectric multi-purpose dam (พลังน้ำ) supplying renewable power and irrigation in the Northeast (Isan).
-3. Mae Moh Power Plant (โรงไฟฟ้าแม่เมาะ - Lampang):
-Lignite coal-fired thermal power plant (โรงไฟฟ้าพลังความร้อนลิกไนต์); largest coal power complex in SE Asia, operating as a critical base load plant.
-4. Nam Pong Power Plant (โรงไฟฟ้าน้ำพอง - Khon Kaen):
-Combined-Cycle gas turbine power plant (โรงไฟฟ้าพลังความร้อนร่วม) fueled primarily by domestic natural gas from Sinphuhorm gas field.</t>
+          <t>1. Major Power Plants in Thailand:
+- Thermal Power Plant (Coal/Lignite): Mae Moh Power Plant (โรงไฟฟ้าแม่เมาะ จ.ลำปาง) uses domestic lignite coal, generating steady base load.
+- Combined-Cycle Power Plant (Gas Turbine + Steam Turbine): Bang Pakong (บางปะกง), South Bangkok (พระนครใต้), Wang Noi (วังน้อย) burning natural gas with high thermal efficiency ($&gt; 55\%$).
+- Pumped-Storage Hydro: Lam Takhong Jolabha Vadhana (เขื่อนลำตะคองชลภาวัฒนา จ.นครราชสีมา), pumps water up at night (cheap base power) and releases it during daytime peak demand.
+- Conventional Hydro: Bhumibol Dam (เขื่อนภูมิพล), Sirikit Dam (เขื่อนสิริกิติ์) used for rapid spinning reserve.</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>1. เขื่อนภูมิพล (จ.ตาก):
-โรงไฟฟ้าพลังน้ำ (Hydroelectric) เป็นเขื่อนคอนกรีตโค้งที่ใหญ่ที่สุดในไทย และมีเครื่องกำเนิดไฟฟ้าพลังน้ำสูบกลับ
-2. เขื่อนอุบลรัตน์ (จ.ขอนแก่น):
-โรงไฟฟ้าพลังน้ำอเนกประสงค์แห่งแรกในภาคอีสาน ใช้ผลิตไฟฟ้า พลประทาน และป้องกันน้ำท่วม
-3. โรงไฟฟ้าแม่เมาะ (จ.ลำปาง):
-โรงไฟฟ้าพลังความร้อน ใช้ถ่านหินลิกไนต์ (Lignite Coal) ในพื้นที่เป็นเชื้อเพลิง ทำหน้าที่เป็นโรงไฟฟ้าฐาน (Base Load) ที่สำคัญที่สุดของภาคเหนือ
-4. โรงไฟฟ้าน้ำพอง (จ.ขอนแก่น):
-โรงไฟฟ้าพลังความร้อนร่วม (Combined Cycle) ใช้ 'ก๊าซธรรมชาติ' จากแหล่งสินภูฮ่อมและน้ำพองเป็นเชื้อเพลิงหลักในการผลิตไฟฟ้าป้อนภาคอีสาน</t>
+          <t>1. โรงไฟฟ้าหลักในประเทศไทยและเชื้อเพลิง:
+- โรงไฟฟ้าพลังความร้อนถ่านหิน (Lignite Thermal): โรงไฟฟ้าแม่เมาะ จ.ลำปาง ใช้ถ่านหินลิกไนต์ในประเทศ เดินเครื่องเป็นโรงไฟฟ้าฐาน (Base Load)
+- โรงไฟฟ้าพลังความร้อนร่วม (Combined-Cycle): โรงไฟฟ้าบางปะกง, โรงไฟฟ้าพระนครใต้, โรงไฟฟ้าวังน้อย ใช้ก๊าซธรรมชาติร่วมกับกังหันไอน้ำ มีประสิทธิภาพความร้อนสูง ($&gt; 55\%$)
+- โรงไฟฟ้าพลังน้ำสูบกลับ (Pumped-Storage Hydro): โรงไฟฟ้าลำตะคองชลภาวัฒนา จ.นครราชสีมา สูบน้ำกลับขึ้นอ่างเก็บน้ำบนเขาตอนกลางคืน และปล่อยน้ำลงมาปั่นไฟเวลารับโหลดสูงสุด (Peak Load)
+- โรงไฟฟ้าพลังน้ำทั่วไป: เขื่อนภูมิพล, เขื่อนสิริกิติ์, เขื่อนศรีนครินทร์ ใช้เสริมช่วงพีกและสำรองฉุกเฉิน</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>Do not confuse Mae Moh (Lignite Coal in Lampang) with Nam Pong (Natural Gas in Khon Kaen).</t>
+          <t>Lam Takhong is a Pumped-Storage Hydro plant, NOT a conventional river dam. It stores energy like a massive hydro battery.</t>
         </is>
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>จำให้แม่น: แม่เมาะ (ลำปาง) = ถ่านหินลิกไนต์, น้ำพอง (ขอนแก่น) = ก๊าซธรรมชาติ, ภูมิพล/อุบลรัตน์ = พลังน้ำ</t>
+          <t>จุดเน้น: โรงไฟฟ้าลำตะคองเป็น 'พลังน้ำสูบกลับ (Pumped Storage)' ทำหน้าที่เหมือนแบตเตอรี่น้ำขนาดใหญ่ ไม่ใช่เขื่อนกักน้ำแม่น้ำทั่วไป</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -4606,72 +4624,73 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Residential Solar PV Rooftop System Components</t>
+          <t>Transmission Tower Grounding Resistance &amp; Lightning Protection</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>องค์ประกอบของระบบโซลาร์เซลล์บนหลังคาบ้าน (Solar PV Rooftop)</t>
+          <t>ความต้านทานดินของเสาสายส่ง (Tower Footing Resistance) และการป้องกันฟ้าผ่า</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Level 1 (Concept)</t>
+          <t>Level 2 (Analysis)</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Lecture Chapter 9 (Renewable Energy)</t>
+          <t>Lecture Chapter 9 (Power Systems)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>List the core components of a grid-tied residential Solar PV Rooftop system and explain the essential safety role of Anti-Islanding protection.</t>
+          <t>What is Tower Footing Resistance, why must it be kept below 10 ohms, and how do overhead ground wires (OHGW / Shield wires) prevent transmission line flashovers during lightning strikes?</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>จงระบุอุปกรณ์หลักในระบบโซลาร์เซลล์บนหลังคาบ้านเรือนแบบเชื่อมต่อโครงข่าย (Grid-Tied Solar PV Rooftop) และอธิบายความสำคัญของการป้องกันการจ่ายไฟแบบเกาะเดี่ยว (Anti-Islanding Protection)</t>
+          <t>ความต้านทานขากราวด์เสาสายส่ง (Tower Footing Resistance) คืออะไร ทำไมต้องคุมให้ต่ำกว่า 10 โอห์ม และสายล่อฟ้าเหนือศีรษะ (Overhead Ground Wire: OHGW) ป้องกันการเกิดฟลัชโอเวอร์ได้อย่างไร?</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>$$\text{PV Panels (DC)} \rightarrow \text{DC Combiner/Breaker} \rightarrow \text{Grid-Tied Inverter (DC to AC)} \rightarrow \text{Bi-directional Meter} \rightarrow \text{Grid}$$
-$$\text{Anti-Islanding: Grid Loss } \implies \text{Inverter disconnects immediately within 2 seconds}$$</t>
+          <t>$$R_{\text{tower}} \le 10\;\Omega$$
+$$V_{\text{tower top}} = I_{\text{lightning}} \cdot R_{\text{tower}} + L_{\text{tower}} \frac{di}{dt}$$
+$$\text{Back Flashover occurs if: } V_{\text{tower top}} - V_{\text{conductor}} &gt; V_{\text{insulator CFO}}$$</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>1. Core Components:
-- Solar PV Modules (แผงโซลาร์เซลล์): Converts sunlight photons into DC electricity.
-- DC Protection Box (ตู้ไฟ DC): Fuses, DC Circuit Breaker, DC Surge Protection Device (SPD).
-- Grid-Tied Inverter (อินเวอร์เตอร์): Converts variable DC into synchronized 220 V 50 Hz AC matching the utility grid.
-- AC Protection Box (ตู้ไฟ AC): AC Breaker, RCBO/RCD, AC SPD.
-- Bi-directional Meter (มิเตอร์ 2 ทาง): Measures both imported energy from grid and surplus exported solar energy.
-2. Anti-Islanding Protection (Mandatory):
-When the public utility grid suffers a blackout or is switched off for line maintenance, the inverter MUST disconnect automatically within 2 seconds. This prevents backfeeding power into downed lines, protecting utility repair technicians from lethal electrocution.</t>
+          <t>1. Tower Footing Resistance ($R_{\text{tower}}$):
+The electrical contact resistance between the steel tower base / counterpoise ground wires and the surrounding earth. It must be kept strictly below $10\;\Omega$ (often $&lt; 5\;\Omega$).
+2. Back Flashover Mechanism:
+When lightning strikes the tower apex or overhead shield wire, huge lightning surge current ($I_{\text{lightning}} \approx 20 - 100\text{ kA}$) rushes down the tower to ground. The transient voltage at the tower top rises to:
+$$V_{\text{tower top}} = I_{\text{lightning}} \cdot R_{\text{tower}} + L \frac{di}{dt}$$
+If $R_{\text{tower}}$ is large, $V_{\text{tower top}}$ spikes to hundreds of kilovolts, flashing over across the insulator string to the phase conductor (Back Flashover), causing a grid trip.
+3. Overhead Ground Wire (OHGW):
+Shield wires positioned at the very top of towers provide an interception shield angle ($&lt; 30^\circ$), capturing direct lightning strikes and draining the current safely into ground.</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>1. อุปกรณ์หลักในระบบ:
-- แผงโซลาร์เซลล์ (PV Modules): เปลี่ยนพลังงานแสงอาทิตย์เป็นไฟฟ้ากระแสตรง (DC)
-- ตู้ควบคุมไฟฟ้ากระแสตรง (DC Combiner/Protection Box): ฟิวส์, DC Breaker, และอุปกรณ์ป้องกันเสิร์จ (SPD)
-- อินเวอร์เตอร์เชื่อมโครงข่าย (Grid-Tied Inverter): แปลงไฟ DC เป็นไฟ AC 220 V 50 Hz ที่ซิงโครไนซ์เฟสตรงกับไฟการไฟฟ้า
-- ตู้ควบคุมไฟฟ้ากระแสสลับ (AC Distribution/Protection Box): เบรกเกอร์ AC และอุปกรณ์ตัดไฟรั่ว
-- มิเตอร์ไฟฟ้าสองทิศทาง (Bi-directional Smart Meter): บันทึกหน่วยไฟฟ้าทั้งฝั่งที่ซื้อจากการไฟฟ้าและฝั่งที่ขายคืนโซลาร์
-2. ระบบป้องกัน Anti-Islanding (หัวใจสำคัญด้านความปลอดภัย):
-เมื่อไฟจากการไฟฟ้าดับ หรือมีการตัดไฟเพื่อซ่อมแซมสายไฟ อินเวอร์เตอร์ต้องหยุดจ่ายไฟและตัดการเชื่อมต่อทันที (ภายใน 2 วินาที) เพื่อป้องกันไฟจากโซลาร์เซลล์ไหลย้อนเข้าสายส่ง ซึ่งอาจช็อตเจ้าหน้าที่การไฟฟ้าที่กำลังปฏิบัติงานจนถึงแก่ชีวิต</t>
+          <t>1. ความต้านทานขากราวด์เสาสายส่ง (Tower Footing Resistance):
+คือความต้านทานระหว่างโครงสร้างเหล็กของเสากับเนื้อดิน ต้องควบคุมให้ต่ำกว่า $10\;\Omega$ (มาตรฐานที่ดีควรต่ำกว่า $5\;\Omega$)
+2. กลไกการเกิด Back Flashover:
+เมื่อฟ้าผ่าลงยอดเสาหรือสายลวดล่อฟ้า กระแสฟ้าผ่ามหาศาล ($20 - 100\text{ kA}$) จะไหลลงดินผ่านโครงสร้างเสา ทำให้เกิดแรงดันตกคร่อมขากราวด์:
+$$V_{\text{tower top}} = I_{\text{lightning}} \cdot R_{\text{tower}} + L \frac{di}{dt}$$
+ถ้าความต้านทานดิน $R_{\text{tower}}$ สูง แรงดันที่ยอดเสาจะพุ่งสูงหลายร้อยกิโลโวลต์ จนเกิดการสปาร์กข้ามลูกถ้วยฉนวนกลับไปยังสายตัวนำเฟส (Back Flashover) ทำให้ระบบตัดวงจร
+3. สายล่อฟ้าเหนือศีรษะ (Overhead Ground Wire: OHGW):
+ขึงอยู่บนยอดสุดของเสาสายส่ง ทำมุมป้องกัน (Shielding Angle $&lt; 30^\circ$) ดักรับฟ้าผ่าโดยตรงแทนสายตัวนำเฟส แล้วกระจายกระแสลงดินอย่างปลอดภัย</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>Anti-Islanding is a strict legal requirement by MEA/PEA for all grid-tied solar installations.</t>
+          <t>High tower footing resistance causes Back Flashover from tower to line, defeating the purpose of insulators.</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>จุดสำคัญ: มาตรฐาน กฟน./กฟภ. บังคับให้อินเวอร์เตอร์ทุกเครื่องต้องมีระบบ Anti-Islanding ป้องกันไฟฟ้าไหลย้อนกลับสายส่งเด็ดขาดเมื่อไฟหลวงดับ</t>
+          <t>ข้อระวัง: หากความต้านทานขากราวด์เสาสูง ฟ้าผ่าลงสายดินแต่จะกระโดดย้อนข้ามลูกถ้วยเข้าสายส่ง (Back Flashover) ทำให้ไฟฟ้าดับได้</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr"/>
@@ -4695,12 +4714,12 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Energy Conservation in Household Washing Machines</t>
+          <t>Household Energy Conservation Measures</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>การอนุรักษ์พลังงานในการใช้เครื่องซักผ้าในบ้านเรือน</t>
+          <t>มาตรการการอนุรักษ์พลังงานไฟฟ้าในบ้านเรือนที่อยู่อาศัย (ข้อสอบไฟนอล)</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -4710,56 +4729,64 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Final Exam ข้อ 5.5 (หน้า 24 - 2 คะแนน)</t>
+          <t>Final Exam ข้อ 5.5 (หน้า 24 - 4 คะแนน)</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>State practical energy-saving guidelines when using a residential washing machine.</t>
+          <t>Propose 4 practical and effective energy conservation measures to reduce electrical consumption in residential homes.</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>จงระบุแนวทางการประหยัดพลังงานและอนุรักษ์ไฟฟ้าในการใช้งานเครื่องซักผ้าในบ้านเรือน</t>
+          <t>จงเสนอ 4 มาตรการประหยัดพลังงานไฟฟ้าที่มีประสิทธิภาพและนำไปปฏิบัติได้จริงสำหรับบ้านเรือนที่อยู่อาศัย (ข้อสอบไฟนอลข้อ 5.5)</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>$$\text{Wash at full rated load} + \text{Use cold water } + \text{Select Inverter Motor}$$</t>
+          <t>$$P = \frac{\text{BTU/hr}}{\text{SEER} \times 3.412} \implies \text{High SEER Inverter saves } 20\% - 30\%$$
+$$\Delta P \approx 10\% \text{ per } 1^\circ\text{C increase (Set AC to } 25^\circ\text{C} - 26^\circ\text{C)}$$
+$$P_{\text{LED}} \approx \frac{1}{5} P_{\text{Incandescent}} \quad (80\% \text{ energy reduction})$$</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>1. Wash at Full Capacity:
-Accumulate clothes and wash at the machine's rated full drum capacity, rather than doing frequent small washes, reducing total motor running cycles and water consumption.
-2. Use Cold Water:
-Use cold water setting (30°C or room temp) instead of hot water heating cycles (60°C - 90°C), as electric water heating elements consume over 80-90% of total wash cycle energy.
-3. Pre-soak Heavy Stains:
-Pre-soak heavily soiled clothes manually before putting them in, allowing standard or quick wash modes rather than heavy prolonged cycles.
-4. Use Inverter Motor &amp; Air Dry:
-Choose washing machines with high energy-efficiency labels (ฉลากประหยัดไฟเบอร์ 5 ดาวสูง) with Inverter BLDC motors, and utilize natural outdoor sunlight for drying instead of electric tumble dryers.</t>
+          <t>Four Practical Residential Energy Conservation Measures:
+1. Air Conditioning Optimization:
+- Set thermostat to $25^\circ\text{C} - 26^\circ\text{C}$ and use a fan simultaneously (each $1^\circ\text{C}$ temperature increase saves $\approx 10\%$ electrical energy).
+- Select High-Efficiency Inverter units with Energy Label No. 5 (5 Stars, high SEER).
+- Clean air filter screens every month and service coils every 6 months.
+2. Lighting Upgrades:
+- Replace all conventional incandescent ($60\text{ W}$) and compact fluorescent ($18\text{ W}$) bulbs with high-efficacy LED lighting ($9\text{ W}$), achieving $&gt; 80\%$ power reduction for identical luminous flux.
+3. Refrigerator Management:
+- Position refrigerator at least $15\text{ cm}$ away from walls to ensure airflow around condenser coils; set dial to medium and avoid opening door frequently.
+4. Eliminate Standby Vampire Power:
+- Unplug entertainment electronics and chargers or switch off power strips when not in use.</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>1. ซักผ้าตามพิกัดความจุถัง (Full Load):
-รวบรวมผ้าซักให้เต็มความจุพิกัดของถังซักในแต่ละรอบ ไม่ควรซักผ้าทีละน้อยชิ้นบ่อยๆ เพื่อลดรอบการทำงานของมอเตอร์และการใช้น้ำ
-2. ใช้น้ำอุณหภูมิปกติ (Cold Water):
-หลีกเลี่ยงการใช้น้ำร้อนในการซักผ้า (ยกเว้นจำเป็น) เพราะขดลวดฮีตเตอร์ต้มน้ำใช้พลังงานไฟฟ้าสูงถึง 80-90% ของพลังงานทั้งหมดในรอบซัก
-3. แช่ผ้าก่อนซักสำหรับผ้าที่สกปรกมาก:
-ขจัดคราบสกปรกหนักก่อนนำเข้าเครื่อง เพื่อให้สามารถใช้โปรแกรมซักแบบปกติหรือ Quick Wash แทนการซักรอบยาว
-4. เลือกเครื่องซักผ้าระบบอินเวอร์เตอร์และตากแดดธรรมชาติ:
-เลือกซื้อเครื่องซักผ้าฉลากเบอร์ 5 แบบมีดาว (Inverter Direct Drive) และตากผ้าด้วยแสงแดดธรรมชาติแทนการใช้เครื่องอบผ้าไฟฟ้าที่กินไฟสูง</t>
+          <t>4 มาตรการประหยัดพลังงานในบ้านเรือน (ตามแนวข้อสอบไฟนอล):
+1. การปรับปรุงระบบปรับอากาศ (กินไฟสูงสุดในบ้าน $\approx 60\%$):
+- ปรับอุณหภูมิที่ $25^\circ\text{C} - 26^\circ\text{C}$ ควบคู่กับการเปิดพัดลมช่วยกระจายลม (การเพิ่มอุณหภูมิ $1^\circ\text{C}$ ประหยัดไฟได้ประมาณ $10\%$)
+- เลือกใช้แอร์ระบบ Inverter เบอร์ 5 ติดดาว (ค่า SEER สูง)
+- ล้างแผ่นกรองอากาศทุกเดือน และล้างเครื่องปรับอากาศทุก 6 เดือน
+2. เปลี่ยนมาใช้หลอดไฟ LED:
+- เปลี่ยนหลอดไส้เดิม ($60\text{ W}$) หรือหลอดฟลูออเรสเซนต์ ($18\text{ W}$) เป็นหลอด LED ($9\text{ W}$) ประหยัดไฟลงได้มากกว่า $50\% - 80\%$ โดยได้ความสว่างเท่าเดิม
+3. การใช้งานตู้เย็นอย่างถูกวิธี:
+- วางตู้เย็นห่างจากผนังอย่างน้อย $15\text{ cm}$ เพื่อระบายความร้อน, ไม่นำของร้อนเข้าแช่ทันที และตรวจเช็กยางขอบประตูไม่ให้รั่ว
+4. ปลดปลั๊กตัด Standby Power (ไฟสแตนด์บาย):
+- ถอดปลั๊กอุปกรณ์อิเล็กทรอนิกส์, ทีวี, และที่ชาร์จเมื่อไม่ใช้งานเพื่อตัดกระแสไฟสแตนด์บายที่กินไฟตลอด 24 ชั่วโมง</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>Electric water heating in washing machines consumes far more energy than the motor itself. Avoid hot wash cycles unless medically required.</t>
+          <t>Air conditioning represents 50-65% of typical home electricity bills. Targeting AC temperature and maintenance yields the largest financial savings.</t>
         </is>
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>จุดสำคัญ: ตัวที่กินไฟที่สุดในเครื่องซักผ้าไม่ใช่ตัวมอเตอร์ แต่คือ 'ฮีตเตอร์ต้มน้ำร้อน' การซักด้วยน้ำอุณหภูมิปกติจะช่วยประหยัดไฟได้มากที่สุด</t>
+          <t>จุดสำคัญ: แอร์กินไฟมากกว่า 60% ของทั้งบ้าน ดังนั้นมาตรการปรับอุณหภูมิแอร์และล้างแอร์เป็นจุดที่ให้ผลประหยัดเงินสูงสุด</t>
         </is>
       </c>
       <c r="N47" s="4" t="inlineStr">
@@ -4791,12 +4818,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Energy Conservation in Industrial Manufacturing Plants</t>
+          <t>Industrial Factory Energy Conservation Measures</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>มาตรการอนุรักษ์พลังงานในโรงงานอุตสาหกรรม (มอเตอร์, แสงสว่าง, ระบบปรับอากาศ)</t>
+          <t>มาตรการการอนุรักษ์พลังงานไฟฟ้าในโรงงานอุตสาหกรรม (ข้อสอบไฟนอล)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -4806,62 +4833,63 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Final Exam ข้อ 5.6 (หน้า 24 - 2 คะแนน)</t>
+          <t>Final Exam ข้อ 5.6 (หน้า 24 - 4 คะแนน)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Propose practical energy conservation measures for an industrial factory across: (a) Electric motors and drives, (b) Lighting systems, and (c) Air conditioning and thermal systems.</t>
+          <t>Propose 4 engineering measures for energy conservation in industrial factories and commercial facilities.</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>จงเสนอมาตรการอนุรักษ์พลังงานไฟฟ้าในโรงงานอุตสาหกรรมใน 3 ด้านหลัก: (a) ระบบมอเตอร์ไฟฟ้าและขับเคลื่อน, (b) ระบบไฟฟ้าแสงสว่าง, และ (c) ระบบปรับอากาศและระบายความร้อน</t>
+          <t>จงเสนอ 4 มาตรการอนุรักษ์พลังงานไฟฟ้าเชิงวิศวกรรมสำหรับโรงงานอุตสาหกรรมและอาคารธุรกิจ (ข้อสอบไฟนอลข้อ 5.6)</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>$$\text{Motor: VFD / Inverter + IE3/IE4 Motors} \quad \Delta P_{\text{save}} \propto (1 - (n_2/n_1)^3)$$
-$$\text{Power Factor Correction: Install Capacitor Banks } \implies PF \ge 0.85$$
-$$\text{Lighting: Replace HID/Fluorescent with LED} \implies 50\% - 70\% \text{ reduction}$$</t>
+          <t>$$Q_C = P \left( \tan\theta_1 - \tan\theta_2 \right) \implies \text{Raise } \text{PF} \ge 0.85 \text{ to avoid PEA/MEA penalty}$$
+$$I_{\text{line}} = \frac{P}{\sqrt{3} V_L \cos\theta} \implies \text{Higher PF reduces cable } I^2 R \text{ loss}$$
+$$\text{VFD Affinity Law: } \frac{P_1}{P_2} = \left(\frac{n_1}{n_2}\right)^3 = \left(\frac{Q_1}{Q_2}\right)^3$$</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>1. Electric Motor Systems (Consumes &gt; 65% of industrial power):
-- Install Variable Frequency Drives (VFD) on centrifugal pumps and fans to adjust motor speed according to real-time load instead of wasteful mechanical throttling valves (affinity laws: P proportional to n^3).
-- Upgrade old motors to Premium High-Efficiency Motors (IE3 or IE4 standard).
-- Correct Plant Power Factor by installing Automatic Capacitor Banks at the main switchboard (MDB) to maintain PF &gt;= 0.85, eliminating PEA/MEA reactive power fines (ค่า kVAR).
-2. Lighting Systems:
-- Retrofit older fluorescent (T8) and high-intensity discharge (HID/Metal Halide) lamps with industrial LED luminaires (saving 50-70% power).
-- Install smart daylight sensors and occupancy sensors in warehouses.
-3. Air Conditioning &amp; Chillers:
-- Optimize chilled water temperatures and schedule chiller sequencing based on production shifts.
-- Maintain and clean chiller condenser tubes and cooling tower fins regularly to prevent heat-transfer scale buildup.</t>
+          <t>Four Engineering Industrial Energy Conservation Measures:
+1. Power Factor (PF) Correction with Capacitor Banks:
+- Install automatic power factor correction (APFC) capacitor banks at main distribution switchboards to boost plant PF from $&lt; 0.80$ to $&gt; 0.95$.
+- Eliminates utility low power factor penalty charges and reduces factory cable $I^2 R$ heat losses.
+2. Variable Frequency Drives (VFD) on Pumps and Fans:
+- Replace mechanical throttle valves and dampers with VFD motor speed controllers.
+- By pump/fan affinity laws ($P \propto n^3$), reducing motor speed by $20\%$ cuts motor shaft power consumption by nearly $50\%$.
+3. High-Efficiency Motors (IE3 / IE4 Premium Efficiency):
+- Retrofit standard induction motors with IE3/IE4 motors equipped with low-loss copper rotors and superior magnetic core laminations.
+4. Compressed Air System Leak Audits &amp; Optimization:
+- Detect and seal compressed air pipe leaks (leaks routinely waste $20\% - 30\%$ of compressor output) and lower system operating pressure to the minimum required level.</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>1. ระบบมอเตอร์ไฟฟ้า (ใช้ไฟมากที่สุดในโรงงาน &gt; 65%):
-- ติดตั้งอินเวอร์เตอร์ปรับความเร็วรอบ (VFD): สำหรับปั๊มน้ำและพัดลมระบายอากาศ เพื่อปรับรอบตามโหลดจริง แทนการหรี่วาล์วเชิงกล (ตามกฎ Affinity Law: กำลังไฟฟ้าแปรผันตามความเร็วรอบยกกำลังสาม P ~ n^3)
-- เปลี่ยนมาใช้มอเตอร์ประสิทธิภาพสูงพิเศษ (IE3 / IE4 Premium Efficiency Motors)
-- ปรับปรุงค่าเพาเวอร์แฟกเตอร์ (PF Correction): ติดตั้ง Capacitor Bank อัตโนมัติที่ตู้ MDB เพื่อรักษาค่า PF &gt;= 0.85 หลีกเลี่ยงค่าปรับเพาเวอร์แฟกเตอร์ของ กฟน./กฟภ.
-2. ระบบแสงสว่าง:
-- เปลี่ยนหลอดไฟโรงงานเดิม (หลอดฟลูออเรสเซนต์ T8 หรือหลอดแสงจันทร์ HID) เป็นหลอดประหยัดไฟ LED คุณภาพสูง (ประหยัดไฟได้ 50-70%)
-- ติดตั้งเซ็นเซอร์ตรวจจับการเคลื่อนไหว (Motion Sensor) และเซ็นเซอร์วัดแสงแดดในคลังสินค้า
-3. ระบบปรับอากาศและทำความเย็น (Chiller &amp; HVAC):
-- ควบคุมอุณหภูมิน้ำเย็น (Chilled Water) ให้เหมาะสม และตั้งเวลาเปิด-ปิดตามกะการทำงานจริง
-- ล้างคอนเดนเซอร์และบำรุงรักษาหอผึ่งน้ำ (Cooling Tower) สม่ำเสมอเพื่อขจัดตะกรันและรักษาประสิทธิภาพการระบายความร้อน</t>
+          <t>4 มาตรการอนุรักษ์พลังงานในโรงงานอุตสาหกรรม (ตามแนวข้อสอบไฟนอล):
+1. ติดตั้งชุดคาปาซิเตอร์แบงก์ปรับปรุงค่าเพาเวอร์แฟกเตอร์ (PF Improvement):
+- ปรับปรุงค่าเพาเวอร์แฟกเตอร์จากเดิมที่ต่ำให้สูงกว่า $0.85$ (มาตรฐานควร $&gt; 0.95$) เพื่อหลีกเลี่ยงค่าปรับเพาเวอร์แฟกเตอร์ของ กฟภ./กฟน. และลดกระแสโหลดในสายเคเบิล ทำให้ลดการสูญเสีย $I^2 R$
+2. ติดตั้งอุปกรณ์ปรับความเร็วรอบมอเตอร์ (Variable Frequency Drive: VFD):
+- นำ VFD มาควบคุมมอเตอร์ปั๊มน้ำและพัดลมระบายอากาศแทนการใช้แดมเปอร์หรือวาล์วหรี่
+- ตามกฎความคล้ายคลึงของปั๊ม ($P \propto n^3$) การลดความเร็วรอบลงเพียง $20\%$ จะช่วยประหยัดพลังงานได้เกือบ $50\%$
+3. เปลี่ยนมาใช้มอเตอร์ประสิทธิภาพสูง (Premium Efficiency Motor IE3/IE4):
+- ใช้มอเตอร์มาตรฐาน IE3/IE4 ที่มีแกนเหล็กสูญเสียต่ำและขดลวดทองแดงหนา ช่วยลดความร้อนสะสมและประหยัดไฟตลอดอายุการใช้งาน
+4. ซ่อมบำรุงระบบอากาศอัด (Compressed Air Leak Repair):
+- ตรวจเช็กและอุดรอยรั่วท่อลมในโรงงาน (ซึ่งมักสูญเสียลมทิ้งเฉลี่ย $20\% - 30\%$ ของกำลังปั๊มลม) และปรับลดแรงดันใช้งานลงให้พอดีกับความต้องการจริง</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>Capacitor banks do NOT reduce active power (kW) consumed by the load, but they eliminate reactive power (kVAR) from the grid, reducing line current and avoiding utility penalty fees.</t>
+          <t>In factories, electric motors account for ~70% of total electrical energy. VFDs and PF correction yield massive financial returns.</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t>ข้อควรระวัง: คาปาซิเตอร์แบงก์ไม่ได้ช่วยลดกำลังไฟฟ้าจริง (kW) ของเครื่องจักร แต่ช่วยลดกำลังไฟฟ้ารีแอคทีฟ (kVAR) ทำให้กระแสรวมในสายลดลง และไม่โดนค่าปรับ PF ตกจากการไฟฟ้า</t>
+          <t>จุดเน้นวิศวกรรม: ในโรงงานอุตสาหกรรม มอเตอร์กินไฟมากกว่า 70% ของโรงงาน การติดตั้ง VFD และคาปาซิเตอร์แบงก์จึงเป็นมาตรการที่คุ้มทุนเร็วที่สุด</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -4908,48 +4936,61 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Homework Chapter 10 &amp; Final Exam ข้อ 3</t>
+          <t>Homework Chapter 10 &amp; Final Exam ข้อ 3.1</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Explain the operating principle of a Permanent Magnet Moving Coil (PMMC / D'Arsonval) instrument. State the formula for deflecting torque and explain why PMMC instruments only measure DC directly.</t>
+          <t>Explain the operating principle of a Permanent Magnet Moving Coil (PMMC / D'Arsonval) instrument. State the formulas for deflecting torque and controlling torque, and explain why PMMC instruments measure only DC directly.</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>จงอธิบายหลักการทำงานของเครื่องมือวัดแบบขดลวดเคลื่อนที่แกนแม่เหล็กถาวร (PMMC / D'Arsonval Galvanometer) เขียนสมการแรงบิดบิดเบน (Deflecting Torque) และอธิบายเหตุผลว่าทำไม PMMC จึงวัดได้เฉพาะไฟฟ้ากระแสตรง (DC) โดยตรง</t>
+          <t>จงอธิบายหลักการทำงานของเครื่องมือวัดแบบขดลวดเคลื่อนที่แกนแม่เหล็กถาวร (PMMC / D'Arsonval Galvanometer) เขียนสมการแรงบิดบิดเบน (Deflecting Torque) และแรงบิดควบคุม (Controlling Torque) พร้อมอธิบายเหตุผลว่าทำไม PMMC จึงวัดได้เฉพาะไฟฟ้ากระแสตรง (DC) โดยตรง</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
           <t>$$T_d = B \cdot I \cdot N \cdot A = G \cdot I$$
 $$T_c = C \cdot \theta$$
-$$\text{At equilibrium: } T_d = T_c \implies \theta = \left(\frac{G}{C}\right) I \propto I$$</t>
+$$\text{At equilibrium: } T_d = T_c \implies \theta = \left(\frac{B \cdot N \cdot A}{C}\right) I \propto I$$
+$$I_{\text{avg, AC}} = \frac{1}{T} \int_0^T I_m \sin(\omega t)\, dt = 0$$</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
           <t>1. Operating Principle:
-A rectangular copper coil carrying current I is pivoted inside the magnetic field B of a permanent magnet. The interaction of current and magnetic flux creates a Lorentz force (F = I*L x B), producing a deflecting torque Td.
-2. Linear Scale:
-Since deflecting torque Td = B*I*N*A and restoring spring torque Tc = C*theta, at steady state:
-theta = (B*N*A / C) * I
-Because B, N, A, and C are constant, the pointer deflection angle theta is directly proportional to current I, yielding a perfectly LINEAR scale.
-3. Why DC Only:
-If connected to alternating current (AC), the torque alternates direction every half-cycle (50 Hz). Due to the mechanical inertia of the moving coil and pointer, the meter cannot follow this rapid oscillation and indicates strictly the AVERAGE value, which is ZERO for pure sinusoidal AC.</t>
+A rectangular coil with $N$ turns and cross-sectional area $A$ carrying current $I$ is suspended in the uniform radial magnetic field $B$ of a permanent magnet. The interaction between current and magnetic flux produces a Lorentz force ($F = I L B$), resulting in a deflecting torque $T_d$:
+$$T_d = B \cdot I \cdot N \cdot A = G \cdot I$$
+where $G = B N A$ is the galvanometer constant.
+2. Controlling Torque &amp; Linear Scale:
+A spiral hairspring produces an opposing restoring torque $T_c$:
+$$T_c = C \cdot \theta$$
+where $C$ is the spring constant and $\theta$ is the angular deflection. At equilibrium ($T_d = T_c$):
+$$\theta = \left(\frac{B \cdot N \cdot A}{C}\right) I = \left(\frac{G}{C}\right) I$$
+Because $B, N, A$, and $C$ are constants, the pointer deflection angle $\theta$ is directly proportional to current $I$ ($\theta \propto I$). This guarantees an evenly spaced, completely linear scale.
+3. Why Measures Only DC Directly:
+If connected to sinusoidal alternating current ($i(t) = I_m \sin\omega t$), torque alternates direction every half-cycle (50 Hz). Due to the mechanical inertia of the moving coil assembly, the pointer cannot track 50 Hz oscillations and responds strictly to the time-average value:
+$$I_{\text{avg}} = \frac{1}{T} \int_0^T I_m \sin(\omega t)\, dt = 0$$
+The pointer vibrates negligibly around zero. To measure AC, a diode rectifier must be placed before the PMMC movement.</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
           <t>1. หลักการทำงาน:
-ขดลวดทองแดงสี่เหลี่ยมที่มีกระแส I ไหลผ่าน ถูกติดตั้งอยู่ระหว่างขั้วแม่เหล็กถาวรความเข้ม B ปฏิกิริยาระหว่างกระแสไฟฟ้าและสนามแม่เหล็กจะทำให้เกิดแรงลอเรนซ์ (Lorentz Force: F = I*L*B) ส่งผลให้เกิดแรงบิดบิดเบน (Deflecting Torque: Td) ผลักให้แกนเข็มหมุน
+ขดลวดทองแดงรูปสี่เหลี่ยมจำนวน $N$ รอบ พื้นที่หน้าตัด $A$ มีกระแส $I$ ไหลผ่าน ถูกติดตั้งอยู่ระหว่างขั้วแม่เหล็กถาวรความเข้มสนามแม่เหล็ก $B$ แรงลอเรนซ์ ($F = I L B$) ทำให้เกิดแรงบิดบิดเบน ($T_d$):
+$$T_d = B \cdot I \cdot N \cdot A = G \cdot I$$
+โดยที่ $G = B N A$ คือค่าคงที่ของกัลวาโนมิเตอร์
 2. สเกลเชิงเส้น (Linear Scale):
-แรงบิดบิดเบน Td = B*I*N*A จะถูกต้านด้วยแรงบิดควบคุมจากสปริงก้นหอย Tc = C*theta เมื่อเข็มชี้หยุดนิ่ง (Td = Tc):
-theta = (B*N*A / C) * I
-เนื่องจากค่า B, N, A, C เป็นค่าคงที่ มุมเบี่ยงเบน theta จึงแปรผันตรงกับกระแส I ทำให้สเกลหน้าปัดแบ่งช่องได้เท่ากันอย่างสม่ำเสมอ (Linear Scale)
-3. ทำไมวัดได้เฉพาะไฟ DC:
-หากนำไปต่อกับไฟสลับ (AC) 50 Hz ทิศทางของแรงบิดจะกลับทิศไปมา 50 ครั้งต่อวินาที ความเฉื่อยเชิงกล (Inertia) ของขดลวดและเข็มชี้ทำให้เข็มขยับตามไม่ทัน จึงชี้ที่ 'ค่าเฉลี่ย' ซึ่งสำหรับไฟสลับรูปคลื่นไซน์ ค่าเฉลี่ยใน 1 คาบจะเท่ากับศูนย์ (เข็มสั่นอยู่ที่ขีด 0)</t>
+สปริงก้นหอยจะสร้างแรงบิดควบคุมต้านกลับ ($T_c$):
+$$T_c = C \cdot \theta$$
+เมื่อเข็มชี้หยุดนิ่งที่สภาวะสมดุล ($T_d = T_c$):
+$$\theta = \left(\frac{B \cdot N \cdot A}{C}\right) I = \left(\frac{G}{C}\right) I$$
+เนื่องจาก $B, N, A, C$ เป็นค่าคงที่ มุมเบี่ยงเบน $\theta$ จึงแปรผันตรงกับกระแส $I$ ส่งผลให้สเกลหน้าปัดแบ่งช่องได้เท่ากันอย่างสม่ำเสมอเป็นเชิงเส้น (Linear Scale)
+3. เหตุผลที่วัดได้เฉพาะไฟ DC:
+หากนำไปต่อกับไฟสลับ (AC) 50 Hz ทิศทางของแรงบิดจะกลับทิศไปมา 50 ครั้งต่อวินาที ความเฉื่อยเชิงกล (Inertia) ของขดลวดทำให้เข็มขยับตามไม่ทัน จึงชี้ที่ค่าเฉลี่ยใน 1 คาบ:
+$$I_{\text{avg}} = \frac{1}{T} \int_0^T I_m \sin(\omega t)\, dt = 0$$
+เข็มชี้จึงสั่นอยู่ที่ขีด 0 หากต้องการวัดไฟ AC ต้องต่อร่วมกับวงจรเรียงกระแส (Rectifier) ก่อนเสมอ</t>
         </is>
       </c>
       <c r="L49" s="5" t="inlineStr">
@@ -4988,7 +5029,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>การคำนวณแรงบิดบิดเบนและมุมเบี่ยงเบนของมิเตอร์ PMMC</t>
+          <t>การคำนวณแรงบิดบิดเบนและมุมเบี่ยงเบนของมิเตอร์ PMMC (การบ้านข้อ 1)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -4998,64 +5039,60 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Homework Chapter 10 ข้อ 1 &amp; Past Exam</t>
+          <t>Homework Chapter 10 ข้อ 1 (Official Problem 1)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>A PMMC coil has N = 100 turns, width w = 2 cm, length l = 3 cm, and sits in a uniform radial flux density B = 0.2 T. The spring constant is C = 1.2 x 10^-6 N*m/degree. Calculate the deflecting torque and pointer deflection angle when carrying a current of 1 mA.</t>
+          <t>A moving coil instrument has N = 150 turns, coil area A = 100 mm^2, and operates in a magnetic flux density B = 0.15 T. The spring constant is C = 2 x 10^-6 N*m/degree. Calculate the deflecting torque Td and pointer deflection angle theta when carrying a current of I = 5 mA.</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>ขดลวด PMMC มีจำนวนรอบ N = 100 รอบ, ความกว้าง w = 2 cm, ความยาว l = 3 cm วางตัวในสนามแม่เหล็กสม่ำเสมอ B = 0.2 T สปริงควบคุมมีค่าคงที่ C = 1.2 x 10^-6 N*m/degree จงคำนวณแรงบิดบิดเบน (Deflecting Torque) และมุมเบี่ยงเบนของเข็มชี้ (theta) เมื่อมีกระแสไหล 1 mA</t>
+          <t>ขดลวดเคลื่อนที่ของเครื่องมือวัดมีจำนวนรอบ N = 150 รอบ, พื้นที่หน้าตัดขดลวด A = 100 mm^2 วางตัวในสนามแม่เหล็ก B = 0.15 T สปริงควบคุมมีค่าคงที่ C = 2 x 10^-6 N*m/degree จงคำนวณหาแรงบิดบิดเบน (Td) และมุมเบี่ยงเบนของเข็มชี้ (theta) เมื่อมีกระแสไหล I = 5 mA (การบ้านบทที่ 10 ข้อ 1)</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>$$A = w \cdot l = (0.02)(0.03) = 6 \times 10^{-4}\text{ m}^2$$
+          <t>$$A = 100\text{ mm}^2 = 100 \times 10^{-6}\text{ m}^2 = 10^{-4}\text{ m}^2$$
 $$T_d = B \cdot I \cdot N \cdot A$$
 $$\theta = \frac{T_d}{C}$$</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>1. Calculate Coil Area:
-A = 0.02 m * 0.03 m = 6 x 10^-4 m^2
-2. Calculate Deflecting Torque (Td):
-Td = B * I * N * A
-Td = (0.2 T) * (1 x 10^-3 A) * (100 turns) * (6 x 10^-4 m^2)
-Td = 1.2 x 10^-5 N*m
-3. Calculate Deflection Angle (theta):
-At equilibrium, Td = Tc = C * theta
-theta = Td / C
-theta = (1.2 x 10^-5 N*m) / (1.2 x 10^-6 N*m/degree)
-theta = 10 degrees.</t>
+          <t>1. Convert Coil Area to SI Units ($m^2$):
+$$A = 100\text{ mm}^2 \times \left(\frac{1\text{ m}}{1000\text{ mm}}\right)^2 = 100 \times 10^{-6}\text{ m}^2 = 10^{-4}\text{ m}^2$$
+2. Calculate Deflecting Torque ($T_d$):
+$$T_d = B \cdot I \cdot N \cdot A$$
+$$T_d = (0.15\text{ T}) \times (5 \times 10^{-3}\text{ A}) \times 150 \times (10^{-4}\text{ m}^2)$$
+$$T_d = 1.125 \times 10^{-5}\text{ N}\cdot\text{m}$$
+3. Calculate Pointer Deflection Angle ($\theta$):
+At steady deflection equilibrium ($T_d = T_c = C \cdot \theta$):
+$$\theta = \frac{T_d}{C} = \frac{1.125 \times 10^{-5}\text{ N}\cdot\text{m}}{2 \times 10^{-6}\text{ N}\cdot\text{m/deg}} = 5.625^\circ$$</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>1. คำนวณพื้นที่หน้าตัดขดลวด A:
-A = กว้าง x ยาว = 0.02 m x 0.03 m = 6 x 10^-4 m^2
-2. คำนวณแรงบิดบิดเบน Td:
-Td = B * I * N * A
-Td = (0.2 T) * (1 x 10^-3 A) * 100 รอบ * (6 x 10^-4 m^2)
-Td = 1.2 x 10^-5 N*m
-3. คำนวณมุมเบี่ยงเบนของเข็มชี้ theta:
-ที่สภาวะสมดุล Td = Tc = C * theta
-theta = Td / C
-theta = (1.2 x 10^-5 N*m) / (1.2 x 10^-6 N*m/degree)
-theta = 10 องศา</t>
+          <t>1. แปลงหน่วยพื้นที่หน้าตัดเป็นตารางเมตร ($m^2$):
+$$A = 100\text{ mm}^2 \times 10^{-6}\text{ m}^2/\text{mm}^2 = 10^{-4}\text{ m}^2$$
+2. คำนวณแรงบิดบิดเบน ($T_d$):
+$$T_d = B \cdot I \cdot N \cdot A$$
+$$T_d = (0.15\text{ T}) \times (5 \times 10^{-3}\text{ A}) \times 150 \times (10^{-4}\text{ m}^2)$$
+$$T_d = 1.125 \times 10^{-5}\text{ N}\cdot\text{m}$$
+3. คำนวณมุมเบี่ยงเบนของเข็มชี้ ($\theta$):
+ที่สภาวะสมดุล ($T_d = T_c = C \cdot \theta$):
+$$\theta = \frac{T_d}{C} = \frac{1.125 \times 10^{-5}\text{ N}\cdot\text{m}}{2 \times 10^{-6}\text{ N}\cdot\text{m/deg}} = 5.625^\circ$$</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>Always convert dimensions from cm to meters (m) to avoid calculation errors by factors of 10,000.</t>
+          <t>Always convert dimensions from mm^2 or cm^2 to m^2 (100 mm^2 = 10^-4 m^2). Failure to convert causes error by 1,000,000x.</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>ข้อควรระวัง: ต้องแปลงหน่วยมิติขดลวดจากเซนติเมตร (cm) เป็นเมตร (m) ก่อนเสมอ เพื่อไม่ให้คำนวณพื้นที่ผิดพลาดไป 10,000 เท่า</t>
+          <t>ข้อควรระวัง: ต้องแปลงหน่วยพื้นที่หน้าตัดจาก mm^2 เป็น m^2 เสมอ (100 mm^2 = 10^-4 m^2) มิฉะนั้นค่าแรงบิดจะผิดไป 1 ล้านเท่า</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr"/>
@@ -5084,7 +5121,7 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>การออกแบบดีซีแอมมิเตอร์ (DC Ammeter) ทั้งกรณีมีและไม่มีความต้านทาน CDRX</t>
+          <t>การออกแบบดีซีแอมมิเตอร์ ทั้งกรณีไม่มีและมีค่าแดมปิ้งวิกฤต CDRX (การบ้านข้อ 2)</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -5094,67 +5131,76 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Homework Chapter 10 ข้อ 2 &amp; Final Exam</t>
+          <t>Homework Chapter 10 ข้อ 2 (Official Problem 2)</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>A Galvanometer has internal resistance Rm = 100 ohms, full-scale current Ifsd = 1 mA, and Critical Damping Resistance CDRX = 900 ohms. Design a DC Ammeter to measure full scale I = 1 A for:
+          <t>A Galvanometer has internal resistance Rg = 50 ohms, full-scale current Ig = 10 mA, and Critical Damping Resistance CDRX = 400 ohms. Design a DC Ammeter to measure full scale I = 100 mA for:
 (a) Pure circuit without CDRX
 (b) Circuit with CDRX (damping resistor).</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>กัลวาโนมิเตอร์ตัวหนึ่งมีความต้านทานภายใน Rm = 100 โอห์ม, พิกัดกระแสเต็มสเกล Ifsd = 1 mA, และมีความต้านทานแดมปิ้งวิกฤต CDRX = 900 โอห์ม จงออกแบบแอมมิเตอร์วัดกระแสเต็มสเกล I = 1 A สำหรับ:
-(a) วงจรปกติที่ไม่มีความต้านทาน CDRX
-(b) วงจรที่มีความต้านทานแดมปิ้ง CDRX ร่วมด้วย</t>
+          <t>กัลวาโนมิเตอร์ตัวหนึ่งมีความต้านทานภายใน Rg = 50 โอห์ม, กระแสเต็มสเกล Ig = 10 mA, และความต้านทานแดมปิ้งวิกฤต CDRX = 400 โอห์ม จงออกแบบดีซีแอมมิเตอร์วัดกระแสเต็มสเกล I = 100 mA สำหรับ:
+(a) วงจรปกติไม่มีความต้านทาน CDRX
+(b) วงจรที่มีความต้านทานแดมปิ้ง CDRX ร่วมด้วย (การบ้านบทที่ 10 ข้อ 2)</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>$$\text{Without CDRX: } R_{\text{sh}} = \frac{I_{\text{fsd}} R_m}{I - I_{\text{fsd}}} = \frac{R_m}{m - 1}$$
-$$\text{With CDRX: Series resistor } R_s = \text{CDRX} - R_m$$
-$$R_{\text{sh}}' = \frac{I_{\text{fsd}} (R_m + R_s)}{I - I_{\text{fsd}}} = \frac{I_{\text{fsd}} \cdot \text{CDRX}}{I - I_{\text{fsd}}}$$
-$$\text{Total Meter Resistance: } R_{\text{in}} = R_{\text{sh}} \parallel (R_m + R_s)$$</t>
+          <t>$$\text{Without CDRX: } R_{\text{sh}} = \frac{I_g R_g}{I - I_g} = \frac{R_g}{m - 1}$$
+$$\text{With CDRX: Series resistor } R_s = \text{CDRX} - R_g = 400 - 50 = 350\;\Omega$$
+$$R_{\text{branch}} = R_g + R_s = \text{CDRX} = 400\;\Omega$$
+$$R_{\text{sh}}' = \frac{I_g \cdot R_{\text{branch}}}{I - I_g} = \frac{I_g \cdot \text{CDRX}}{I - I_g}$$
+$$R_{\text{in}} = R_{\text{sh}}' \parallel R_{\text{branch}}$$</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
           <t>1. Part (a) Without CDRX:
-- Shunt resistor Rsh is connected in parallel with Rm:
-I_sh = I - Ifsd = 1 A - 0.001 A = 0.999 A
-Rsh = (Ifsd * Rm) / (I - Ifsd) = (0.001 * 100) / 0.999 = 0.1001 ohms.
-2. Part (b) With CDRX:
-- To achieve critical damping, the total resistance across meter terminals must equal CDRX = 900 ohms.
-- Add series resistor Rs = CDRX - Rm = 900 - 100 = 800 ohms.
-- Now the effective meter branch resistance is (Rm + Rs) = CDRX = 900 ohms.
-- New Shunt Resistor Rsh':
-Rsh' = (Ifsd * CDRX) / (I - Ifsd) = (0.001 * 900) / 0.999 = 0.9009 ohms.</t>
+Shunt current bypassing the coil:
+$$I_{\text{sh}} = I - I_g = 100\text{ mA} - 10\text{ mA} = 90\text{ mA} = 0.090\text{ A}$$
+Shunt resistor $R_{\text{sh}}$:
+$$R_{\text{sh}} = \frac{I_g \cdot R_g}{I - I_g} = \frac{(0.010\text{ A})(50\;\Omega)}{0.090\text{ A}} = \frac{0.50}{0.090} = 5.556\;\Omega$$
+2. Part (b) With Critical Damping Resistance (CDRX = 400 ohms):
+To ensure critical damping in an ammeter, insert a series damping resistor $R_s$ in the galvanometer branch:
+$$R_s = \text{CDRX} - R_g = 400\;\Omega - 50\;\Omega = 350\;\Omega$$
+Effective meter branch resistance:
+$$R_{\text{branch}} = R_g + R_s = 400\;\Omega$$
+New shunt resistor $R_{\text{sh}}'$:
+$$R_{\text{sh}}' = \frac{I_g \cdot R_{\text{branch}}}{I - I_g} = \frac{(0.010\text{ A})(400\;\Omega)}{0.090\text{ A}} = \frac{4.0}{0.090} = 44.444\;\Omega$$
+Total ammeter input resistance:
+$$R_{\text{in}} = R_{\text{sh}}' \parallel R_{\text{branch}} = \frac{(44.444)(400)}{44.444 + 400} = 40.0\;\Omega$$</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
           <t>1. ข้อ (a) กรณีไม่มีความต้านทาน CDRX:
-- ตัวต้านทานชันต์ Rsh ต่อขนานกับขดลวดมิเตอร์ Rm เพื่อแบ่งกระแสส่วนเกินออกไป:
-I_sh = I - Ifsd = 1 A - 0.001 A = 0.999 A
-Rsh = (Ifsd * Rm) / (I - Ifsd) = (0.001 * 100) / 0.999 = 0.1001 โอห์ม
-2. ข้อ (b) กรณีมีค่าแดมปิ้งวิกฤต CDRX:
-- ขดลวดมิเตอร์ต้องเห็นความต้านทานรวมเท่ากับ CDRX = 900 โอห์ม เพื่อให้เข็มชี้หยุดนิ่งเร็วที่สุดโดยไม่แกว่ง
-- ต่อตัวต้านทานอนุกรม Rs เพิ่มในขามิเตอร์: Rs = CDRX - Rm = 900 - 100 = 800 โอห์ม
-- ค่าความต้านทานรวมในกิ่งมิเตอร์กลายเป็น (Rm + Rs) = CDRX = 900 โอห์ม
-- คำนวณค่าตัวต้านทานชันต์ใหม่ Rsh':
-Rsh' = (Ifsd * CDRX) / (I - Ifsd) = (0.001 * 900) / 0.999 = 0.9009 โอห์ม</t>
+กระแสที่ต้องแบ่งไหลผ่านตัวต้านทานชันต์:
+$$I_{\text{sh}} = I - I_g = 100\text{ mA} - 10\text{ mA} = 90\text{ mA} = 0.090\text{ A}$$
+คำนวณค่าตัวต้านทานชันต์ $R_{\text{sh}}$:
+$$R_{\text{sh}} = \frac{I_g \cdot R_g}{I - I_g} = \frac{(0.010\text{ A})(50\;\Omega)}{0.090\text{ A}} = \frac{0.50}{0.090} = 5.556\;\Omega$$
+2. ข้อ (b) กรณีมีค่าแดมปิ้งวิกฤต (CDRX = 400 ohms):
+เพื่อให้ขดลวดมิเตอร์เห็นความต้านทานรวมเท่ากับ CDRX พอดี ต้องต่อตัวต้านทานอนุกรม $R_s$ ในกิ่งมิเตอร์:
+$$R_s = \text{CDRX} - R_g = 400\;\Omega - 50\;\Omega = 350\;\Omega$$
+ความต้านทานรวมในกิ่งมิเตอร์กลายเป็น:
+$$R_{\text{branch}} = R_g + R_s = 400\;\Omega$$
+คำนวณค่าตัวต้านทานชันต์ใหม่ $R_{\text{sh}}'$:
+$$R_{\text{sh}}' = \frac{I_g \cdot R_{\text{branch}}}{I - I_g} = \frac{(0.010\text{ A})(400\;\Omega)}{0.090\text{ A}} = \frac{4.0}{0.090} = 44.444\;\Omega$$
+ความต้านทานอินพุตรวมของแอมมิเตอร์:
+$$R_{\text{in}} = R_{\text{sh}}' \parallel R_{\text{branch}} = \frac{(44.444)(400)}{44.444 + 400} = 40.0\;\Omega$$</t>
         </is>
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>Do not connect CDRX in parallel with Rm! Rs is connected in SERIES with Rm so their sum equals CDRX, and then Rsh is connected in parallel with the entire combination.</t>
+          <t>In Ammeters, CDRX requires a SERIES resistor Rs. Do not connect CDRX in parallel with Rg!</t>
         </is>
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>ข้อผิดบ่อย: ตัวต้านทานปรับแดมปิ้ง Rs ต้องต่อ 'อนุกรม' เข้ากับ Rm (เพื่อให้ได้ผลรวมเป็น CDRX) จากนั้นจึงนำ Rsh มาต่อ 'ขนาน' ร่วมภายนอก</t>
+          <t>ข้อผิดบ่อย: ในแอมมิเตอร์ ตัวต้านทานปรับแดมปิ้ง Rs ต้องต่อ 'อนุกรม' เข้ากับ Rg เพื่อให้ได้ค่ารวมเป็น CDRX แล้วจึงนำ Rsh มาขนานภายนอก</t>
         </is>
       </c>
       <c r="N51" s="4" t="inlineStr">
@@ -5191,7 +5237,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>การออกแบบดีซีโวลต์มิเตอร์ (DC Voltmeter) ทั้งกรณีมีและไม่มีความต้านทาน CDRX</t>
+          <t>การออกแบบดีซีโวลต์มิเตอร์ ทั้งกรณีไม่มีและมีค่าแดมปิ้งวิกฤต CDRX (การบ้านข้อ 3)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -5201,59 +5247,73 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Homework Chapter 10 ข้อ 3 &amp; Final Exam</t>
+          <t>Homework Chapter 10 ข้อ 3 (Official Problem 3)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>A Galvanometer has Rm = 100 ohms, Ifsd = 1 mA, and CDRX = 900 ohms. Design a DC Voltmeter to measure full-scale V = 100 V for:
+          <t>A Galvanometer has internal resistance Rg = 50 ohms, full-scale current Ig = 10 mA, and Critical Damping Resistance CDRX = 400 ohms. Design a DC Voltmeter to measure full scale V = 50 V for:
 (a) Pure circuit without CDRX
 (b) Circuit with CDRX (damping resistor).</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>กัลวาโนมิเตอร์ตัวเดิม Rm = 100 โอห์ม, Ifsd = 1 mA และ CDRX = 900 โอห์ม จงออกแบบดีซีโวลต์มิเตอร์วัดแรงดันเต็มสเกล V = 100 V สำหรับ:
+          <t>กัลวาโนมิเตอร์ตัวเดิมมีความต้านทานภายใน Rg = 50 โอห์ม, กระแสเต็มสเกล Ig = 10 mA, และความต้านทานแดมปิ้งวิกฤต CDRX = 400 โอห์ม จงออกแบบดีซีโวลต์มิเตอร์วัดแรงดันเต็มสเกล V = 50 V สำหรับ:
 (a) วงจรปกติไม่มีความต้านทาน CDRX
-(b) วงจรที่มีความต้านทานแดมปิ้ง CDRX ร่วมด้วย</t>
+(b) วงจรที่มีความต้านทานแดมปิ้ง CDRX ร่วมด้วย (การบ้านบทที่ 10 ข้อ 3)</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>$$\text{Without CDRX: } R_s = \frac{V}{I_{\text{fsd}}} - R_m$$
-$$\text{With CDRX: Shunt damping resistor } R_p = \text{CDRX} = 900\;\Omega$$
-$$I_{\text{total}} = I_{\text{fsd}} + I_p = I_{\text{fsd}} \left(1 + \frac{R_m}{R_p}\right)$$
-$$R_s' = \frac{V - V_m}{I_{\text{total}}} = \frac{V - I_{\text{fsd}} R_m}{I_{\text{total}}}$$
-$$\text{Sensitivity: } S = \frac{1}{I_{\text{fsd}}} \;(\Omega/\text{V})$$</t>
+          <t>$$\text{Without CDRX: } R_s = \frac{V}{I_g} - R_g$$
+$$\text{With CDRX: Parallel damping resistor } R_p = \text{CDRX} = 400\;\Omega$$
+$$V_m = I_g \cdot R_g \qquad I_p = \frac{V_m}{R_p}$$
+$$I_{\text{total}} = I_g + I_p = I_g \left(1 + \frac{R_g}{R_p}\right)$$
+$$R_s' = \frac{V - V_m}{I_{\text{total}}}$$
+$$\text{Sensitivity: } S = \frac{1}{I_{\text{total}}} \;(\Omega/\text{V})$$</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
           <t>1. Part (a) Without CDRX:
-- Total required resistance R_total = V / Ifsd = 100 V / 0.001 A = 100,000 ohms (100 k-ohms).
-- Multiplier series resistor Rs = R_total - Rm = 100,000 - 100 = 99,900 ohms (99.9 k-ohms).
-2. Part (b) With CDRX:
-- To provide critical damping in a voltmeter, a parallel damping resistor Rp = CDRX = 900 ohms is connected in PARALLEL with Rm.
-- Voltage drop across coil at full scale: Vm = Ifsd * Rm = 0.001 A * 100 ohms = 0.1 V.
-- Current through Rp: Ip = Vm / Rp = 0.1 V / 900 ohms = 0.1111 mA.
-- Total circuit current: I_total = Ifsd + Ip = 1.0 mA + 0.1111 mA = 1.1111 mA.
-- Multiplier series resistor Rs':
-Rs' = (V - Vm) / I_total = (100 V - 0.1 V) / (1.1111 x 10^-3 A) = 89,910 ohms (89.91 k-ohms).</t>
+Total circuit resistance required:
+$$R_{\text{total}} = \frac{V}{I_g} = \frac{50\text{ V}}{0.010\text{ A}} = 5,000\;\Omega = 5\text{ k}\Omega$$
+Multiplier series resistor $R_s$:
+$$R_s = R_{\text{total}} - R_g = 5,000\;\Omega - 50\;\Omega = 4,950\;\Omega = 4.95\text{ k}\Omega$$
+2. Part (b) With Critical Damping Resistance (CDRX = 400 ohms):
+For a voltmeter, connect damping resistor $R_p = \text{CDRX} = 400\;\Omega$ in PARALLEL across the meter movement:
+- Voltage drop across coil at full scale:
+$$V_m = I_g \cdot R_g = (0.010\text{ A})(50\;\Omega) = 0.5\text{ V}$$
+- Current drawn by parallel damping resistor $R_p$:
+$$I_p = \frac{V_m}{R_p} = \frac{0.5\text{ V}}{400\;\Omega} = 1.25\text{ mA} = 0.00125\text{ A}$$
+- Total current entering the voltmeter:
+$$I_{\text{total}} = I_g + I_p = 10\text{ mA} + 1.25\text{ mA} = 11.25\text{ mA} = 0.01125\text{ A}$$
+- Multiplier series resistor $R_s'$:
+$$R_s' = \frac{V - V_m}{I_{\text{total}}} = \frac{50\text{ V} - 0.5\text{ V}}{0.01125\text{ A}} = \frac{49.5\text{ V}}{0.01125\text{ A}} = 4,400\;\Omega = 4.4\text{ k}\Omega$$
+- Voltmeter sensitivity:
+$$S = \frac{1}{I_{\text{total}}} = \frac{1}{0.01125\text{ A}} = 88.89\;\Omega/\text{V}$$</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
           <t>1. ข้อ (a) กรณีไม่มีความต้านทาน CDRX:
-- ความต้านทานรวมของวงจรโวลต์มิเตอร์: R_total = V / Ifsd = 100 V / 0.001 A = 100,000 โอห์ม (100 k-ohms)
-- ตัวต้านทานอนุกรมตัวคูณแรงดัน (Multiplier Resistor Rs):
-Rs = R_total - Rm = 100,000 - 100 = 99,900 โอห์ม (99.9 k-ohms)
-2. ข้อ (b) กรณีมีค่าแดมปิ้งวิกฤต CDRX:
-- สำหรับโวลต์มิเตอร์ การให้ขดลวดมิเตอร์เห็นความต้านทาน CDRX ต้องต่อตัวต้านทานขนาน Rp = CDRX = 900 โอห์ม 'คร่อมขนาน' กับขดลวดมิเตอร์ Rm
-- แรงดันตกคร่อมขดลวดเมื่อเต็มสเกล: Vm = Ifsd * Rm = 0.001 A * 100 โอห์ม = 0.1 V
-- กระแสที่ไหลผ่าน Rp: Ip = Vm / Rp = 0.1 V / 900 โอห์ม = 0.1111 mA
-- กระแสรวมที่เข้าวงจรโวลต์มิเตอร์: I_total = Ifsd + Ip = 1 mA + 0.1111 mA = 1.1111 mA
-- ตัวต้านทานอนุกรม Rs':
-Rs' = (V - Vm) / I_total = (100 - 0.1) / (1.1111 x 10^-3 A) = 89,910 โอห์ม (89.91 k-ohms)</t>
+ความต้านทานรวมของวงจรโวลต์มิเตอร์:
+$$R_{\text{total}} = \frac{V}{I_g} = \frac{50\text{ V}}{0.010\text{ A}} = 5,000\;\Omega = 5\text{ k}\Omega$$
+ตัวต้านทานตัวคูณแรงดันอนุกรม ($R_s$):
+$$R_s = R_{\text{total}} - R_g = 5,000\;\Omega - 50\;\Omega = 4,950\;\Omega = 4.95\text{ k}\Omega$$
+2. ข้อ (b) กรณีมีค่าแดมปิ้งวิกฤต (CDRX = 400 ohms):
+สำหรับโวลต์มิเตอร์ การให้ขดลวดเห็นค่าแดมปิ้ง ต้องต่อตัวต้านทาน $R_p = \text{CDRX} = 400\;\Omega$ แบบ 'ขนาน' คร่อมขดลวด:
+- แรงดันตกคร่อมขดลวดเมื่อเต็มสเกล:
+$$V_m = I_g \cdot R_g = (0.010\text{ A})(50\;\Omega) = 0.5\text{ V}$$
+- กระแสที่ไหลผ่านตัวต้านทานขนาน $R_p$:
+$$I_p = \frac{V_m}{R_p} = \frac{0.5\text{ V}}{400\;\Omega} = 1.25\text{ mA} = 0.00125\text{ A}$$
+- กระแสรวมที่เข้าสู่วงจรโวลต์มิเตอร์:
+$$I_{\text{total}} = I_g + I_p = 10\text{ mA} + 1.25\text{ mA} = 11.25\text{ mA} = 0.01125\text{ A}$$
+- ตัวต้านทานตัวคูณแรงดันอนุกรมใหม่ ($R_s'$):
+$$R_s' = \frac{V - V_m}{I_{\text{total}}} = \frac{50\text{ V} - 0.5\text{ V}}{0.01125\text{ A}} = \frac{49.5\text{ V}}{0.01125\text{ A}} = 4,400\;\Omega = 4.4\text{ k}\Omega$$
+- ความไวของโวลต์มิเตอร์ (Sensitivity: $S$):
+$$S = \frac{1}{I_{\text{total}}} = \frac{1}{0.01125\text{ A}} = 88.89\;\Omega/\text{V}$$</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -5300,7 +5360,7 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>การออกแบบดีซีแอมมิเตอร์หลายย่านวัด (Multi-Range) ร่วมกับความต้านทานแดมปิ้ง CDRX</t>
+          <t>การออกแบบดีซีแอมมิเตอร์หลายย่านวัดร่วมกับความต้านทานแดมปิ้งวิกฤต CDRX (ข้อสอบไฟนอล 3.5)</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -5315,57 +5375,64 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Design a 3-range DC Ammeter for ranges I1 = 10 mA, I2 = 50 mA, and I3 = 100 mA using a PMMC meter with Rm = 50 ohms, Ifsd = 1 mA, and CDRX = 450 ohms. Determine the damping resistor Rs and each individual shunt resistor Rsh1, Rsh2, and Rsh3.</t>
+          <t>A galvanometer has sensitivity 0.1 uA/mm, full scale deflection 10 mm, coil resistance Rg = 100 ohms, and critical damping resistance CDRX = 400 ohms. Design a 3-range DC ammeter for I1 = 1 mA, I2 = 50 mA, and I3 = 1 A using individual shunts. Determine damping resistor Rs and shunt resistors R11, R21, R31.</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>จงออกแบบดีซีแอมมิเตอร์ 3 ย่านวัด: I1 = 10 mA, I2 = 50 mA และ I3 = 100 mA โดยใช้กัลวาโนมิเตอร์ Rm = 50 โอห์ม, Ifsd = 1 mA และ CDRX = 450 โอห์ม จงคำนวณหาค่าความต้านทานแดมปิ้ง Rs และความต้านทานชันต์แต่ละย่านวัด Rsh1, Rsh2, Rsh3</t>
+          <t>กัลวาโนมิเตอร์มีความไว 0.1 uA/mm, สเกลเบี่ยงเบนเต็มที่ 10 mm, ความต้านทานขดลวด Rg = 100 โอห์ม, และความต้านทานแดมปิ้งวิกฤต CDRX = 400 โอห์ม จงออกแบบแอมมิเตอร์วัดกระแสตรง 3 ย่านวัด: I1 = 1 mA, I2 = 50 mA, และ I3 = 1 A โดยคำนวณหาค่าความต้านทานแดมปิ้งอนุกรม Rs และความต้านทานชันต์แต่ละย่านวัด R11, R21, R31 (ข้อสอบไฟนอลข้อ 3.5 หน้า 29)</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>$$R_s = \text{CDRX} - R_m = 450 - 50 = 400\;\Omega$$
-$$R_{\text{branch}} = R_m + R_s = 450\;\Omega$$
-$$R_{\text{sh},n} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_n - I_{\text{fsd}}} = \frac{(0.001)(450)}{I_n - 0.001}$$</t>
+          <t>$$I_{\text{fsd}} = \text{Sensitivity} \times \text{Scale Length} = (0.1\;\mu\text{A/mm})(10\text{ mm}) = 1\;\mu\text{A} = 10^{-6}\text{ A}$$
+$$R_s = \text{CDRX} - R_g = 400\;\Omega - 100\;\Omega = 300\;\Omega$$
+$$R_{\text{branch}} = R_g + R_s = 400\;\Omega$$
+$$R_{n1} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_n - I_{\text{fsd}}}$$</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>1. Determine Series Damping Resistor Rs:
-Rs = CDRX - Rm = 450 - 50 = 400 ohms.
-Effective meter branch resistance: R_branch = Rm + Rs = 450 ohms.
-2. Calculate Shunt Resistors for Each Range:
-- Range 1 (10 mA):
-Rsh1 = (0.001 * 450) / (0.010 - 0.001) = 0.450 / 0.009 = 50.0 ohms.
-- Range 2 (50 mA):
-Rsh2 = (0.001 * 450) / (0.050 - 0.001) = 0.450 / 0.049 = 9.184 ohms.
-- Range 3 (100 mA):
-Rsh3 = (0.001 * 450) / (0.100 - 0.001) = 0.450 / 0.099 = 4.545 ohms.</t>
+          <t>1. Determine Full-Scale Galvanometer Current ($I_{\text{fsd}}$):
+$$I_{\text{fsd}} = 0.1\;\mu\text{A/mm} \times 10\text{ mm} = 1\;\mu\text{A} = 10^{-6}\text{ A}$$
+2. Determine Series Damping Resistor ($R_s$):
+$$R_s = \text{CDRX} - R_g = 400\;\Omega - 100\;\Omega = 300\;\Omega$$
+Total meter branch resistance:
+$$R_{\text{branch}} = R_g + R_s = 400\;\Omega$$
+3. Calculate Shunt Resistors for Each Range:
+- Range 1 ($I_1 = 1\text{ mA} = 10^{-3}\text{ A}$):
+$$R_{11} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_1 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{10^{-3}\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.000999} = 0.4004\;\Omega$$
+- Range 2 ($I_2 = 50\text{ mA} = 0.05\text{ A}$):
+$$R_{21} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_2 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{0.05\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.049999} = 0.00800\;\Omega$$
+- Range 3 ($I_3 = 1\text{ A}$):
+$$R_{31} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_3 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{1.0\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.999999} = 0.000400\;\Omega$$</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>1. คำนวณตัวต้านทานแดมปิ้งอนุกรม Rs:
-Rs = CDRX - Rm = 450 - 50 = 400 โอห์ม
-ส่งผลให้ความต้านทานกิ่งมิเตอร์มีค่าเท่ากับ CDRX พอดี คือ R_branch = 450 โอห์ม
-2. คำนวณค่า Shunt Resistor ในแต่ละย่านวัด:
-- ย่านที่ 1 (I1 = 10 mA):
-Rsh1 = (0.001 * 450) / (0.010 - 0.001) = 0.45 / 0.009 = 50.0 โอห์ม
-- ย่านที่ 2 (I2 = 50 mA):
-Rsh2 = (0.001 * 450) / (0.050 - 0.001) = 0.45 / 0.049 = 9.184 โอห์ม
-- ย่านที่ 3 (I3 = 100 mA):
-Rsh3 = (0.001 * 450) / (0.100 - 0.001) = 0.45 / 0.099 = 4.545 โอห์ม</t>
+          <t>1. คำนวณพิกัดกระแสเต็มสเกลของกัลวาโนมิเตอร์ ($I_{\text{fsd}}$):
+$$I_{\text{fsd}} = 0.1\;\mu\text{A/mm} \times 10\text{ mm} = 1\;\mu\text{A} = 10^{-6}\text{ A}$$
+2. คำนวณตัวต้านทานแดมปิ้งอนุกรม ($R_s$):
+$$R_s = \text{CDRX} - R_g = 400\;\Omega - 100\;\Omega = 300\;\Omega$$
+ความต้านทานรวมในกิ่งมิเตอร์:
+$$R_{\text{branch}} = R_g + R_s = 400\;\Omega$$
+3. คำนวณหาค่าความต้านทานชันต์แต่ละย่านวัด:
+- ย่านวัดที่ 1 ($I_1 = 1\text{ mA}$):
+$$R_{11} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_1 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{10^{-3}\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.000999} = 0.4004\;\Omega$$
+- ย่านวัดที่ 2 ($I_2 = 50\text{ mA}$):
+$$R_{21} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_2 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{0.05\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.049999} = 0.00800\;\Omega$$
+- ย่านวัดที่ 3 ($I_3 = 1\text{ A}$):
+$$R_{31} = \frac{I_{\text{fsd}} \cdot R_{\text{branch}}}{I_3 - I_{\text{fsd}}} = \frac{(10^{-6}\text{ A})(400\;\Omega)}{1.0\text{ A} - 10^{-6}\text{ A}} = \frac{0.0004}{0.999999} = 0.000400\;\Omega$$</t>
         </is>
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
-          <t>Notice that higher current range requires SMALLER shunt resistance (Rsh3 &lt; Rsh2 &lt; Rsh1) because more current must be bypassed around the meter movement.</t>
+          <t>Notice that higher current range requires SMALLER shunt resistance (R31 &lt; R21 &lt; R11) because more current must be bypassed around the meter movement.</t>
         </is>
       </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
-          <t>ข้อสังเกต: ยิ่งย่านวัดกระแสสูง ค่าความต้านทานชันต์ยิ่งต้องมีค่าน้อยลง (Rsh3 &lt; Rsh2 &lt; Rsh1) เพื่อให้กระแสส่วนใหญ่ไหลบายพาสผ่านตัวชันต์ไป</t>
+          <t>ข้อสังเกต: ยิ่งย่านวัดกระแสสูง ค่าความต้านทานชันต์ยิ่งต้องมีค่าน้อยลง (R31 &lt; R21 &lt; R11) เพื่อให้กระแสส่วนใหญ่ไหลบายพาสผ่านตัวชันต์ไป</t>
         </is>
       </c>
       <c r="N53" s="4" t="inlineStr">
@@ -5436,19 +5503,33 @@
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>1. What is an Ayrton Shunt:
-A tapped chain of resistors (Ra + Rb + Rc) continuously connected across the meter movement. Changing ranges alters which portion acts as shunt and which portion acts as series resistance.
-2. Decisive Advantage over Individual Shunts:
-- Make-Before-Break Safety: In individual shunts, if the rotary switch momentarily disconnects between contacts, the FULL circuit current would blast through the fragile meter coil (Rm), destroying it immediately.
-- Ayrton shunt ensures the meter movement is ALWAYS shunted by resistance, preventing destructive overload during range switching.</t>
+A tapped series chain of resistors ($R_a + R_b + R_c$) permanently connected in parallel across the meter movement $R_m$. Switching ranges moves the circuit input tap, altering which resistors act as shunt and which are added in series with the meter coil.
+2. Decisive Advantage Over Individual Shunts:
+- Make-Before-Break Safety: In individual shunts, if the rotary switch momentarily opens between contacts, the entire line current would blast through the fragile meter movement ($R_m$), destroying it instantly.
+- In Ayrton shunt, the meter movement is NEVER left open without a parallel bypass path during range switching.
+3. Equations for 3 Ranges:
+- Lowest current $I_1$:
+$$R_a + R_b + R_c = \frac{I_{\text{fsd}} R_m}{I_1 - I_{\text{fsd}}}$$
+- Medium current $I_2$:
+$$R_b + R_c = \frac{I_{\text{fsd}} (R_m + R_a)}{I_2}$$
+- Highest current $I_3$:
+$$R_c = \frac{I_{\text{fsd}} (R_m + R_a + R_b)}{I_3}$$</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>1. ชันต์ของแอร์ตันคืออะไร:
-คือวงจรตัวต้านทานต่ออนุกรมกันเป็นลูกโซ่ (Ra + Rb + Rc) ต่อคร่อมถาวรกับขดลวดมิเตอร์ Rm การเปลี่ยนย่านวัดทำได้โดยการย้ายตำแหน่งแท็ป ซึ่งจะทำให้ความต้านทานส่วนหนึ่งกลายมาเป็นชันต์ และอีกส่วนหนึ่งกลายเป็นตัวต้านทานอนุกรมกับมิเตอร์
-2. ข้อดีสำคัญที่สุดเหนือกว่าชันต์แบบแยกเดี่ยว:
-- ป้องกันมิเตอร์พังขณะสับสวิตช์: ในชันต์แบบเดิม หากสวิตช์หมุนเกิดจังหวะ 'หน้าสัมผัสลอย (Open-circuit)' ชั่วคราว กระแสโหลดทั้งหมดจะทะลักเข้าขดลวดมิเตอร์ Rm ทำให้ขดลวดไหม้ขาดทันที
-- วงจร Ayrton Shunt รับประกันว่าขดลวดมิเตอร์จะมีตัวต้านทานต่อขนานบายพาสกระแสอยู่ตลอดเวลาอย่างปลอดภัยแม้ขณะหมุนสวิตช์เปลี่ยนย่านวัด</t>
+          <t>1. วงจรชันต์ของแอร์ตันคืออะไร:
+คือวงจรตัวต้านทานต่ออนุกรมกัน ($R_a + R_b + R_c$) ต่อคร่อมถาวรกับขดลวดมิเตอร์ $R_m$ การเปลี่ยนย่านวัดทำได้โดยการย้ายจุดต่อแท็ป ซึ่งจะทำให้ความต้านทานบางส่วนทำหน้าที่เป็นตัวชันต์ และส่วนที่เหลือจะถูกต่ออนุกรมเข้ากับมิเตอร์
+2. ข้อดีสำคัญที่สุดเหนือกว่าชันต์แบบสวิตช์เดี่ยว:
+- ป้องกันมิเตอร์พังขณะสับสวิตช์: ในชันต์แบบเดี่ยว หากหน้าสัมผัสของสวิตช์เกิดลอย (Open-circuit) ชั่วขณะขณะหมุน กระแสโหลดทั้งหมดจะไหลทะลักเข้าขดลวดมิเตอร์ $R_m$ ทำให้ขดลวดไหม้ขาดทันที
+- วงจร Ayrton Shunt รับประกันว่าขดลวดมิเตอร์จะมีตัวต้านทานต่อขนานบายพาสกระแสอยู่ตลอดเวลาอย่างปลอดภัยแม้ขณะหมุนสวิตช์เปลี่ยนย่านวัด
+3. สมการคำนวณค่าตัวต้านทานแต่ละย่าน:
+- ย่านกระแสต่ำสุด $I_1$:
+$$R_a + R_b + R_c = \frac{I_{\text{fsd}} R_m}{I_1 - I_{\text{fsd}}}$$
+- ย่านกระแสปานกลาง $I_2$:
+$$R_b + R_c = \frac{I_{\text{fsd}} (R_m + R_a)}{I_2}$$
+- ย่านกระแสสูงสุด $I_3$:
+$$R_c = \frac{I_{\text{fsd}} (R_m + R_a + R_b)}{I_3}$$</t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
@@ -5520,7 +5601,7 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>$$S = \frac{1}{I_{\text{fsd}}} = \frac{1}{50 \times 10^{-6}} = 20,000\;\Omega/\text{V} \quad (20\text{ k}\Omega/\text{V})$$
+          <t>$$S = \frac{1}{I_{\text{fsd}}} = \frac{1}{50 \times 10^{-6}\text{ A}} = 20,000\;\Omega/\text{V} \quad (20\text{ k}\Omega/\text{V})$$
 $$R_{\text{total},1} = S \cdot V_1 = (20\text{ k}\Omega/\text{V})(10\text{ V}) = 200\text{ k}\Omega$$
 $$R_1 = R_{\text{total},1} - R_m = 200\text{ k}\Omega - 100\;\Omega = 199.9\text{ k}\Omega$$
 $$R_2 = S(V_2 - V_1) = 20\text{ k}\Omega/\text{V} \cdot (50 - 10) = 800\text{ k}\Omega$$
@@ -5529,32 +5610,30 @@
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>1. Voltmeter Sensitivity (S):
-S = 1 / Ifsd = 1 / (50 x 10^-6 A) = 20,000 ohms/V (20 k-ohm/V).
-2. Range 1 (10 V):
-R_total1 = S * 10 V = 200,000 ohms.
-R1 = R_total1 - Rm = 200,000 - 100 = 199,900 ohms (199.9 k-ohms).
-3. Range 2 (50 V):
-R_total2 = S * 50 V = 1,000,000 ohms.
-R2 = R_total2 - R_total1 = 1,000,000 - 200,000 = 800,000 ohms (800 k-ohms).
-4. Range 3 (250 V):
-R_total3 = S * 250 V = 5,000,000 ohms.
-R3 = R_total3 - R_total2 = 5,000,000 - 1,000,000 = 4,000,000 ohms (4 M-ohms).</t>
+          <t>1. Voltmeter Sensitivity ($S$):
+$$S = \frac{1}{I_{\text{fsd}}} = \frac{1}{50 \times 10^{-6}\text{ A}} = 20,000\;\Omega/\text{V} = 20\text{ k}\Omega/\text{V}$$
+2. Range 1 ($V_1 = 10\text{ V}$):
+$$R_{\text{total},1} = S \cdot V_1 = (20\text{ k}\Omega/\text{V})(10\text{ V}) = 200\text{ k}\Omega$$
+$$R_1 = R_{\text{total},1} - R_m = 200\text{ k}\Omega - 0.1\text{ k}\Omega = 199.9\text{ k}\Omega$$
+3. Range 2 ($V_2 = 50\text{ V}$):
+In a tapped series chain, each incremental resistor spans the voltage difference between adjacent ranges:
+$$R_2 = S \cdot (V_2 - V_1) = (20\text{ k}\Omega/\text{V})(50\text{ V} - 10\text{ V}) = (20\text{ k}\Omega/\text{V})(40\text{ V}) = 800\text{ k}\Omega$$
+4. Range 3 ($V_3 = 250\text{ V}$):
+$$R_3 = S \cdot (V_3 - V_2) = (20\text{ k}\Omega/\text{V})(250\text{ V} - 50\text{ V}) = (20\text{ k}\Omega/\text{V})(200\text{ V}) = 4,000\text{ k}\Omega = 4\text{ M}\Omega$$</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>1. ความไวของโวลต์มิเตอร์ (Sensitivity: S):
-S = 1 / Ifsd = 1 / (50 x 10^-6 A) = 20,000 โอห์ม/โวลต์ (20 k-ohm/V)
-2. ย่านวัดที่ 1 (V1 = 10 V):
-R_total1 = S * 10 V = 200,000 โอห์ม
-R1 = R_total1 - Rm = 200,000 - 100 = 199,900 โอห์ม (199.9 k-ohms)
-3. ย่านวัดที่ 2 (V2 = 50 V):
-R_total2 = S * 50 V = 1,000,000 โอห์ม
-R2 = R_total2 - R_total1 = 1,000,000 - 200,000 = 800,000 โอห์ม (800 k-ohms)
-4. ย่านวัดที่ 3 (V3 = 250 V):
-R_total3 = S * 250 V = 5,000,000 โอห์ม
-R3 = R_total3 - R_total2 = 5,000,000 - 1,000,000 = 4,000,000 โอห์ม (4 M-ohms)</t>
+          <t>1. ความไวของโวลต์มิเตอร์ (Sensitivity: $S$):
+$$S = \frac{1}{I_{\text{fsd}}} = \frac{1}{50 \times 10^{-6}\text{ A}} = 20,000\;\Omega/\text{V} = 20\text{ k}\Omega/\text{V}$$
+2. ย่านวัดที่ 1 ($V_1 = 10\text{ V}$):
+$$R_{\text{total},1} = S \cdot V_1 = (20\text{ k}\Omega/\text{V})(10\text{ V}) = 200\text{ k}\Omega$$
+$$R_1 = R_{\text{total},1} - R_m = 200\text{ k}\Omega - 0.1\text{ k}\Omega = 199.9\text{ k}\Omega$$
+3. ย่านวัดที่ 2 ($V_2 = 50\text{ V}$):
+ในวงจรตัวคูณแบบอนุกรมเรียงลำดับ ความต้านทานตัวถัดไปคำนวณจากผลต่างของแรงดันระหว่างสองย่านวัด:
+$$R_2 = S \cdot (V_2 - V_1) = (20\text{ k}\Omega/\text{V})(50\text{ V} - 10\text{ V}) = 800\text{ k}\Omega$$
+4. ย่านวัดที่ 3 ($V_3 = 250\text{ V}$):
+$$R_3 = S \cdot (V_3 - V_2) = (20\text{ k}\Omega/\text{V})(250\text{ V} - 50\text{ V}) = 4,000\text{ k}\Omega = 4\text{ M}\Omega$$</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -5627,33 +5706,38 @@
       <c r="I56" s="3" t="inlineStr">
         <is>
           <t>$$I = \frac{E}{R_{\text{in}} + R_x}$$
-$$R_x = 0 \implies I = I_{\text{fsd}} \quad (\text{Rightmost edge})$$
-$$R_x = R_{\text{in}} \implies I = 0.5\, I_{\text{fsd}} \quad (\text{Center of scale: } R_h)$$
-$$R_x = \infty \implies I = 0 \quad (\text{Leftmost zero current})$$</t>
+$$R_x = 0 \implies I = I_{\text{fsd}} = \frac{E}{R_{\text{in}}} \quad (\text{Far Right: } 0\;\Omega)$$
+$$R_x = R_h = R_{\text{in}} \implies I = 0.5\, I_{\text{fsd}} \quad (\text{Center of scale: } R_h)$$
+$$R_x = \infty \implies I = 0 \quad (\text{Far Left zero current: } \infty\;\Omega)$$</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
           <t>1. Circuit Topology:
-A battery E, current-limiting resistor R1, zero-adjust rheostat R2, and meter movement Rm are connected in series with the unknown resistor Rx.
-2. Calibration Points:
-- Rx = 0 (Short Circuit): Full current flows, pointer deflects to FULL SCALE (far RIGHT) = 0 ohms.
-- Rx = R_half (R_in): Total resistance doubles, current drops to 50% Ifsd, pointer sits exactly at MID-SCALE = Rh.
-- Rx = infinity (Open Circuit): Current is 0, pointer remains at REST (far LEFT) = infinity ohms.
-3. Non-linear &amp; Backwards Scale:
-Because current I = E / (R_in + Rx) is an inverse hyperbolic function of Rx, deflection is NOT linear. Scale markings are widely spaced on the right (low ohms) and heavily compressed on the left (high ohms).</t>
+An internal battery $E$, current-limiting resistor $R_1$, zero-adjust rheostat $R_2$, and galvanometer $R_m$ are all connected in series with the unknown resistance $R_x$ across test terminals.
+2. Scale Deflection Points:
+- $R_x = 0$ (Short Circuit): Maximum current flows, deflecting pointer to full-scale at the far RIGHT:
+$$I = I_{\text{fsd}} = \frac{E}{R_{\text{in}}} \implies 0\;\Omega$$
+- $R_x = R_{\text{in}} = R_h$ (Half-Scale Resistance): Total resistance doubles, halving current to exactly mid-scale:
+$$I = \frac{E}{2 R_{\text{in}}} = 0.5\, I_{\text{fsd}} \implies R_h$$
+- $R_x = \infty$ (Open Circuit): No current flows, pointer remains at rest at far LEFT:
+$$I = 0 \implies \infty\;\Omega$$
+3. Why Scale is Non-Linear &amp; Reads Backwards:
+Because current $I = E / (R_{\text{in}} + R_x)$ varies inversely with $R_x$, deflection is hyperbolic. Markings are widely spaced on the right (low ohms) and heavily compressed on the left (high ohms).</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>1. โครงสร้างวงจร:
-ประกอบด้วยแบตเตอรี่ภายใน E, ตัวต้านทานจำกัดกระแส R1, ตัวต้านทานปรับศูนย์ (Zero-adjust R2) และขดลวดมิเตอร์ Rm ต่ออนุกรมทั้งหมดเข้ากับความต้านทานที่ต้องการวัด Rx
+ประกอบด้วยแบตเตอรี่ภายใน $E$, ตัวต้านทานจำกัดกระแส $R_1$, ตัวต้านทานปรับศูนย์ ($R_2$) และขดลวดมิเตอร์ $R_m$ ต่ออนุกรมทั้งหมดเข้ากับความต้านทานที่ต้องการวัด $R_x$
 2. ตำแหน่งเข็มชี้ตามพิกัดความต้านทาน:
-- เมื่อ Rx = 0 (ช็อตปลายสายวัด): กระแสไหลสูงสุดเต็มสเกล (Ifsd) เข็มชี้เบี่ยงเบนไปสุดทาง 'ขวามือ' = อ่านค่า 0 โอห์ม
-- เมื่อ Rx = R_in (ความต้านทานเท่ากับความต้านทานภายในมิเตอร์): กระแสลดลงเหลือครึ่งหนึ่ง (0.5 Ifsd) เข็มชี้ตรง 'กึ่งกลางหน้าปัด' = จุด Half-Scale (Rh)
-- เมื่อ Rx = อินฟินิตี้ (เปิดวงจร ไม่ต่อสาย): ไม่มีกระแสไหล เข็มชี้ไม่กระดิก อยู่ที่ตำแหน่งพัก 'ซ้ายมือสุด' = อ่านค่า อินฟินิตี้
+- เมื่อ $R_x = 0$ (ช็อตปลายสายวัด): กระแสไหลสูงสุดเต็มสเกล ($I_{\text{fsd}}$) เข็มชี้เบี่ยงเบนไปสุดทาง 'ขวามือ' อ่านค่า $0\;\Omega$:
+$$I = I_{\text{fsd}} = \frac{E}{R_{\text{in}}} \implies 0\;\Omega$$
+- เมื่อ $R_x = R_{\text{in}} = R_h$ (ความต้านทานเท่ากับความต้านทานภายในมิเตอร์): ความต้านทานรวมเพิ่มเป็น 2 เท่า กระแสลดลงครึ่งหนึ่ง ($0.5 I_{\text{fsd}}$) เข็มชี้ตรง 'กึ่งกลางหน้าปัด' พอดี:
+$$I = 0.5\, I_{\text{fsd}} \implies R_h$$
+- เมื่อ $R_x = \infty$ (เปิดวงจร ไม่ต่อสาย): ไม่มีกระแสไหล ($I = 0$) เข็มชี้อยู่ที่ตำแหน่งพัก 'ซ้ายมือสุด' อ่านค่า $\infty\;\Omega$
 3. ทำไมสเกลอ่านกลับด้านและไม่สม่ำเสมอ:
-จากสมการ I = E / (R_in + Rx) กระแส I แปรผกผันกับ Rx ส่งผลให้สเกลอ่านจากขวาไปซ้าย และระยะห่างของขีดบนหน้าปัดจะไม่เท่ากัน โดยช่องจะกว้างทางฝั่งขวา (โอห์มต่ำ) และเบียดชิดกันมากทางฝั่งซ้าย (โอห์มสูง)</t>
+จากสมการ $I = E / (R_{\text{in}} + R_x)$ กระแส $I$ แปรผกผันกับ $R_x$ สเกลจึงอ่านจากขวาไปซ้าย โดยช่องจะกว้างทางฝั่งขวา (โอห์มต่ำ) และเบียดชิดกันมากทางฝั่งซ้าย (โอห์มสูง)</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
@@ -5726,33 +5810,40 @@
       <c r="I57" s="5" t="inlineStr">
         <is>
           <t>$$I_m = I_{\text{total}} \cdot \frac{R_x}{R_m + R_x}$$
-$$R_x = 0 \implies I_m = 0 \quad (\text{Leftmost edge = 0 }\Omega)$$
-$$R_x = \infty \implies I_m = I_{\text{fsd}} \quad (\text{Rightmost edge = } \infty\;\Omega)$$
-$$\text{Suited for LOW resistance measurement } (5\;\text{m}\Omega - 100\;\Omega)$$</t>
+$$R_x = 0 \implies I_m = 0 \quad (\text{Far Left edge = } 0\;\Omega)$$
+$$R_x = R_m \implies I_m = 0.5\, I_{\text{total}} \quad (\text{Center of scale = } R_m)$$
+$$R_x = \infty \implies I_m = I_{\text{fsd}} \quad (\text{Far Right edge = } \infty\;\Omega)$$
+$$\text{Measurement range: Low resistance } (5\;\text{m}\Omega - 100\;\Omega)$$</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
           <t>1. Operating Principle:
-The unknown resistor Rx is connected in PARALLEL (shunt) across the meter movement Rm, rather than in series. A series battery and switch provide supply current.
-2. Scale Behavior:
-- Rx = 0 (Short Circuit): All current bypasses through the zero-ohm short; coil current Im = 0. Pointer stays at far LEFT = 0 ohms.
-- Rx = infinity (Open Circuit): No current bypassed; full current flows through Rm, deflecting pointer to far RIGHT = infinity ohms.
-- Result: Shunt ohmmeter scale reads from LEFT TO RIGHT (0 on left, infinity on right), exactly matching voltmeter/ammeter scale direction!
+The unknown resistor $R_x$ is connected in PARALLEL (shunt) across the meter movement $R_m$, rather than in series. A series battery and resistor supply constant circuit current.
+2. Scale Deflection Points:
+- $R_x = 0$ (Short Circuit): All current bypasses through the zero-ohm short; coil current $I_m = 0$. Pointer stays at far LEFT = $0\;\Omega$:
+$$I_m = 0 \implies 0\;\Omega$$
+- $R_x = R_m$: Current splits equally; pointer deflects to mid-scale ($0.5 I_{\text{fsd}}$) = $R_m$.
+- $R_x = \infty$ (Open Circuit): No current bypassed; full current flows through $R_m$, deflecting pointer to far RIGHT = $\infty\;\Omega$:
+$$I_m = I_{\text{fsd}} \implies \infty\;\Omega$$
+Result: Shunt ohmmeter scale reads from LEFT TO RIGHT ($0$ on left, $\infty$ on right), matching normal voltmeter/ammeter scale direction!
 3. Primary Application:
-Measuring very LOW resistances (0.1 ohm to a few tens of ohms), such as motor winding coils, contact resistance, and transformer wire.</t>
+Measuring very LOW resistances ($0.01\;\Omega$ to a few tens of ohms), such as motor winding coils, contact resistance, and transformer wire.</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
           <t>1. หลักการทำงาน:
-นำความต้านทานที่ไม่ทราบค่า Rx มาต่อ 'ขนาน (Shunt)' คร่อมขดลวดมิเตอร์ Rm แทนการต่ออนุกรม
+นำความต้านทานที่ไม่ทราบค่า $R_x$ มาต่อ 'ขนาน (Shunt)' คร่อมขดลวดมิเตอร์ $R_m$ แทนการต่ออนุกรม
 2. ทิศทางสเกลหน้าปัด:
-- เมื่อ Rx = 0 (ช็อตสายวัด): กระแสทั้งหมดจะไหลลัดวงจรผ่าน Rx ทำให้ไม่มีกระแสเข้าขดลวดมิเตอร์ (Im = 0) เข็มชี้อยู่ที่ตำแหน่งพัก 'ซ้ายสุด' = 0 โอห์ม
-- เมื่อ Rx = อินฟินิตี้ (เปิดวงจร): ไม่มีกระแสแยกไหลผ่าน Rx กระแสไหลเข้าขดลวดมิเตอร์เต็มที่ เข็มชี้เบี่ยงเบนไป 'ขวาสุด' = อินฟินิตี้
-- สรุป: สเกลของโอห์มมิเตอร์แบบขนานจะอ่านจาก 'ซ้ายไปขวา' (0 อยู่ซ้าย, อินฟินิตี้อยู่ขวา) เหมือนกับโวลต์มิเตอร์และแอมมิเตอร์ทั่วไป
+- เมื่อ $R_x = 0$ (ช็อตสายวัด): กระแสทั้งหมดจะไหลลัดวงจรผ่าน $R_x$ ทำให้ไม่มีกระแสเข้าขดลวดมิเตอร์ ($I_m = 0$) เข็มชี้อยู่ที่ตำแหน่งพัก 'ซ้ายสุด' อ่านค่า $0\;\Omega$:
+$$I_m = 0 \implies 0\;\Omega$$
+- เมื่อ $R_x = R_m$: กระแสแบ่งไหลเท่ากัน เข็มชี้เบี่ยงเบนกึ่งกลางสเกล ($0.5 I_{\text{fsd}}$)
+- เมื่อ $R_x = \infty$ (เปิดวงจร): ไม่มีกระแสแยกไหลผ่าน $R_x$ กระแสทั้งหมดไหลเข้าขดลวดมิเตอร์เต็มที่ เข็มชี้เบี่ยงเบนไป 'ขวาสุด' อ่านค่า $\infty\;\Omega$:
+$$I_m = I_{\text{fsd}} \implies \infty\;\Omega$$
+สรุป: สเกลของโอห์มมิเตอร์แบบขนานจะอ่านจาก 'ซ้ายไปขวา' ($0$ อยู่ซ้าย, $\infty$ อยู่ขวา) เหมือนกับโวลต์มิเตอร์และแอมมิเตอร์ทั่วไป
 3. การประยุกต์ใช้งาน:
-เหมาะอย่างยิ่งสำหรับการวัดค่าความต้านทานต่ำมาก (Low Resistance เช่น 0.1 โอห์ม - 50 โอห์ม) เช่น ขดลวดมอเตอร์, ขดลวดหม้อแปลง, และความต้านทานหน้าสัมผัสของสวิตช์</t>
+เหมาะอย่างยิ่งสำหรับการวัดค่าความต้านทานต่ำมาก (Low Resistance เช่น $0.01\;\Omega - 50\;\Omega$) เช่น ขดลวดมอเตอร์, ขดลวดหม้อแปลง, และความต้านทานหน้าสัมผัสของสวิตช์</t>
         </is>
       </c>
       <c r="L57" s="5" t="inlineStr">
@@ -5824,25 +5915,29 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>$$R_{\text{scale}} = \text{Reading on Dial} \times \text{Range Multiplier}$$
+          <t>$$R_{\text{measured}} = \text{Dial Reading} \times \text{Range Multiplier}$$
 $$R_{h,\text{new}} = R_h \times \text{Multiplier}$$
-$$\text{Battery Aging: } E \downarrow \implies \text{Adjust } R_{\text{zero}} \downarrow \text{ to maintain } I_{\text{fsd}} = \frac{E}{R_{\text{in}}}$$</t>
+$$\text{Battery Decline: } E \downarrow \implies \text{Decrease } R_{\text{zero}} \text{ so that } I_{\text{fsd}} = \frac{E}{R_{\text{in}}}$$</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
           <t>1. Purpose of Zero-Adjust Rheostat:
-As the internal dry cell battery ages, its open-circuit terminal voltage E drops and its internal resistance rises. The Zero-Adjust potentiometer compensates for this battery voltage decline by adjusting total internal resistance so that shorting test leads still yields exactly full-scale current Ifsd (pointer aligns perfectly to 0 ohms).
+As the internal dry cell battery ages, its open-circuit terminal voltage $E$ drops and its internal resistance rises. The Zero-Adjust potentiometer compensates for this battery decline by decreasing circuit resistance so that shorting test leads ($R_x = 0$) still yields exactly full-scale current $I_{\text{fsd}}$ (pointer aligns perfectly to $0\;\Omega$).
 2. Multi-Range Operation:
-Switching to higher ranges (e.g., Rx10, Rx1k, Rx10k) changes internal shunt/series divider resistors, multiplying the center-scale half-deflection resistance Rh by that factor. To measure 100 k-ohms accurately, use Rx10k so the pointer lands near center scale where reading precision is highest.</t>
+Switching to higher ranges (e.g., $R \times 1, R \times 10, R \times 100, R \times 1\text{k}, R \times 10\text{k}$) modifies internal shunt/series divider resistors, multiplying the center-scale half-deflection resistance $R_h$ by that factor:
+$$R_{h,\text{new}} = R_h \times \text{Multiplier}$$
+To measure $100\text{ k}\Omega$ accurately, select $R \times 10\text{k}$ so the pointer deflects near center scale ($R_h$) where reading precision is highest.</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
           <t>1. หน้าที่ของปุ่มปรับศูนย์โอห์ม (Zero-Adjust Rheostat):
-เมื่อแบตเตอรี่ภายในมัลติมิเตอร์ถูกใช้งานไปนานๆ แรงดันไฟฟ้า E จะค่อยๆ ตกและค่าความต้านทานภายในถ่านจะสูงขึ้น ปุ่ม Zero-Adjust มีไว้เพื่อปรับลดค่าความต้านทานวงจรภายในชดเชยแรงดันถ่านที่ลดลง ทำให้เมื่อนำปลายสายวัดมาช็อตกัน เข็มชี้ยังคงเบี่ยงเบนไปตรงขีด 0 โอห์มได้อย่างแม่นยำ
+เมื่อแบตเตอรี่ภายในมัลติมิเตอร์ถูกใช้งานไปนานๆ แรงดันไฟฟ้า $E$ จะค่อยๆ ลดลงและค่าความต้านทานภายในถ่านจะสูงขึ้น ปุ่ม Zero-Adjust มีไว้เพื่อปรับลดค่าความต้านทานวงจรภายในชดเชยแรงดันถ่านที่ลดลง ทำให้เมื่อนำปลายสายวัดมาช็อตกัน ($R_x = 0$) เข็มชี้ยังคงเบี่ยงเบนไปตรงขีด $0\;\Omega$ ได้อย่างแม่นยำ
 2. การทำงานของย่านวัดตัวคูณ (Multipliers):
-การเปลี่ยนสวิตช์ย่านวัด (เช่น R x 1, R x 100, R x 10k) จะสลับวงจรแบ่งแรงดันภายใน ทำให้ความต้านทานกึ่งกลางสเกล (Half-scale Rh) ขยายตามตัวคูณนั้น ผู้ใช้ควรรักษาตำแหน่งเข็มให้อยู่บริเวณกึ่งกลางหน้าปัดเสมอเพื่อความเที่ยงตรงสูงสุด</t>
+การเปลี่ยนสวิตช์ย่านวัด (เช่น $R \times 1, R \times 100, R \times 10\text{k}$) จะสลับวงจรแบ่งแรงดันภายใน ทำให้ความต้านทานกึ่งกลางสเกล (Half-scale $R_h$) ขยายตามตัวคูณนั้น:
+$$R_{h,\text{new}} = R_h \times \text{Multiplier}$$
+ผู้ใช้ควรรักษาตำแหน่งเข็มให้อยู่บริเวณกึ่งกลางหน้าปัดเสมอเพื่อความเที่ยงตรงสูงสุด</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
@@ -5881,7 +5976,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>เอซีโวลต์มิเตอร์แบบใช้วงจรเรียงกระแส (Rectifier AC Voltmeter) และฟอร์มแฟกเตอร์</t>
+          <t>เอซีโวลต์มิเตอร์แบบใช้วงจรเรียงกระแส (Rectifier AC Voltmeter) และฟอร์มแฟกเตอร์ (ข้อสอบไฟนอล 3.2)</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -5891,7 +5986,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Lecture Chapter 10 &amp; Jele Sheet</t>
+          <t>Final Exam ข้อ 3.2 (หน้า 30 - 3 คะแนน)</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -5901,39 +5996,43 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>เมื่อนำมิเตอร์ PMMC มาต่อร่วมกับวงจรบริดจ์เรกติไฟเออร์แบบเต็มคลื่น (Full-Wave Rectifier) เพื่อวัดแรงดันไฟฟ้ากระแสสลับรูปคลื่นไซน์ จงอธิบายความสัมพันธ์ระหว่างค่าเฉลี่ย DC ที่มิเตอร์ตอบสนอง กับค่า RMS ของแรงดัน AC และอธิบายว่าจะเกิดความผิดพลาดอย่างไรหากนำไปวัดคลื่นสี่เหลี่ยมหรือคลื่นสามเหลี่ยม</t>
+          <t>เมื่อนำมิเตอร์ PMMC มาต่อร่วมกับวงจรบริดจ์เรกติไฟเออร์แบบเต็มคลื่น (Full-Wave Rectifier) เพื่อวัดแรงดันไฟฟ้ากระแสสลับรูปคลื่นไซน์ จงอธิบายความสัมพันธ์ระหว่างค่าเฉลี่ย DC ที่มิเตอร์ตอบสนอง กับค่า RMS ของแรงดัน AC และอธิบายว่าจะเกิดความผิดพลาดอย่างไรหากนำไปวัดคลื่นสี่เหลี่ยมหรือคลื่นสามเหลี่ยม (ข้อสอบไฟนอลข้อ 3.2 หน้า 30)</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>$$V_{\text{avg}} = \frac{2}{\pi} V_m = 0.637\, V_m$$
-$$V_{\text{rms}} = \frac{V_m}{\sqrt{2}} = 0.707\, V_m$$
-$$\text{Form Factor } k_f = \frac{V_{\text{rms}}}{V_{\text{avg}}} = \frac{0.707}{0.637} = 1.11$$
-$$V_{\text{scale}} = 1.11 \times V_{\text{avg}}$$</t>
+          <t>$$V_{\text{avg}} = \frac{2}{\pi} V_m \approx 0.637\, V_m$$
+$$V_{\text{rms}} = \frac{V_m}{\sqrt{2}} \approx 0.707\, V_m$$
+$$\text{Form Factor } k_f = \frac{V_{\text{rms}}}{V_{\text{avg}}} = \frac{0.707\, V_m}{0.637\, V_m} = 1.11$$
+$$V_{\text{scale}} = 1.11 \times V_{\text{avg}} = V_{\text{rms}}$$</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
           <t>1. PMMC Mechanism Response:
-The PMMC movement responds strictly to average rectified current: V_avg = (2/pi) * Vm = 0.637 Vm.
-2. AC Calibration:
-Users expect the dial to indicate Effective / Root-Mean-Square (RMS) voltage. For pure sinusoidal AC, the Form Factor is:
-kf = V_rms / V_avg = 1.11
-Manufacturers calibrate the dial markings by multiplying the actual deflection by 1.11.
+The moving coil responds strictly to average rectified DC current:
+$$V_{\text{avg}} = \frac{2}{\pi} V_m \approx 0.637\, V_m$$
+2. AC Calibration (Form Factor):
+Users require the dial to display Effective / Root-Mean-Square (RMS) voltage. For pure sinusoidal AC, the Form Factor is:
+$$k_f = \frac{V_{\text{rms}}}{V_{\text{avg}}} = \frac{V_m / \sqrt{2}}{2 V_m / \pi} = \frac{\pi}{2 \sqrt{2}} \approx 1.11$$
+Manufacturers calibrate dial markings by multiplying average deflection by $1.11$:
+$$V_{\text{dial}} = 1.11 \times V_{\text{avg}} = V_{\text{rms}}$$
 3. Non-Sinusoidal Waveform Error:
-If measuring non-sinusoidal waveforms (square wave kf = 1.0, triangular wave kf = 1.155), the 1.11 calibration scale causes significant measurement error. True RMS meters (thermal or digital sampling) must be used for non-sine waves.</t>
+For a square wave, $k_f = 1.00$. Measuring a $10\text{ V}$ peak square wave causes the meter to read $1.11 \times 10 = 11.1\text{ V}$ (an error of $+11\%$)! For non-sinusoidal waveforms, True-RMS meters must be utilized.</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
           <t>1. การตอบสนองของ PMMC:
-ขดลวดเคลื่อนที่ PMMC ตอบสนองต่อ 'ค่าเฉลี่ย (Average DC)' หลังผ่านการเรียงกระแส: V_avg = (2/pi)*Vm = 0.637 Vm
+ขดลวดเคลื่อนที่ PMMC ตอบสนองต่อ 'ค่าเฉลี่ย (Average DC)' หลังผ่านการเรียงกระแส:
+$$V_{\text{avg}} = \frac{2}{\pi} V_m \approx 0.637\, V_m$$
 2. การปรับเทียบสเกลหน้าปัด (AC Calibration):
-ผู้ใช้งานต้องการอ่านค่าแรงดันใช้งานจริง หรือค่ายังผล (RMS) หน้าปัดจึงถูกสเกลค่าล่วงหน้าโดยคูณด้วย 'ฟอร์มแฟกเตอร์ (Form Factor: kf)':
-kf = V_rms / V_avg = (Vm / sqrt(2)) / (2*Vm / pi) = 1.11
-ดังนั้น สเกล AC จึงถูกตั้งไว้ที่ 1.11 เท่าของค่าเฉลี่ย
+ผู้ใช้งานต้องการอ่านค่าแรงดันยังผล หรือค่ายังผล (RMS) หน้าปัดจึงถูกปรับสเกลล่วงหน้าโดยคูณด้วย 'ฟอร์มแฟกเตอร์ (Form Factor: $k_f$)':
+$$k_f = \frac{V_{\text{rms}}}{V_{\text{avg}}} = \frac{V_m / \sqrt{2}}{2 V_m / \pi} = \frac{\pi}{2 \sqrt{2}} \approx 1.11$$
+ดังนั้น สเกล AC จึงถูกตั้งค่าให้อ่านเป็น $1.11$ เท่าของค่าเฉลี่ย:
+$$V_{\text{dial}} = 1.11 \times V_{\text{avg}} = V_{\text{rms}}$$
 3. ข้อผิดพลาดเมื่อวัดรูปคลื่นอื่นที่ไม่ใช่ไซน์:
-หากนำไปวัดรูปคลื่นสี่เหลี่ยม (Square Wave ซึ่งมี kf = 1.00) มิเตอร์จะอ่านค่าสูงเกินจริง 11% หากต้องการวัดสัญญาณรูปคลื่นใดๆ ให้แม่นยำ ต้องใช้มิเตอร์ประเภท 'True RMS'</t>
+สำหรับคลื่นสี่เหลี่ยม (Square Wave) มีค่า $k_f = 1.00$ หากนำมิเตอร์นี้ไปวัดไฟคลื่นสี่เหลี่ยม $10\text{ V}$ มิเตอร์จะคูณ $1.11$ และอ่านได้ $11.1\text{ V}$ (ผิดพลาดสูงเกินจริง $+11\%$) หากต้องการวัดสัญญาณรูปคลื่นใดๆ ให้แม่นยำ ต้องใช้มิเตอร์ประเภท 'True RMS'</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -5992,36 +6091,39 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>จงอธิบายโครงสร้างของวัตต์มิเตอร์แบบอิเล็กโทรไดนาโมมิเตอร์ (Electrodynamometer Wattmeter) ขดลวดกระแส (Current Coil: CC) และขดลวดแรงดัน (Potential Coil: PC) ต้องต่อเข้ากับโหลดอย่างไร และมีข้อควรระวังใดในการป้องกันขดลวดไหม้?</t>
+          <t>จงอธิบายโครงสร้างของวัตต์มิเตอร์แบบอิเล็กโทรไดนาโมมิเตอร์ (Electrodynamometer Wattmeter) ขดลวดกระแส (Current Coil: CC) และขดลวดแรงดัน (Potential Coil: PC) ต้องต่อเข้ากับโหลดอย่างไร และมีข้อควรระวังใดในการป้องกันขดลวดไหม้? (ข้อสอบไฟนอลข้อ 3.4 หน้า 30)</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
           <t>$$P = V_{\text{load}} \cdot I_{\text{load}} \cdot \cos\theta$$
-$$\text{Current Coil (CC): Fixed, thick wire, low turns } \implies \text{Connected in SERIES with load}$$
-$$\text{Potential Coil (PC): Moving, fine wire, high turns } \implies \text{Connected in PARALLEL across load}$$</t>
+$$\text{Current Coil (CC): Fixed, thick wire, low turns } \implies \text{Connected in SERIES with load (Terminals 1--2)}$$
+$$\text{Potential Coil (PC): Moving, fine wire, high turns } \implies \text{Connected in PARALLEL across load (Terminals 3--5)}$$
+$$\text{Burnout Hazard: Connecting CC in parallel creates a dead short circuit } I_{\text{sc}} = \frac{V}{R_{\text{CC}}} \approx \infty$$</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
           <t>1. Wattmeter Coils &amp; Connection:
-- Current Coil (CC / ขดลวดกระแส): Made of thick copper wire with few turns (near-zero impedance). MUST be connected in SERIES with the load to carry full line current.
-- Potential Coil (PC / ขดลวดแรงดัน): Made of thin wire with many turns, connected in series with a high multiplier resistance. MUST be connected in PARALLEL across the load terminals to measure line voltage.
+- Current Coil (CC / ขดลวดกระแส): Made of thick copper wire with few turns (near-zero impedance). MUST be connected in SERIES with the load (terminals 1-2) to carry full line current.
+- Potential Coil (PC / ขดลวดแรงดัน): Made of fine wire with many turns, connected in series with a high non-inductive multiplier resistance. MUST be connected in PARALLEL across the load terminals (terminals 3-5) to measure voltage.
 2. Power Indication:
-Instantaneous torque is proportional to the product i_cc * i_pc, so average pointer deflection indicates real average active power: P = V * I * cos(theta).
+Instantaneous torque is proportional to the product of magnetic fields produced by both coils: $T_d \propto i_{\text{cc}}(t) \cdot i_{\text{pc}}(t)$, deflecting the pointer to indicate true real average active power:
+$$P = V_{\text{load}} \cdot I_{\text{load}} \cdot \cos\theta$$
 3. Burnout Hazard:
-NEVER connect the Current Coil in parallel across the voltage supply! Because CC has near-zero resistance, connecting it in parallel creates a dead short circuit, drawing hundreds of amps and instantly vaporizing the coil.</t>
+NEVER connect the Current Coil (CC) in parallel across the voltage supply! Because CC has near-zero resistance, connecting it in parallel creates an immediate dead short circuit ($I_{\text{sc}} = V / R_{\text{CC}} \approx \infty$), vaporizing the coil instantly.</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
           <t>1. โครงสร้างและการต่อใช้งาน:
-- ขดลวดกระแส (Current Coil: CC): เป็นขดลวดลวดทองแดงเส้นใหญ่ จำนวนรอบน้อย (ความต้านทานต่ำมากใกล้ศูนย์) ต้องต่อ 'อนุกรม' กับโหลด เพื่อให้กระแสโหลดทั้งหมดไหลผ่าน
-- ขดลวดแรงดัน (Potential Coil: PC): เป็นขดลวดเส้นเล็ก จำนวนรอบมาก ต่ออนุกรมกับตัวต้านทานค่าสูง ต้องต่อ 'ขนาน' คร่อมโหลด เพื่อวัดแรงดันตกคร่อมโหลด
+- ขดลวดกระแส (Current Coil: CC): เป็นขดลวดลวดทองแดงเส้นใหญ่ จำนวนรอบน้อย (ความต้านทานต่ำมากใกล้ศูนย์) ต้องต่อ 'อนุกรม' กับโหลด (ขั้ว 1-2) เพื่อให้กระแสโหลดทั้งหมดไหลผ่าน
+- ขดลวดแรงดัน (Potential Coil: PC): เป็นขดลวดเส้นเล็ก จำนวนรอบมาก ต่ออนุกรมกับตัวต้านทานค่าสูง ต้องต่อ 'ขนาน' คร่อมโหลด (ขั้ว 3-5) เพื่อวัดแรงดันตกคร่อมโหลด
 2. การแสดงค่ากำลังไฟฟ้า:
-แรงบิดของเข็มชี้จะแปรผันตามผลคูณของสนามแม่เหล็กจากทั้งสองขดลวด ทำให้เข็มชี้แสดงค่ากำลังไฟฟ้าจริงเฉลี่ย: P = V * I * cos(theta)
+แรงบิดของเข็มชี้จะแปรผันตามผลคูณของสนามแม่เหล็กจากทั้งสองขดลวด ทำให้เข็มชี้แสดงค่ากำลังไฟฟ้าจริงเฉลี่ย:
+$$P = V_{\text{load}} \cdot I_{\text{load}} \cdot \cos\theta$$
 3. ข้อควรระวังอันตรายขดลวดไหม้:
-ห้ามนำขดลวดกระแส (CC) ไปต่อขนานคร่อมแหล่งจ่ายไฟเด็ดขาด! เพราะ CC มีความต้านทานต่ำมาก หากต่อขนานจะเกิดการลัดวงจรโดยตรง ทำให้ขดลวดไหม้ละลายทันที</t>
+ห้ามนำขดลวดกระแส (CC) ไปต่อขนานคร่อมแหล่งจ่ายไฟเด็ดขาด! เพราะ CC มีความต้านทานต่ำมาก หากต่อขนานจะเกิดการลัดวงจรโดยตรง ($I_{\text{sc}} \approx \infty$) ทำให้ขดลวดไหม้ละลายทันที</t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
@@ -6078,7 +6180,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Final Exam ข้อ 3.1 (หน้า 30 - 2 คะแนน)</t>
+          <t>Final Exam ข้อ 3.3 (หน้า 30 - 2 คะแนน)</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -6088,7 +6190,7 @@
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>จงอธิบายหลักการทำงานของมาตรวัดพลังงานไฟฟ้าแบบเหนี่ยวนำ (Induction Kilowatt-Hour Meter จานหมุน) อะไรเป็นตัวสร้างแรงบิดขับจานอะลูมิเนียม และแม่เหล็กถาวรหน่วงการหมุน (Braking Magnet) มีหน้าที่อะไร?</t>
+          <t>จงอธิบายหลักการทำงานของมาตรวัดพลังงานไฟฟ้าแบบเหนี่ยวนำ (Induction Kilowatt-Hour Meter จานหมุน) อะไรเป็นตัวสร้างแรงบิดขับจานอะลูมิเนียม และแม่เหล็กถาวรหน่วงการหมุน (Braking Magnet) มีหน้าที่อะไร? (ข้อสอบไฟนอลข้อ 3.3 หน้า 30)</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -6102,21 +6204,30 @@
       <c r="J61" s="5" t="inlineStr">
         <is>
           <t>1. Driving Torque Generation:
-The meter contains a shunt electromagnet (connected across line voltage) and a series electromagnet (carrying load current). Their alternating fluxes induce eddy currents inside a lightweight aluminum disc. The interaction between each eddy current and the other magnet's flux creates a continuous rotational driving torque Td proportional to instantaneous real power P.
+The meter contains a shunt electromagnet (connected across line voltage) and a series electromagnet (carrying load current). Their alternating magnetic fluxes induce eddy currents inside a lightweight aluminum disc. The interaction between each eddy current and the alternating flux produces a continuous rotational driving torque $T_d$ proportional to instantaneous real power $P$:
+$$T_d \propto V \cdot I \cdot \cos\theta = P$$
 2. Braking Magnet Role:
-A C-shaped permanent magnet sits near the edge of the disc. As the disc spins through its field, eddy currents are induced that create a retarding torque Tb proportional to rotational speed (Tb proportional to omega).
+A C-shaped permanent magnet sits near the outer edge of the disc. As the disc spins through this stationary field, eddy currents are induced in the disc, creating a retarding braking torque $T_b$ directly proportional to rotational speed $\omega$:
+$$T_b \propto \omega$$
 3. Energy Integration:
-Equating Td = Tb yields disc speed omega proportional to power P. Therefore, the total number of disc revolutions over time is directly proportional to cumulative electrical energy: Energy = Integral(P dt) in kWh, registered on gear dials.</t>
+Equating driving and braking torque ($T_d = T_b$) yields:
+$$\omega \propto P$$
+The total number of disc revolutions $N$ over time is directly proportional to cumulative electrical energy in kilowatt-hours (kWh):
+$$N = \int \omega\, dt \propto \int P\, dt = \text{Energy (kWh)}$$</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
           <t>1. การสร้างแรงบิดขับหมุนจานอะลูมิเนียม:
-มาตรวัดประกอบด้วยแม่เหล็กไฟฟ้าขดลวดแรงดัน (Shunt Magnet) และแม่เหล็กไฟฟ้าขดลวดกระแส (Series Magnet) ฟลักซ์แม่เหล็กสลับจากทั้งสองขดลวดจะเหนี่ยวนำให้เกิดกระแสไหลวน (Eddy Currents) บนจานอะลูมิเนียม ปฏิกิริยาระหว่างกระแสไหลวนและฟลักซ์แม่เหล็กทำให้เกิดแรงผลักเป็นแรงบิดหมุนขับ (Driving Torque: Td) ซึ่งแปรผันตรงกับกำลังไฟฟ้าจริง P
+มาตรวัดประกอบด้วยแม่เหล็กไฟฟ้าขดลวดแรงดัน (Shunt Magnet) และแม่เหล็กไฟฟ้าขดลวดกระแส (Series Magnet) ฟลักซ์แม่เหล็กสลับจากทั้งสองขดลวดจะเหนี่ยวนำให้เกิดกระแสไหลวน (Eddy Currents) บนจานอะลูมิเนียม ปฏิกิริยาระหว่างกระแสไหลวนและฟลักซ์แม่เหล็กทำให้เกิดแรงผลักเป็นแรงบิดหมุนขับ ($T_d$) ซึ่งแปรผันตรงกับกำลังไฟฟ้าจริง $P$:
+$$T_d \propto V \cdot I \cdot \cos\theta = P$$
 2. หน้าที่ของแม่เหล็กเบรก (Braking Magnet):
-แม่เหล็กถาวรรูปเกือกม้าที่ติดตั้งคร่อมขอบจาน จะสร้างแรงบิดหน่วง (Braking Torque: Tb) ที่แปรผันตรงกับความเร็วรอบการหมุน (omega) โดยอาศัยหลักการของ Eddy Current Braking
+แม่เหล็กถาวรรูปเกือกม้าที่ติดตั้งคร่อมขอบจาน จะสร้างแรงบิดหน่วง ($T_b$) ที่แปรผันตรงกับความเร็วรอบการหมุน ($\omega$) โดยอาศัยหลักการของ Eddy Current Braking:
+$$T_b \propto \omega$$
 3. การรวมหน่วยพลังงานไฟฟ้า (kWh):
-เมื่อแรงบิดขับสมดุลกับแรงบิดเบรก (Td = Tb) ความเร็วรอบจานหมุนจะแปรผันตรงกับกำลังไฟฟ้า P ทำให้จำนวนรอบการหมุนทั้งหมดของจานแปรผันตรงกับพลังงานไฟฟ้ารวม: Energy = Integral(P dt) ซึ่งจะส่งผ่านชุดเฟืองไปหมุนตัวเลขหน้าปัดบอกค่าเป็น กิโลวัตต์-ชั่วโมง (kWh)</t>
+เมื่อแรงบิดขับสมดุลกับแรงบิดเบรก ($T_d = T_b$) ความเร็วรอบจานหมุนจะแปรผันตรงกับกำลังไฟฟ้า $P$ ทำให้จำนวนรอบการหมุนทั้งหมดของจานแปรผันตรงกับพลังงานไฟฟ้ารวม:
+$$N = \int \omega\, dt \propto \int P\, dt = \text{Energy (kWh)}$$
+ซึ่งส่งผ่านชุดเฟืองไปหมุนตัวเลขหน้าปัดบอกค่าเป็น กิโลวัตต์-ชั่วโมง (kWh)</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -6183,33 +6294,41 @@
           <t>$$\text{Absolute Error: } e = Y_n - X_n$$
 $$\text{Relative Error: } e_r = \frac{Y_n - X_n}{X_n}$$
 $$\%\text{ Error} = \frac{|Y_n - X_n|}{X_n} \times 100\%$$
-$$\%\text{ Accuracy } A = 100\% - \%\text{ Error}$$</t>
+$$\%\text{ Accuracy } A = 100\% - \%\text{ Error} = \left(1 - \frac{|Y_n - X_n|}{X_n}\right) \times 100\%$$</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
           <t>1. Accuracy (ความแม่นยำ/ความถูกต้อง):
-How close the measured value Yn is to the true accepted standard value Xn.
+How close the measured reading $Y_n$ is to the true, accepted standard value $X_n$.
 2. Precision (ความเที่ยงตรง):
-The repeatability or consistency of successive measurements of the exact same quantity under identical conditions, regardless of whether it is near the true value.
-3. Error Formulas:
-- Absolute Error: e = Yn - Xn (Measured value minus True value)
-- Relative Error: e_r = (Yn - Xn) / Xn
-- % Error: (% Error) = (|Yn - Xn| / Xn) * 100%
-- % Accuracy: A = 100% - % Error = [1 - |Yn - Xn| / Xn] * 100%.</t>
+The repeatability or consistency of successive measurements of the exact same physical quantity under identical conditions, regardless of whether it is near the true value.
+3. Error &amp; Accuracy Formulas:
+- Absolute Error:
+$$e = Y_n - X_n$$
+- Relative Error:
+$$e_r = \frac{Y_n - X_n}{X_n}$$
+- Percentage Error:
+$$\%\text{ Error} = \frac{|Y_n - X_n|}{X_n} \times 100\%$$
+- Percentage Accuracy ($A$):
+$$A = 100\% - \%\text{ Error} = \left(1 - \frac{|Y_n - X_n|}{X_n}\right) \times 100\%$$</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
           <t>1. ความถูกต้อง (Accuracy):
-ระดับความใกล้เคียงของค่าที่วัดได้ (Measured Value Yn) กับค่าจริงที่แท้จริง (True Value Xn)
+ระดับความใกล้เคียงของค่าที่วัดได้ ($Y_n$) กับค่าจริงที่แท้จริง ($X_n$)
 2. ความเที่ยงตรง (Precision):
-ความสามารถในการวัดซ้ำแล้วได้ค่าเดิมสม่ำเสมอ (Repeatability/Consistency) ของปริมาณเดิมภายใต้สภาวะเดียวกัน แม้ค่านั้นอาจจะไม่ตรงกับค่าจริงก็ตาม
+ความสามารถในการวัดซ้ำแล้วได้ค่าเดิมสม่ำเสมอ (Repeatability / Consistency) ของปริมาณเดิมภายใต้สภาวะเดียวกัน แม้ค่านั้นอาจจะไม่ตรงกับค่าจริงก็ตาม
 3. สูตรการคำนวณความผิดพลาด:
-- ค่าความผิดพลาดสัมบูรณ์: e = Yn - Xn (ค่าที่วัดได้ ลบ ค่าจริง)
-- ค่าความผิดพลาดสัมพัทธ์: e_r = (Yn - Xn) / Xn
-- เปอร์เซ็นต์ความผิดพลาด: % Error = (|Yn - Xn| / Xn) * 100%
-- เปอร์เซ็นต์ความถูกต้อง: % Accuracy = 100% - % Error</t>
+- ค่าความผิดพลาดสัมบูรณ์:
+$$e = Y_n - X_n$$
+- ค่าความผิดพลาดสัมพัทธ์:
+$$e_r = \frac{Y_n - X_n}{X_n}$$
+- เปอร์เซ็นต์ความผิดพลาด:
+$$\%\text{ Error} = \frac{|Y_n - X_n|}{X_n} \times 100\%$$
+- เปอร์เซ็นต์ความถูกต้อง ($A$):
+$$A = 100\% - \%\text{ Error} = \left(1 - \frac{|Y_n - X_n|}{X_n}\right) \times 100\%$$</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
@@ -6248,7 +6367,7 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>สารกึ่งตัวนำบริสุทธิ์ vs สารเจือปน, ชนิด N-Type และ P-Type</t>
+          <t>สารกึ่งตัวนำบริสุทธิ์ vs สารเจือปน, ชนิด N-Type และ P-Type (ข้อสอบไฟนอล 4.1)</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
@@ -6268,7 +6387,7 @@
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>จงอธิบายความแตกต่างระหว่างสารกึ่งตัวนำบริสุทธิ์ (Intrinsic) และสารกึ่งตัวนำไม่บริสุทธิ์ (Extrinsic) อธิบายกระบวนการโดปสารชนิด N-Type และ P-Type พร้อมระบุพาหะข้างมาก (Majority Carrier) และพาหะข้างน้อย (Minority Carrier) ของแต่ละชนิด</t>
+          <t>จงอธิบายความแตกต่างระหว่างสารกึ่งตัวนำบริสุทธิ์ (Intrinsic) และสารกึ่งตัวนำไม่บริสุทธิ์ (Extrinsic) อธิบายกระบวนการโดปสารชนิด N-Type และ P-Type พร้อมระบุพาหะข้างมาก (Majority Carrier) และพาหะข้างน้อย (Minority Carrier) ของแต่ละชนิด (ข้อสอบไฟนอลข้อ 4.1 หน้า 24)</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
@@ -6281,33 +6400,37 @@
       <c r="J63" s="5" t="inlineStr">
         <is>
           <t>1. Intrinsic vs Extrinsic Semiconductors:
-- Intrinsic: Extremely pure semiconductor crystal (Silicon or Germanium, valence = 4) with no impurities. Electrical conductivity at room temperature is very low.
-- Extrinsic: Doped with tiny amounts of impurity atoms to dramatically increase electrical conductivity.
+- Intrinsic: Pure semiconductor crystal (Silicon, valence = 4) with no impurities. Low conductivity at room temperature.
+- Extrinsic: Doped with tiny concentrations of impurity atoms to dramatically increase conductivity.
 2. N-Type Semiconductor:
-- Doped with Pentavalent impurity (valence 5: Phosphorus, Arsenic, Antimony).
-- 4 valence electrons form covalent bonds with Silicon, while the 5th electron becomes a free conduction electron.
-- Majority Carriers: Free Electrons (e-); Minority Carriers: Holes (h+).
+- Doped with Pentavalent impurities (valence 5: Phosphorus, Arsenic, Antimony).
+- 4 valence electrons bond with Silicon; the 5th electron becomes a free conduction electron.
+- Majority Carriers: Free Electrons ($e^-$); Minority Carriers: Holes ($h^+$).
 3. P-Type Semiconductor:
-- Doped with Trivalent impurity (valence 3: Boron, Gallium, Indium).
-- 3 valence electrons bond with Silicon, leaving a vacancy or 'hole' that eagerly accepts an electron.
-- Majority Carriers: Holes (h+); Minority Carriers: Electrons (e-).</t>
+- Doped with Trivalent impurities (valence 3: Boron, Gallium, Indium).
+- 3 valence electrons bond with Silicon, leaving a vacancy or 'hole' ($h^+$).
+- Majority Carriers: Holes ($h^+$); Minority Carriers: Electrons ($e^-$).
+4. Mass Action Law:
+$$n \cdot p = n_i^2$$</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
           <t>1. สารกึ่งตัวนำ Intrinsic vs Extrinsic:
-- สารบริสุทธิ์ (Intrinsic Semiconductor): ผลึกซิลิคอน (Si) หรือเจอร์เมเนียม (Ge) บริสุทธิ์ มีเวเลนซ์อิเล็กตรอน 4 ตัว นำไฟฟ้าได้ต่ำมากที่อุณหภูมิห้อง
-- สารเจือปน (Extrinsic Semiconductor): สารกึ่งตัวนำที่ผ่านการโดป (Doping) เติมสารเจือปนเพื่อเพิ่มการนำไฟฟ้าอย่างมหาศาล
+- สารบริสุทธิ์ (Intrinsic): ผลึกซิลิคอน (Si) บริสุทธิ์ มีเวเลนซ์อิเล็กตรอน 4 ตัว นำไฟฟ้าได้ต่ำมากที่อุณหภูมิห้อง
+- สารเจือปน (Extrinsic): สารที่ผ่านการโดป (Doping) เติมสารเจือปนเพื่อเพิ่มการนำไฟฟ้าอย่างมหาศาล
 2. สารกึ่งตัวนำชนิด N (N-Type):
 - โดปด้วยสารเจือปนที่มีเวเลนซ์ 5 (Pentavalent เช่น ฟอสฟอรัส P, สารหนู As)
 - อิเล็กตรอน 4 ตัวจับคู่กับ Si เหลืออิเล็กตรอนตัวที่ 5 หลุดเป็นอิสระ
-- พาหะข้างมาก (Majority Carrier): อิเล็กตรอนอิสระ (Electrons)
-- พาหะข้างน้อย (Minority Carrier): โฮล (Holes)
+- พาหะข้างมาก (Majority Carrier): อิเล็กตรอนอิสระ ($e^-$)
+- พาหะข้างน้อย (Minority Carrier): โฮล ($h^+$)
 3. สารกึ่งตัวนำชนิด P (P-Type):
 - โดปด้วยสารเจือปนที่มีเวเลนซ์ 3 (Trivalent เช่น โบรอน B, แกลเลียม Ga)
-- อิเล็กตรอน 3 ตัวจับคู่กับ Si ทำให้ขาดอิเล็กตรอนไป 1 ตำแหน่ง เกิดเป็น 'โฮล (Hole)' หรือที่ว่าง
-- พาหะข้างมาก (Majority Carrier): โฮล (Holes)
-- พาหะข้างน้อย (Minority Carrier): อิเล็กตรอน (Electrons)</t>
+- อิเล็กตรอน 3 ตัวจับคู่กับ Si ขาดไป 1 ตำแหน่ง เกิดเป็น 'โฮล ($h^+$)'
+- พาหะข้างมาก (Majority Carrier): โฮล ($h^+$)
+- พาหะข้างน้อย (Minority Carrier): อิเล็กตรอน ($e^-$)
+4. กฎสมดุลพาหะ (Mass Action Law):
+$$n \cdot p = n_i^2$$</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
@@ -6354,7 +6477,7 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>มอสเฟต (MOSFET) นิยาม โครงสร้าง คุณสมบัติเด่น และการประยุกต์ใช้งาน</t>
+          <t>มอสเฟต (MOSFET) นิยาม โครงสร้าง คุณสมบัติเด่น และการประยุกต์ใช้งาน (ข้อสอบไฟนอล 4.2)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -6374,7 +6497,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>MOSFET ย่อมาจากอะไร? จงอธิบายโครงสร้าง 3 ขาหลัก อธิบายเหตุผลที่ขาเกต (Gate) มีอินพุตอิมพีแดนซ์สูงมากเกือบเป็นอนันต์ และระบุข้อดีที่เหนือกว่าทรานซิสเตอร์แบบ BJT</t>
+          <t>MOSFET ย่อมาจากอะไร? จงอธิบายโครงสร้าง 3 ขาหลัก อธิบายเหตุผลที่ขาเกต (Gate) มีอินพุตอิมพีแดนซ์สูงมากเกือบเป็นอนันต์ และระบุข้อดีที่เหนือกว่าทรานซิสเตอร์แบบ BJT (ข้อสอบไฟนอลข้อ 4.2 หน้า 24)</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -6388,25 +6511,27 @@
       <c r="J64" s="3" t="inlineStr">
         <is>
           <t>1. Definition &amp; Terminals:
-MOSFET stands for Metal-Oxide-Semiconductor Field-Effect Transistor. Its 3 functional terminals are Gate (G), Drain (D), and Source (S) (with a substrate/body terminal internally tied to Source).
+MOSFET stands for Metal-Oxide-Semiconductor Field-Effect Transistor. Its 3 active terminals are Gate (G), Drain (D), and Source (S).
 2. Near-Infinite Gate Input Impedance:
-The Gate electrode is physically isolated from the semiconductor conducting channel by an ultra-thin dielectric layer of Silicon Dioxide (SiO2). Because SiO2 is an exceptional electrical insulator, steady-state gate current IG is practically ZERO (nanoamperes to picoamperes), giving an input impedance of 10^12 to 10^14 ohms.
-3. Advantages over BJT:
-- Voltage-controlled (requires zero static gate current to remain ON, unlike BJT which demands continuous base current IB).
-- Extremely fast switching speeds (ideal for high-frequency switch-mode power supplies and CPU logic gates).
-- Low conduction resistance RDS(on) in modern power MOSFETs, yielding high efficiency.</t>
+The Gate electrode is physically isolated from the conducting channel by an ultra-thin dielectric layer of Silicon Dioxide ($SiO_2$). Because $SiO_2$ is an outstanding electrical insulator, static gate current is practically zero:
+$$I_G \approx 0 \implies R_{\text{in, gate}} \approx 10^{12} - 10^{14}\;\Omega$$
+3. Key Advantages Over BJT:
+- Voltage-Controlled: Requires zero continuous gate current to stay ON, unlike BJT which demands base current $I_B$.
+- High Switching Speed: Fast transition times ideal for high-frequency switch-mode power supplies and CPU logic gates.
+- Positive Thermal Coefficient: Prevents thermal runaway and allows straightforward parallel connection.</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
           <t>1. นิยามและขาใช้งาน:
 MOSFET ย่อมาจาก 'Metal-Oxide-Semiconductor Field-Effect Transistor' มี 3 ขาหลักคือ ขาเกต Gate (G), ขาเดรน Drain (D) และขาซอร์ส Source (S)
-2. เหตุผลที่ขาเกตมีอิมพีแดนซ์สูงมาก (R_in เกือบอนันต์):
-เพราะขาเกตถูกคั่นแยกจากช่องนำกระแสด้วยชั้นฉนวนบางของ 'ซิลิคอนไดออกไซด์ (Silicon Dioxide: SiO2)' ซึ่งเป็นฉนวนไฟฟ้าชั้นยอด ทำให้ไม่มีกระแสไฟตรงไหลเข้าขาเกตเลย (IG = 0) อิมพีแดนซ์ขาเข้าจึงสูงถึง 10^12 - 10^14 โอห์ม
+2. เหตุผลที่ขาเกตมีอิมพีแดนซ์สูงมาก ($R_{\text{in}}$ เกือบอนันต์):
+เพราะขาเกตถูกคั่นแยกจากช่องนำกระแสด้วยชั้นฉนวนบางของ 'ซิลิคอนไดออกไซด์ ($SiO_2$)' ซึ่งเป็นฉนวนไฟฟ้าชั้นยอด ทำให้ไม่มีกระแสไฟตรงไหลเข้าขาเกตเลย:
+$$I_G \approx 0 \implies R_{\text{in, gate}} \approx 10^{12} - 10^{14}\;\Omega$$
 3. ข้อดีเด่นชัดเหนือกว่าทรานซิสเตอร์ BJT:
-- ควบคุมด้วยแรงดัน (Voltage-Controlled): ไม่กินกระแสขับขาเข้า ต่างจาก BJT ที่ต้องจ่ายกระแสไบแอสที่ขาเบส IB ตลอดเวลา
+- ควบคุมด้วยแรงดัน (Voltage-Controlled): ไม่กินกระแสขับขาเข้า ต่างจาก BJT ที่ต้องจ่ายกระแสไบแอสที่ขาเบส $I_B$ ตลอดเวลา
 - ความเร็วในการสวิตชิ่งสูงมาก (Fast Switching): เหมาะสำหรับสวิตชิ่งความถี่สูงในวงจรดิจิทัลและสวิตชิ่งเพาเวอร์ซัพพลาย
-- ประสิทธิภาพสูง: กินพลังงานขับต่ำมาก ทำให้ไม่ร้อนและนำไปสร้างเป็นไมโครโปรเซสเซอร์ที่มีทรานซิสเตอร์นับพันล้านตัวได้</t>
+- สัมประสิทธิ์อุณหภูมิเป็นบวก: ไม่เกิดปัญหาความร้อนทำลายตัวเอง (No Thermal Runaway) และต่อขนานได้ง่าย</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
@@ -6453,7 +6578,7 @@
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>วงจรรวม (Integrated Circuit: IC) นิยาม ความสำคัญ และวิวัฒนาการ</t>
+          <t>วงจรรวม (Integrated Circuit: IC) นิยาม ความสำคัญ และวิวัฒนาการ (ข้อสอบไฟนอล 4.3)</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
@@ -6473,7 +6598,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>วงจรรวม (Integrated Circuit: IC) คืออะไร? ถูกผลิตขึ้นบนแผ่นเวเฟอร์สารกึ่งตัวนำอย่างไร และให้ประโยชน์ที่พลิกโฉมวงการเหนือวงจรที่ประกอบด้วยชิ้นส่วนแยกชิ้น (Discrete Components) อย่างไร?</t>
+          <t>วงจรรวม (Integrated Circuit: IC) คืออะไร? ถูกผลิตขึ้นบนแผ่นเวเฟอร์สารกึ่งตัวนำอย่างไร และให้ประโยชน์ที่พลิกโฉมวงการเหนือวงจรที่ประกอบด้วยชิ้นส่วนแยกชิ้น (Discrete Components) อย่างไร? (ข้อสอบไฟนอลข้อ 4.3 หน้า 24)</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -6484,34 +6609,36 @@
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>1. Definition of an IC:
-An Integrated Circuit (IC or microchip) is a complete electronic circuit consisting of millions or billions of interconnected microscopic components (transistors, diodes, resistors, capacitors) fabricated monolithically on a single tiny crystal semiconductor substrate (usually Silicon).
+          <t>1. Definition of an Integrated Circuit (IC):
+An Integrated Circuit (IC or microchip) is a complete electronic circuit consisting of millions to billions ($&gt; 10^9$) of interconnected microscopic components (transistors, diodes, resistors, capacitors) fabricated monolithically on a single tiny semiconductor die (Silicon wafer):
+$$\text{Microscopic Integration: } \text{Transistors } (&gt; 10^9) + \text{Interconnects on single } \text{Si die}$$
 2. Revolutionary Advantages over Discrete Circuits:
-- Extreme Miniaturization: Packs complex computers into a fingernail-sized silicon chip.
-- Mass Production &amp; Low Cost: Fabricated simultaneously in huge batches on silicon wafers using photolithography, drastically lowering cost per gate.
-- High Reliability: Monolithic internal metal interconnections eliminate thousands of fragile soldered joints and mechanical wiring failures.
-- High Speed &amp; Low Power: Nanometer-scale distances between transistors allow gigahertz switching speeds with negligible parasitic capacitance and minimal power dissipation.</t>
+- Extreme Miniaturization: Shrinks entire computers onto a thumbnail-sized die ($&lt; 1\text{ cm}^2$).
+- Low Unit Cost: Mass-produced simultaneously by the thousands on silicon wafers using optical photolithography.
+- High Reliability: Monolithic metal layers replace thousands of fragile soldered wire joints.
+- High Speed &amp; Low Power: Nanometer trace distances allow gigahertz clock rates with negligible parasitic delays ($R C \rightarrow 0$).</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
           <t>1. นิยามของวงจรรวม (IC):
-วงจรรวม (Integrated Circuit หรือ Microchip) คือการรวมวงจรอิเล็กทรอนิกส์ทั้งหมด ซึ่งประกอบด้วยทรานซิสเตอร์, ไดโอด, ตัวต้านทาน และตัวเก็บประจุ ขนาดไมโครเมตร/นาโนเมตรนับล้านถึงหมื่นล้านตัว สร้างขึ้นพร้อมกันบนผลึกสารกึ่งตัวนำซิลิคอนแผ่นเดียว (Silicon Chip)
-2. ประโยชน์ที่เหนือกว่าวงจรแยกชิ้น (Discrete Circuits):
-- ขนาดเล็กกะทัดรัดอย่างยิ่ง: ย่อคอมพิวเตอร์ทั้งระบบลงบนชิปขนาดเท่าปลายนิ้ว
-- ต้นทุนต่ำ ผลิตได้จำนวนมาก: ผลิตด้วยกระบวนการโฟโตลิโทกราฟี (Photolithography) บนเวเฟอร์ทีละหลายพันชิ้นพร้อมกัน
-- ความน่าเชื่อถือสูงมาก: วงจรเชื่อมต่อกันระดับโมเลกุลภายในชิป ไม่มีจุดบัดกรีภายนอกที่อาจหลุดหลวมหรือขึ้นสนิม
-- ความเร็วสูงและกินไฟต่ำ: ระยะห่างระหว่างทรานซิสเตอร์สั้นมากระดับนาโนเมตร ทำให้ส่งสัญญาณได้เร็วในระดับกิกะเฮิรตซ์ (GHz) โดยสูญเสียพลังงานน้อยมาก</t>
+วงจรรวม (Integrated Circuit หรือ Microchip) คือการรวมวงจรอิเล็กทรอนิกส์ทั้งหมด ซึ่งประกอบด้วยทรานซิสเตอร์, ไดโอด, ตัวต้านทาน และตัวเก็บประจุจำนวนหลายล้านถึงหลายพันล้านตัว ($&gt; 10^9$ ตัว) สร้างขึ้นพร้อมกันบนแผ่นผลึกซิลิคอนชิ้นเดียว (Monolithic Silicon Substrate):
+$$\text{วงจรรวม: ทรานซิสเตอร์ } (&gt; 10^9\text{ ตัว}) + \text{สายเชื่อมต่อบนชิปซิลิคอนขนาดจิ๋ว}$$
+2. ประโยชน์ที่เหนือกว่าวงจรแบบแยกชิ้น (Discrete Components):
+- ขนาดเล็กมาก (Miniaturization): ย่อคอมพิวเตอร์ทั้งเครื่องลงบนชิปขนาดเท่าปลายนิ้ว ($&lt; 1\text{ cm}^2$)
+- ต้นทุนต่ำมากในการผลิตจำนวนมาก: ผลิตได้ครั้งละหลายพันชิ้นพร้อมกันบนเวเฟอร์ด้วยเทคโนโลยีโฟโทลิโทกราฟี (Photolithography)
+- ความน่าเชื่อถือสูงมาก: ลดจุดบัดกรีต่อสายภายนอกที่อาจหลุดหลวม
+- ความเร็วสูงและกินไฟต่ำ: ระยะทางระหว่างทรานซิสเตอร์สั้นระดับนาโนเมตร ทำให้ทำงานที่ความถี่ระดับกิกะเฮิรตซ์ (GHz) ได้โดยมีความหน่วงต่ำมาก ($R C \rightarrow 0$)</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>An IC is not merely a single transistor packaged in plastic; it is a COMPLETE SYSTEM of millions of interconnected transistors, diodes, and resistors.</t>
+          <t>ICs are monolithic (all components created simultaneously on the same crystal substrate), not soldered discrete parts.</t>
         </is>
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
-          <t>ความเข้าใจที่ถูกต้อง: IC ไม่ใช่แค่ทรานซิสเตอร์ตัวเดียว แต่เป็นระบบวงจรอิเล็กทรอนิกส์ทั้งวงจรที่ถูกย่อส่วนลงบนแผ่นชิปซิลิคอน</t>
+          <t>จุดเน้น: IC สร้างขึ้นแบบ Monolithic (ทุกชิ้นส่วนหลอมรวมเป็นเนื้อเดียวบนผลึกซิลิคอน) ไม่ได้เกิดจากการนำอุปกรณ์เดี่ยวมาบัดกรีรวมกัน</t>
         </is>
       </c>
       <c r="N65" s="4" t="inlineStr">
@@ -6574,28 +6701,28 @@
       <c r="I66" s="3" t="inlineStr">
         <is>
           <t>$$V_{\text{knee, Si}} \approx 0.7\text{ V} \qquad V_{\text{knee, Ge}} \approx 0.3\text{ V}$$
-$$\text{Forward: } V_{\text{anode}} &gt; V_{\text{cathode}} + V_{\text{knee}} \implies \text{Conducts heavy current } I_D$$
-$$\text{Reverse: } V_{\text{cathode}} &gt; V_{\text{anode}} \implies I_D \approx I_s \text{ (Reverse Saturation Current } \approx \text{nA)}$$</t>
+$$\text{Forward Bias: } V_{\text{anode}} &gt; V_{\text{cathode}} + V_{\text{knee}} \implies I_D \text{ conducts heavily}$$
+$$\text{Reverse Bias: } V_{\text{cathode}} &gt; V_{\text{anode}} \implies I_D \approx I_s \text{ (Reverse Saturation Current } \approx \text{nA)}$$</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>1. Forward Bias:
-Positive terminal of source connected to Anode (P-type), Negative to Cathode (N-type). When applied voltage exceeds the barrier potential (0.7 V for Si, 0.3 V for Ge), the depletion layer collapses and large forward current flows exponentially.
-2. Reverse Bias:
-Positive terminal to Cathode (N-type), Negative to Anode (P-type). The external voltage widens the depletion layer, preventing majority carrier flow. Only a tiny temperature-dependent reverse saturation current Is (picoamps to nanoamps) flows.
+          <t>1. Forward Bias (ไบแอสตรง):
+Positive supply terminal connected to Anode (P-side), Negative to Cathode (N-side). When applied voltage overcomes the internal barrier potential ($0.7\text{ V}$ for Silicon, $0.3\text{ V}$ for Germanium), the depletion layer collapses and large forward current $I_D$ conducts exponentially.
+2. Reverse Bias (ไบแอสกลับ):
+Positive supply to Cathode (N-side), Negative to Anode (P-side). External voltage widens the depletion barrier, preventing majority carrier transit. Only an ultra-tiny temperature-dependent reverse saturation current $I_s$ (picoamps to nanoamps) leaks through.
 3. Reverse Breakdown:
-If reverse voltage exceeds the Peak Inverse Voltage (PIV / Breakdown Voltage Vz), avalanche multiplication or zener tunneling occurs, causing sudden massive reverse current. Unless current is externally limited by a resistor, the diode will burn out.</t>
+If reverse voltage exceeds Peak Inverse Voltage (PIV), avalanche multiplication causes sudden massive reverse current. Unless current is externally limited by a resistor, the diode burns out instantly.</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
           <t>1. การไบแอสตรง (Forward Bias):
-ต่อขั้วบวกของแหล่งจ่ายเข้ากับแอโนด (P-type) และขั้วลบเข้ากับแคโทด (N-type) เมื่อแรงดันสูงเกินแรงดันคัตอิน (Knee Voltage: 0.7 V สำหรับ Si, 0.3 V สำหรับ Ge) รอยต่อปลอดพาหะ (Depletion Region) จะแคบลงจนยุบตัว ทำให้กระแสไหลผ่านไดโอดได้อย่างสะดวก
+ต่อขั้วบวกเข้ากับแอโนด (P-side) และขั้วลบเข้ากับแคโทด (N-side) เมื่อแรงดันสูงกว่าแรงดันคัตอิน ($0.7\text{ V}$ สำหรับ Silicon, $0.3\text{ V}$ สำหรับ Germanium) รอยต่อปลอดพาหะ (Depletion Region) จะยุบตัวลง ทำให้กระแส $I_D$ ไหลผ่านได้อย่างสะดวก
 2. การไบแอสกลับ (Reverse Bias):
-ต่อขั้วบวกเข้ากับแคโทด (N-type) และขั้วลบเข้ากับแอโนด (P-type) สนามไฟฟ้าภายนอกจะดึงพาหะข้างมากออกจากรอยต่อ ทำให้ชั้นรอยต่อกว้างขึ้น กระแสหลักไม่สามารถไหลผ่านได้ จะมีเพียงกระแสรั่วไหลย้อนกลับเล็กน้อยมาก (Reverse Saturation Current Is ระดับ nA)
+ต่อขั้วบวกเข้ากับแคโทด (N-side) และขั้วลบเข้ากับแอโนด (P-side) สนามไฟฟ้าภายนอกจะดึงพาหะออกจากรอยต่อ ทำให้ชั้นรอยต่อกว้างขึ้น กระแสหลักไม่สามารถไหลได้ จะมีเพียงกระแสรั่วไหลย้อนกลับเล็กน้อยมาก ($I_s$ ระดับ nA)
 3. การพังทลายเมื่อไบแอสกลับ (Breakdown):
-หากป้อนแรงดันย้อนกลับเกินพิกัดทนแรงดันย้อนกลับสูงสุด (PIV) ไดโอดจะเกิดปรากฏการณ์ Avalanche หรือ Zener Breakdown ทำให้กระแสย้อนกลับพุ่งสูงอย่างรวดเร็ว หากไม่มีตัวต้านทานจำกัดกระแส ไดโอดจะไหม้เสียหายทันที</t>
+หากป้อนแรงดันย้อนกลับเกินพิกัดทนแรงดันย้อนกลับสูงสุด (PIV) ไดโอดจะเกิดปรากฏการณ์ Avalanche Breakdown ทำให้กระแสย้อนกลับพุ่งสูงอย่างรวดเร็ว หากไม่มีตัวต้านทานจำกัดกระแส ไดโอดจะไหม้เสียหายทันที</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -6675,28 +6802,32 @@
       <c r="J67" s="5" t="inlineStr">
         <is>
           <t>1. Shockley Diode Equation:
-ID = Is * [exp(VD / (n*VT)) - 1]
-where Is = reverse saturation current, n = ideality factor (1 to 2), VT = thermal voltage = kT/q = 26 mV at room temperature (27°C / 300 K).
-2. Dynamic AC Resistance (rd):
-Taking the derivative dVD/dID yields:
-rd = 26 mV / ID (where ID is in milliamperes).
-At ID = 2 mA, rd = 26 mV / 2 mA = 13 ohms.
-3. LED Resistor Calculation:
-R = (Vcc - V_led) / I_led = (12 V - 2.0 V) / 0.015 A = 10 V / 0.015 A = 666.67 ohms.
-Select standard resistor R = 680 ohms.</t>
+$$I_D = I_s \left( e^{\frac{V_D}{n V_T}} - 1 \right)$$
+where $I_s$ is reverse saturation current, $n$ is ideality factor (1 to 2), and $V_T = kT/q \approx 26\text{ mV}$ at room temperature ($300\text{ K}$).
+2. Dynamic AC Resistance ($r_d$):
+Taking the derivative $d V_D / d I_D$ yields:
+$$r_d = \frac{26\text{ mV}}{I_D}$$
+At $I_D = 2\text{ mA}$:
+$$r_d = \frac{26\text{ mV}}{2\text{ mA}} = 13\;\Omega$$
+3. Calculate LED Series Resistor ($R$):
+Applying KVL around the loop:
+$$R = \frac{V_{CC} - V_{\text{LED}}}{I_{\text{LED}}} = \frac{12\text{ V} - 2.0\text{ V}}{15 \times 10^{-3}\text{ A}} = \frac{10\text{ V}}{0.015\text{ A}} = 666.67\;\Omega$$
+Standard practical resistor value: $680\;\Omega$.</t>
         </is>
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
           <t>1. สมการไดโอดของช็อคลีย์ (Shockley Equation):
-ID = Is * [exp(VD / (n*VT)) - 1]
-โดยที่ Is คือกระแสอิ่มตัวย้อนกลับ, n คือแฟกเตอร์อุดมคติ (1-2), และ VT คือแรงดันความร้อน = kT/q = 26 mV ที่อุณหภูมิห้อง (300 K)
-2. ความต้านทานพลวัต (Dynamic Resistance rd):
-คำนวณจากอนุพันธ์ของเส้นโค้ง I-V: rd = 26 mV / ID
-เช่น ที่กระแส ID = 2 mA จะมี rd = 26 mV / 2 mA = 13 โอห์ม
-3. การคำนวณตัวต้านทานจำกัดกระแส LED:
-R = (Vcc - V_led) / I_led = (12 V - 2.0 V) / 0.015 A = 10 V / 0.015 A = 666.7 โอห์ม
-(ในทางปฏิบัติเลือกใช้ตัวต้านทานค่ามาตรฐาน 680 โอห์ม)</t>
+$$I_D = I_s \left( e^{\frac{V_D}{n V_T}} - 1 \right)$$
+โดยที่ $I_s$ คือกระแสอิ่มตัวย้อนกลับ, $n$ คือแฟกเตอร์อุดมคติ (1-2), และ $V_T = kT/q \approx 26\text{ mV}$ ที่อุณหภูมิห้อง ($300\text{ K}$)
+2. ความต้านทานพลวัต (Dynamic Resistance $r_d$):
+คำนวณจากอนุพันธ์ของเส้นโค้ง I-V:
+$$r_d = \frac{26\text{ mV}}{I_D}$$
+เช่น ที่กระแส $I_D = 2\text{ mA}$ จะได้:
+$$r_d = \frac{26\text{ mV}}{2\text{ mA}} = 13\;\Omega$$
+3. การคำนวณตัวต้านทานจำกัดกระแส LED ($R$):
+$$R = \frac{V_{CC} - V_{\text{LED}}}{I_{\text{LED}}} = \frac{12\text{ V} - 2.0\text{ V}}{15 \times 10^{-3}\text{ A}} = \frac{10\text{ V}}{0.015\text{ A}} = 666.67\;\Omega$$
+(ในทางปฏิบัติเลือกใช้ตัวต้านทานค่ามาตรฐาน $680\;\Omega$)</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
@@ -6762,38 +6893,40 @@
         <is>
           <t>$$I_L = \frac{V_Z}{R_L} = \frac{10\text{ V}}{500\;\Omega} = 20\text{ mA}$$
 $$I_{Z,\max} = \frac{P_{Z,\max}}{V_Z} = \frac{1\text{ W}}{10\text{ V}} = 100\text{ mA}$$
-$$R_{\min} = \frac{V_{\text{in},\max} - V_Z}{I_{Z,\max} + I_L} = \frac{20 - 10}{0.100 + 0.020} = \frac{10}{0.120} = 83.3\;\Omega$$
-$$R_{\max} = \frac{V_{\text{in},\min} - V_Z}{I_{Z,\min} + I_L} = \frac{15 - 10}{0.005 + 0.020} = \frac{5}{0.025} = 200\;\Omega$$</t>
+$$R_{\min} = \frac{V_{\text{in},\max} - V_Z}{I_{Z,\max} + I_L} = \frac{20 - 10}{0.100 + 0.020} = 83.3\;\Omega$$
+$$R_{\max} = \frac{V_{\text{in},\min} - V_Z}{I_{Z,\min} + I_L} = \frac{15 - 10}{0.005 + 0.020} = 200\;\Omega$$</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
           <t>1. Zener Regulation Mechanism:
-A Zener diode operates in the REVERSE breakdown region. When reverse-biased beyond its breakdown voltage Vz, terminal voltage remains remarkably constant at Vz over a broad range of Zener current Iz.
-2. Load Current:
-IL = Vz / RL = 10 V / 500 ohms = 20 mA (constant as long as Vz is regulated).
-3. Maximum Zener Current:
-Iz_max = Pz_max / Vz = 1 W / 10 V = 100 mA.
-4. Calculate Minimum Series Resistance R_min (at Vin_max = 20 V):
-R_min = (Vin_max - Vz) / (Iz_max + IL) = (20 - 10) / (0.100 + 0.020) = 10 / 0.120 = 83.3 ohms.
-5. Calculate Maximum Series Resistance R_max (at Vin_min = 15 V, assuming Iz_min = 5 mA):
-R_max = (Vin_min - Vz) / (Iz_min + IL) = (15 - 10) / (0.005 + 0.020) = 5 / 0.025 = 200 ohms.
-Any value between 84 ohms and 200 ohms (e.g. standard 120 ohms) guarantees stable 10 V regulation.</t>
+A Zener diode operates in the REVERSE breakdown region. When reverse-biased beyond $V_Z$, terminal voltage remains clamped at $V_Z$ over a wide range of reverse current $I_Z$.
+2. Load Current ($I_L$):
+$$I_L = \frac{V_Z}{R_L} = \frac{10\text{ V}}{500\;\Omega} = 20\text{ mA} = 0.020\text{ A}$$
+3. Maximum Zener Current ($I_{Z,\max}$):
+$$I_{Z,\max} = \frac{P_{Z,\max}}{V_Z} = \frac{1\text{ W}}{10\text{ V}} = 100\text{ mA} = 0.100\text{ A}$$
+4. Calculate Minimum Series Resistor ($R_{\min}$):
+To protect the Zener from exceeding maximum power when $V_{\text{in}}$ is highest ($20\text{ V}$):
+$$R_{\min} = \frac{V_{\text{in},\max} - V_Z}{I_{Z,\max} + I_L} = \frac{20\text{ V} - 10\text{ V}}{0.100\text{ A} + 0.020\text{ A}} = \frac{10\text{ V}}{0.120\text{ A}} = 83.3\;\Omega$$
+5. Calculate Maximum Series Resistor ($R_{\max}$):
+To maintain regulation at lowest $V_{\text{in}}$ ($15\text{ V}$) assuming $I_{Z,\min} = 5\text{ mA}$:
+$$R_{\max} = \frac{V_{\text{in},\min} - V_Z}{I_{Z,\min} + I_L} = \frac{15\text{ V} - 10\text{ V}}{0.005\text{ A} + 0.020\text{ A}} = \frac{5\text{ V}}{0.025\text{ A}} = 200\;\Omega$$
+Choose standard resistor $R = 120\;\Omega$ or $150\;\Omega$.</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
           <t>1. กลไกการรักษาระดับแรงดันของซีเนอร์ไดโอด:
-ซีเนอร์ไดโอดถูกออกแบบมาให้ทำงานในย่าน 'ไบแอสกลับ (Reverse Breakdown)' โดยเมื่อแรงดันย้อนกลับถึงค่าแรงดันซีเนอร์ (Vz) แรงดันตกคร่อมตัวมันจะคงที่อยู่ที่ Vz เกือบสมบูรณ์ แม้กระแสที่ไหลผ่านตัวมันจะเปลี่ยนแปลงไปก็ตาม
-2. คำนวณกระแสโหลด IL:
-IL = Vz / RL = 10 V / 500 โอห์ม = 20 mA
-3. คำนวณพิกัดกระแสซีเนอร์สูงสุด Iz_max:
-Iz_max = Pz_max / Vz = 1 W / 10 V = 100 mA (0.1 A)
-4. คำนวณความต้านทานอนุกรมต่ำสุด R_min (ป้องกันซีเนอร์ไหม้เมื่อ Vin สูงสุด 20 V):
-R_min = (Vin_max - Vz) / (Iz_max + IL) = (20 - 10) / (0.100 + 0.020) = 10 / 0.120 = 83.3 โอห์ม
-5. คำนวณความต้านทานอนุกรมสูงสุด R_max (รักษาการคุมแรงดันเมื่อ Vin ต่ำสุด 15 V และ Iz_min = 5 mA):
-R_max = (Vin_min - Vz) / (Iz_min + IL) = (15 - 10) / (0.005 + 0.020) = 5 / 0.025 = 200 โอห์ม
-สรุป: สามารถเลือกใช้ตัวต้านทานค่ามาตรฐานระหว่าง 84 ถึง 200 โอห์ม (เช่น 120 โอห์ม)</t>
+ซีเนอร์ไดโอดทำงานในย่าน 'ไบแอสกลับ (Reverse Breakdown)' โดยเมื่อแรงดันย้อนกลับถึงค่า $V_Z$ แรงดันตกคร่อมตัวมันจะคงที่อยู่ที่ $V_Z$ แม้กระแสจะเปลี่ยนแปลงไป
+2. คำนวณกระแสโหลด $I_L$:
+$$I_L = \frac{V_Z}{R_L} = \frac{10\text{ V}}{500\;\Omega} = 20\text{ mA} = 0.020\text{ A}$$
+3. คำนวณพิกัดกระแสซีเนอร์สูงสุด $I_{Z,\max}$:
+$$I_{Z,\max} = \frac{P_{Z,\max}}{V_Z} = \frac{1\text{ W}}{10\text{ V}} = 100\text{ mA} = 0.100\text{ A}$$
+4. คำนวณความต้านทานอนุกรมต่ำสุด $R_{\min}$ (ป้องกันซีเนอร์ไหม้เมื่อ $V_{\text{in}}$ สูงสุด $20\text{ V}$):
+$$R_{\min} = \frac{V_{\text{in},\max} - V_Z}{I_{Z,\max} + I_L} = \frac{20\text{ V} - 10\text{ V}}{0.100\text{ A} + 0.020\text{ A}} = \frac{10\text{ V}}{0.120\text{ A}} = 83.3\;\Omega$$
+5. คำนวณความต้านทานอนุกรมสูงสุด $R_{\max}$ (รักษาการคุมแรงดันเมื่อ $V_{\text{in}}$ ต่ำสุด $15\text{ V}$ และ $I_{Z,\min} = 5\text{ mA}$):
+$$R_{\max} = \frac{V_{\text{in},\min} - V_Z}{I_{Z,\min} + I_L} = \frac{15\text{ V} - 10\text{ V}}{0.005\text{ A} + 0.020\text{ A}} = \frac{5\text{ V}}{0.025\text{ A}} = 200\;\Omega$$
+สรุป: เลือกใช้ตัวต้านทานค่ามาตรฐานระหว่าง $84\;\Omega$ ถึง $200\;\Omega$ (เช่น $120\;\Omega$ หรือ $150\;\Omega$)</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
@@ -6873,30 +7006,38 @@
       </c>
       <c r="J69" s="5" t="inlineStr">
         <is>
-          <t>1. Solar Cell Equivalent Circuit:
-Consists of a photocurrent source Iph (proportional to solar irradiance) in parallel with:
-- An intrinsic PN junction diode (Shockley equation)
-- A shunt resistance Rsh (representing leakage current across cell edges, ideally infinity)
-- A series resistance Rs (representing bulk silicon and metal contact resistance, ideally zero).
-2. Key Parameters:
-- Short-Circuit Current (Isc): Output current when terminals are shorted (V = 0), almost equal to light-generated current Iph.
-- Open-Circuit Voltage (Voc): Terminal voltage when net current is zero (I = 0), typically ~0.6 V per silicon cell.
-- Maximum Power Point (MPP): The specific point (Vmp, Imp) on the I-V curve where product P = V*I is maximized.
-- Fill Factor (FF): Ratio of actual maximum power to theoretical product (Voc * Isc). Higher FF (typically 0.75 - 0.85) denotes a squarer curve and superior cell quality.</t>
+          <t>1. Solar Cell Equivalent Circuit Components:
+Consists of a light-generated photocurrent source $I_{\text{ph}}$ in parallel with:
+- An intrinsic PN junction diode $D$
+- A shunt resistance $R_{\text{sh}}$ (leakage path across cell edges, ideally $\infty$)
+- A series resistance $R_s$ (bulk silicon and contact resistance, ideally $0$).
+2. Key Parameters Defined:
+- Short-Circuit Current ($I_{sc}$): Current when terminals are shorted ($V = 0$):
+$$I_{sc} \approx I_{\text{ph}}$$
+- Open-Circuit Voltage ($V_{oc}$): Voltage when net current is zero ($I = 0$), typically $\approx 0.6\text{ V}$ per silicon cell.
+- Maximum Power Point ($P_{\max}$): Optimal operating point on the I-V curve:
+$$P_{\max} = V_{\text{mp}} \cdot I_{\text{mp}}$$
+- Fill Factor ($FF$): Ratio of peak power to theoretical product ($V_{oc} I_{sc}$):
+$$FF = \frac{V_{\text{mp}} I_{\text{mp}}}{V_{oc} I_{sc}}$$
+Typically ranges from $0.75$ to $0.85$ for high-quality commercial silicon cells.</t>
         </is>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t>1. วงจรสมมูลของโซลาร์เซลล์:
-ประกอบด้วยแหล่งจ่ายกระแสที่เกิดจากแสง Iph (แปรผันตามความเข้มแสงแดด) ต่อขนานกับ:
-- ตัวไดโอดรอยต่อ PN แท้จริง (Diode D)
-- ความต้านทานขนาน Rsh (แทนการรั่วไหลของกระแสตามขอบเซลล์ ในอุดมคติมีค่าเป็นอนันต์)
-- ความต้านทานอนุกรม Rs (แทนความต้านทานเนื้อซิลิคอนและขั้วโลหะ ในอุดมคติมีค่าเป็นศูนย์)
+          <t>1. องค์ประกอบวงจรสมมูลของโซลาร์เซลล์:
+ประกอบด้วยแหล่งจ่ายกระแสโฟโต $I_{\text{ph}}$ (แปรผันตามแสงแดด) ต่อขนานกับ:
+- ตัวไดโอดรอยต่อ PN แท้จริง (Diode $D$)
+- ความต้านทานขนาน $R_{\text{sh}}$ (แทนกระแสรั่วไหลตามขอบเซลล์ ในอุดมคติมีค่าเป็นอนันต์)
+- ความต้านทานอนุกรม $R_s$ (แทนความต้านทานเนื้อซิลิคอนและขั้วโลหะ ในอุดมคติมีค่าเป็นศูนย์)
 2. พารามิเตอร์สำคัญของเซลล์แสงอาทิตย์:
-- กระแสลัดวงจร (Short-Circuit Current: Isc): กระแสที่ไหลเมื่อต่อลัดวงจรขั้วเซลล์ (V = 0) มีค่าใกล้เคียงกระแสโฟโต Iph
-- แรงดันเปิดวงจร (Open-Circuit Voltage: Voc): แรงดันที่วัดได้เมื่อเปิดวงจร (I = 0) มีค่าประมาณ 0.6 V ต่อเซลล์ซิลิคอน 1 เซลล์
-- จุดทำงานกำลังสูงสุด (Maximum Power Point: MPP): จุดบนกราฟ I-V Curve ที่ให้ผลคูณ P = Vmp * Imp สูงที่สุด
-- ฟิลแฟกเตอร์ (Fill Factor: FF): อัตราส่วนระหว่างกำลังไฟฟ้าสูงสุดจริง ต่อ ผลคูณเชิงทฤษฎี (Voc * Isc) ยิ่งค่า FF สูง (0.75 - 0.85) กราฟจะยิ่งเป็นรูปสี่เหลี่ยม แสดงว่าเซลล์มีคุณภาพสูง</t>
+- กระแสลัดวงจร ($I_{sc}$): กระแสเมื่อลัดวงจรขั้วเซลล์ ($V = 0$):
+$$I_{sc} \approx I_{\text{ph}}$$
+- แรงดันเปิดวงจร ($V_{oc}$): แรงดันเมื่อเปิดวงจร ($I = 0$) มีค่าประมาณ $0.6\text{ V}$ ต่อเซลล์
+- จุดกำลังสูงสุด ($P_{\max}$): จุดที่ให้ผลคูณแรงดันและกระแสสูงสุด:
+$$P_{\max} = V_{\text{mp}} \cdot I_{\text{mp}}$$
+- ฟิลแฟกเตอร์ ($FF$): อัตราส่วนกำลังจริงต่อผลคูณเชิงทฤษฎี ($V_{oc} I_{sc}$):
+$$FF = \frac{V_{\text{mp}} I_{\text{mp}}}{V_{oc} I_{sc}}$$
+เซลล์คุณภาพสูงจะมีค่า $FF \approx 0.75 - 0.85$</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
@@ -6968,37 +7109,37 @@
       <c r="J70" s="3" t="inlineStr">
         <is>
           <t>1. Kirchhoff's Current Law for BJT:
-By KCL, the total current leaving/entering the emitter equals the sum of base and collector currents:
-IE = IB + IC
-2. Current Gains Defined:
-- Common-Emitter DC Current Gain (Beta or hFE):
-Beta = IC / IB (typically ranges from 50 to 300).
-- Common-Base DC Current Gain (Alpha):
-Alpha = IC / IE (slightly less than 1, typically 0.98 to 0.998).
-3. Relationship Derivation:
-Divide IE = IB + IC by IC:
-IE / IC = (IB / IC) + 1
-1 / Alpha = (1 / Beta) + 1 = (Beta + 1) / Beta
-Inverting yields: Alpha = Beta / (Beta + 1)
-Solving for Beta yields: Beta = Alpha / (1 - Alpha).</t>
+By KCL, total current passing through the emitter equals the sum of base and collector currents:
+$$I_E = I_B + I_C$$
+2. DC Current Gains Defined:
+- Common-Emitter Gain ($\beta$ or $h_{FE}$):
+$$\beta = \frac{I_C}{I_B} \quad (\text{typically } 50 - 300)$$
+- Common-Base Gain ($\alpha$):
+$$\alpha = \frac{I_C}{I_E} \quad (\text{slightly less than 1, typically } 0.98 - 0.998)$$
+3. Mathematical Relationship Derivation:
+Dividing $I_E = I_B + I_C$ by $I_C$:
+$$\frac{I_E}{I_C} = \frac{I_B}{I_C} + 1$$
+$$\frac{1}{\alpha} = \frac{1}{\beta} + 1 = \frac{\beta + 1}{\beta}$$
+Inverting yields:
+$$\alpha = \frac{\beta}{\beta + 1} \qquad \beta = \frac{\alpha}{1 - \alpha}$$</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
           <t>1. กฎกระแสเคอร์ชอฟฟ์ของทรานซิสเตอร์ BJT:
 กระแสที่ไหลผ่านขาอิมิตเตอร์มีค่าเท่ากับผลรวมของกระแสขาเบสและขาคอลเลกเตอร์เสมอ:
-IE = IB + IC
+$$I_E = I_B + I_C$$
 2. นิยามอัตราขยายกระแส:
-- อัตราขยายกระแสแบบคอมมอนอิมิตเตอร์ (Beta หรือ hFE):
-Beta = IC / IB (ค่าทั่วไปอยู่ในช่วง 50 ถึง 300 เท่า)
-- อัตราขยายกระแสแบบคอมมอนเบส (Alpha):
-Alpha = IC / IE (มีค่าน้อยกว่า 1 เล็กน้อย ค่าทั่วไปประมาณ 0.98 ถึง 0.998)
-3. การพิสูจน์ความสัมพันธ์ระหว่าง Alpha และ Beta:
-จาก IE = IB + IC นำ IC มาหารตลอด:
-IE / IC = (IB / IC) + 1
-1 / Alpha = (1 / Beta) + 1 = (Beta + 1) / Beta
-กลับเศษส่วนจะได้: Alpha = Beta / (Beta + 1)
-หรือแปลงรูปหาค่า Beta: Beta = Alpha / (1 - Alpha)</t>
+- อัตราขยายกระแสคอมมอนอิมิตเตอร์ ($\beta$ หรือ $h_{FE}$):
+$$\beta = \frac{I_C}{I_B} \quad (\text{ค่าทั่วไปอยู่ในช่วง } 50 - 300)$$
+- อัตราขยายกระแสคอมมอนเบส ($\alpha$):
+$$\alpha = \frac{I_C}{I_E} \quad (\text{มีค่าน้อยกว่า 1 เล็กน้อย ประมาณ } 0.98 - 0.998)$$
+3. การพิสูจน์ความสัมพันธ์ระหว่าง $\alpha$ และ $\beta$:
+จาก $I_E = I_B + I_C$ นำ $I_C$ มาหารตลอด:
+$$\frac{I_E}{I_C} = \frac{I_B}{I_C} + 1$$
+$$\frac{1}{\alpha} = \frac{1}{\beta} + 1 = \frac{\beta + 1}{\beta}$$
+กลับเศษส่วนจะได้:
+$$\alpha = \frac{\beta}{\beta + 1} \qquad \beta = \frac{\alpha}{1 - \alpha}$$</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
@@ -7070,38 +7211,38 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>$$\text{Cutoff (OFF): } V_{in} = 0 \implies I_B = 0, \; I_C = 0, \; V_{CE} = V_{CC}$$
+          <t>$$\text{Cutoff (OFF): } V_{\text{in}} = 0 \implies I_B = 0, \; I_C = 0, \; V_{CE} = V_{CC}$$
 $$\text{Saturation (ON): } I_B \ge \frac{I_{C,\text{sat}}}{\beta_{\text{sat}}} \implies V_{CE} = V_{CE,\text{sat}} \approx 0.2\text{ V}$$
 $$I_{C,\text{sat}} = \frac{V_{CC} - V_{CE,\text{sat}}}{R_{\text{load}}}$$
-$$R_B = \frac{V_{in} - V_{BE,\text{sat}}}{I_B}$$</t>
+$$R_B = \frac{V_{\text{in}} - V_{BE,\text{sat}}}{I_B}$$</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
           <t>1. Operating States as a Switch:
-- Cutoff (Switch OFF): When Vin = 0 V, Vbe &lt; 0.7 V. Base current IB = 0, Collector current IC = 0. The transistor behaves as an open switch; full supply Vcc appears across C-E.
-- Saturation (Switch ON): Sufficient base current IB is injected so both B-E and B-C junctions become forward-biased. Vce collapses to Vce(sat) ~ 0.2 V. The transistor acts as a closed switch, passing full load current.
+- Cutoff (Switch OFF): When $V_{\text{in}} = 0\text{ V}$ ($V_{BE} &lt; 0.7\text{ V}$), base current $I_B = 0$ and collector current $I_C = 0$. The transistor behaves as an open switch ($V_{CE} = V_{CC}$).
+- Saturation (Switch ON): Ample base current $I_B$ forward-biases both B-E and B-C junctions. $V_{CE}$ drops to $V_{CE,\text{sat}} \approx 0.2\text{ V}$, acting as a closed contact.
 2. Base Resistor Calculation:
-- Target load current: IC_sat = 100 mA = 0.1 A.
-- Overdrive base current for hard saturation (using forced Beta = 10):
-IB = IC_sat / Beta_sat = 100 mA / 10 = 10 mA.
-- Calculate RB:
-RB = (Vin - Vbe_sat) / IB = (5.0 V - 0.7 V) / (10 x 10^-3 A) = 4.3 V / 0.010 A = 430 ohms.
-(Select standard 430 ohms or 390 ohms for robust saturation).</t>
+- Required collector load current: $I_{C,\text{sat}} = 100\text{ mA} = 0.100\text{ A}$.
+- Required base current for deep saturation (using forced $\beta_{\text{sat}} = 10$):
+$$I_B = \frac{I_{C,\text{sat}}}{\beta_{\text{sat}}} = \frac{100\text{ mA}}{10} = 10\text{ mA} = 0.010\text{ A}$$
+- Calculate base resistor $R_B$:
+$$R_B = \frac{V_{\text{in}} - V_{BE,\text{sat}}}{I_B} = \frac{5.0\text{ V} - 0.7\text{ V}}{0.010\text{ A}} = \frac{4.3\text{ V}}{0.010\text{ A}} = 430\;\Omega$$
+Standard practical resistor: $430\;\Omega$ or $390\;\Omega$.</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
           <t>1. สภาวะการทำงานเป็นสวิตช์:
-- สภาวะคัตออฟ (Cutoff - สวิตช์เปิด/OFF): เมื่อป้อน Vin = 0 V (Vbe &lt; 0.7 V) จะไม่มีกระแสเบส IB = 0 ทำให้ IC = 0 ทรานซิสเตอร์ทำตัวเหมือนสวิตช์เปิดวงจร แรงดัน Vce เท่ากับ Vcc เต็มที่
-- สภาวะอิ่มตัว (Saturation - สวิตช์ปิด/ON): ป้อนกระแสเบส IB มากเพียงพอจนรอยต่อทั้งสองได้รับไบแอสตรง แรงดันตกคร่อม Vce จะลดฮวบลงเหลือ Vce(sat) เพียงประมาณ 0.2 V ทรานซิสเตอร์ทำตัวเหมือนสวิตช์ลัดวงจร จ่ายกระแสโหลดเต็มที่
-2. การคำนวณค่าตัวต้านทานขาเบส RB:
-- กระแสโหลดคอลเลกเตอร์ที่ต้องการ: IC_sat = 100 mA
-- คำนวณกระแสเบสเพื่อให้เข้าสู่ภาวะอิ่มตัวอย่างสมบูรณ์ (Overdrive โดยใช้ Forced Beta = 10):
-IB = IC_sat / Beta_sat = 100 mA / 10 = 10 mA
-- คำนวณค่า RB:
-RB = (Vin - Vbe_sat) / IB = (5.0 V - 0.7 V) / 0.010 A = 4.3 V / 0.010 A = 430 โอห์ม
-(ในทางปฏิบัติเลือกใช้ตัวต้านทานมาตรฐาน 430 โอห์ม หรือ 390 โอห์ม)</t>
+- สภาวะคัตออฟ (Cutoff - สวิตช์เปิด/OFF): เมื่อ $V_{\text{in}} = 0\text{ V}$ ($V_{BE} &lt; 0.7\text{ V}$) ไม่มีกระแสเบส $I_B = 0$ ทำให้ $I_C = 0$ ทรานซิสเตอร์ทำตัวเหมือนสวิตช์เปิดวงจร แรงดัน $V_{CE} = V_{CC}$
+- สภาวะอิ่มตัว (Saturation - สวิตช์ปิด/ON): ป้อนกระแสเบส $I_B$ มากพอจนรอยต่อทั้งสองได้รับไบแอสตรง แรงดันตกคร่อมลดลงเหลือ $V_{CE,\text{sat}} \approx 0.2\text{ V}$ ทำตัวเหมือนสวิตช์ลัดวงจร
+2. การคำนวณค่าตัวต้านทานขาเบส $R_B$:
+- กระแสโหลดคอลเลกเตอร์ที่ต้องการ: $I_{C,\text{sat}} = 100\text{ mA} = 0.100\text{ A}$
+- คำนวณกระแสเบสสำหรับภาวะอิ่มตัว (ใช้ Forced $\beta_{\text{sat}} = 10$):
+$$I_B = \frac{I_{C,\text{sat}}}{\beta_{\text{sat}}} = \frac{100\text{ mA}}{10} = 10\text{ mA} = 0.010\text{ A}$$
+- คำนวณค่า $R_B$:
+$$R_B = \frac{V_{\text{in}} - V_{BE,\text{sat}}}{I_B} = \frac{5.0\text{ V} - 0.7\text{ V}}{0.010\text{ A}} = \frac{4.3\text{ V}}{0.010\text{ A}} = 430\;\Omega$$
+(ในทางปฏิบัติเลือกใช้ตัวต้านทานค่ามาตรฐาน $430\;\Omega$ หรือ $390\;\Omega$)</t>
         </is>
       </c>
       <c r="L71" s="5" t="inlineStr">
@@ -7140,7 +7281,7 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>ตารางเปรียบเทียบเชิงลึก BJT vs FET / MOSFET</t>
+          <t>ตารางเปรียบเทียบเชิงลึก BJT vs FET / MOSFET (ข้อสอบไฟนอล 4.2)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -7173,34 +7314,34 @@
         <is>
           <t>Comprehensive Comparison:
 1. Carrier Conduction:
-- BJT is BIPOLAR (current conduction involves both electrons and holes).
+- BJT is BIPOLAR (current conduction involves both electrons and holes simultaneously).
 - MOSFET is UNIPOLAR (current conduction relies strictly on majority carriers in the channel).
 2. Control Mechanism:
-- BJT is CURRENT-CONTROLLED: Output current IC is controlled by input base current IB (IC = Beta * IB).
-- MOSFET is VOLTAGE-CONTROLLED: Output drain current ID is controlled by gate-to-source voltage VGS.
-3. Input Impedance:
-- BJT: Low to moderate input impedance (1 k-ohm to 10 k-ohms) because the base-emitter junction is forward-biased.
-- MOSFET: Near-infinite input impedance (10^12 to 10^14 ohms) due to the insulating silicon dioxide gate dielectric.
+- BJT is CURRENT-CONTROLLED: Output collector current $I_C$ is controlled by input base current $I_B$ ($I_C = \beta I_B$).
+- MOSFET is VOLTAGE-CONTROLLED: Output drain current $I_D$ is controlled by gate-to-source voltage $V_{GS}$.
+3. Input Impedance ($R_{\text{in}}$):
+- BJT: Moderate ($1\text{ k}\Omega - 10\text{ k}\Omega$) because the B-E junction is forward-biased.
+- MOSFET: Near-infinite ($10^{12} - 10^{14}\,\Omega$) due to the insulating $SiO_2$ gate dielectric.
 4. Thermal Stability:
-- BJT has negative temperature coefficient for Vbe, making it vulnerable to Thermal Runaway.
-- MOSFET has positive temperature coefficient for RDS(on), naturally preventing thermal runaway and allowing easy parallel operation.</t>
+- BJT has negative temperature coefficient for $V_{BE}$, making it vulnerable to Thermal Runaway.
+- MOSFET has positive temperature coefficient for $R_{DS(\text{on})}$, preventing thermal runaway.</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>ตารางเปรียบเทียบ BJT vs MOSFET:
+          <t>ตารางเปรียบเทียบเชิงลึก BJT vs MOSFET:
 1. ชนิดของพาหะที่นำกระแส:
 - BJT: เป็นแบบ 'Bipolar' คือใช้ทั้งอิเล็กตรอนและโฮลในการนำกระแสพร้อมกัน
 - MOSFET: เป็นแบบ 'Unipolar' คือใช้เฉพาะพาหะข้างมากชนิดเดียวในแชนแนลในการนำกระแส
 2. กลไกการควบคุม:
-- BJT: ควบคุมด้วยกระแส (Current-Controlled) โดยกระแสขาเข้า IB เป็นตัวกำหนดกระแสขาออก IC (IC = Beta * IB)
-- MOSFET: ควบคุมด้วยแรงดัน (Voltage-Controlled) โดยแรงดัน VGS เป็นตัวกำหนดกระแสขาออก ID
+- BJT: ควบคุมด้วยกระแส (Current-Controlled) โดยกระแสขาเข้า $I_B$ กำหนดกระแสขาออก $I_C = \beta I_B$
+- MOSFET: ควบคุมด้วยแรงดัน (Voltage-Controlled) โดยแรงดัน $V_{GS}$ กำหนดกระแสขาออก $I_D$
 3. อิมพีแดนซ์ขาเข้า (Input Impedance):
-- BJT: ปานกลาง (1 k-ohm ถึง 10 k-ohm) เพราะรอยต่อ B-E ได้รับไบแอสตรง
-- MOSFET: สูงมากเกือบเป็นอนันต์ (10^12 ถึง 10^14 โอห์ม) เพราะมีชั้นฉนวน SiO2 กั้นขาเกตไว้
+- BJT: ปานกลาง ($1\text{ k}\Omega - 10\text{ k}\Omega$) เพราะรอยต่อ B-E ได้รับไบแอสตรง
+- MOSFET: สูงมากเกือบเป็นอนันต์ ($10^{12} - 10^{14}\,\Omega$) เพราะมีชั้นฉนวน $SiO_2$ กั้นขาเกต
 4. เสถียรภาพทางอุณหภูมิ (Thermal Stability):
-- BJT: มีสัมประสิทธิ์อุณหภูมิเป็นลบ เกิดปรากฏการณ์ Thermal Runaway (ยิ่งร้อนยิ่งกินกระแสจนไหม้) ได้ง่าย
-- MOSFET: มีสัมประสิทธิ์อุณหภูมิของ RDS(on) เป็นบวก เมื่อร้อนความต้านทานจะเพิ่มขึ้น ช่วยป้องกันความเสียหายและต่อขนานกันได้ง่าย</t>
+- BJT: มีสัมประสิทธิ์อุณหภูมิเป็นลบ เกิดปรากฏการณ์ Thermal Runaway ได้ง่าย
+- MOSFET: มีสัมประสิทธิ์อุณหภูมิของ $R_{DS(\text{on})}$ เป็นบวก ช่วยป้องกันความเสียหายและต่อขนานกันได้ง่าย</t>
         </is>
       </c>
       <c r="L72" s="3" t="inlineStr">
@@ -7272,47 +7413,47 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>$$\text{Half-Wave: } V_{\text{dc}} = \frac{V_m}{\pi} = 0.318\, V_m \qquad f_{\text{ripple}} = f_{\text{in}} \qquad \text{PIV} = V_m$$
-$$\text{Center-Tapped: } V_{\text{dc}} = \frac{2V_m}{\pi} = 0.637\, V_m \qquad f_{\text{ripple}} = 2f_{\text{in}} \qquad \text{PIV} = 2V_m$$
-$$\text{Bridge Rectifier: } V_{\text{dc}} = \frac{2V_m}{\pi} = 0.637\, V_m \qquad f_{\text{ripple}} = 2f_{\text{in}} \qquad \text{PIV} = V_m$$</t>
+          <t>$$\text{Half-Wave: } V_{\text{dc}} = \frac{V_m}{\pi} \approx 0.318\, V_m \qquad f_{\text{ripple}} = f_{\text{in}} \qquad \text{PIV} = V_m$$
+$$\text{Center-Tapped: } V_{\text{dc}} = \frac{2V_m}{\pi} \approx 0.637\, V_m \qquad f_{\text{ripple}} = 2f_{\text{in}} \qquad \text{PIV} = 2V_m$$
+$$\text{Bridge Rectifier: } V_{\text{dc}} = \frac{2V_m}{\pi} \approx 0.637\, V_m \qquad f_{\text{ripple}} = 2f_{\text{in}} \qquad \text{PIV} = V_m$$</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
           <t>1. Half-Wave Rectifier (1 Diode):
-- Vdc = Vm / pi = 0.318 Vm
-- Ripple frequency = fin (50 Hz)
-- Maximum theoretical efficiency = 40.6%
-- Diode PIV = Vm
-2. Center-Tapped Full-Wave Rectifier (2 Diodes + Center-Tapped Transformer):
-- Vdc = 2*Vm / pi = 0.637 Vm
-- Ripple frequency = 2*fin (100 Hz, easier to filter)
-- Maximum theoretical efficiency = 81.2%
-- Diode PIV = 2*Vm (Major drawback: diodes must withstand twice peak voltage!)
-3. Bridge Full-Wave Rectifier (4 Diodes, Standard Transformer):
-- Vdc = 2*Vm / pi = 0.637 Vm
-- Ripple frequency = 2*fin (100 Hz)
-- Maximum theoretical efficiency = 81.2%
-- Diode PIV = Vm (Only 1*Vm, allowing lower-voltage diodes; dominant industry standard).</t>
+- DC Average Voltage: $V_{\text{dc}} = V_m / \pi = 0.318\, V_m$
+- Ripple frequency: $f_{\text{ripple}} = f_{\text{in}}$ (50 Hz)
+- Maximum theoretical efficiency: $40.6\%$
+- Diode PIV: $\text{PIV} = V_m$
+2. Center-Tapped Full-Wave Rectifier (2 Diodes):
+- DC Average Voltage: $V_{\text{dc}} = 2V_m / \pi = 0.637\, V_m$
+- Ripple frequency: $f_{\text{ripple}} = 2f_{\text{in}}$ (100 Hz, easier to filter)
+- Maximum theoretical efficiency: $81.2\%$
+- Diode PIV: $\text{PIV} = 2V_m$ (Major drawback: diodes must withstand twice peak voltage!)
+3. Bridge Full-Wave Rectifier (4 Diodes):
+- DC Average Voltage: $V_{\text{dc}} = 2V_m / \pi = 0.637\, V_m$
+- Ripple frequency: $f_{\text{ripple}} = 2f_{\text{in}}$ (100 Hz)
+- Maximum theoretical efficiency: $81.2\%$
+- Diode PIV: $\text{PIV} = V_m$ (Dominant industry standard).</t>
         </is>
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
           <t>1. วงจรเรียงกระแสแบบครึ่งคลื่น (Half-Wave - ใช้ไดโอด 1 ตัว):
-- แรงดันไฟตรงเฉลี่ย: Vdc = Vm / pi = 0.318 Vm
-- ความถี่ริปเปิล: เท่ากับความถี่ไฟเข้า = fin (50 Hz)
-- ประสิทธิภาพสูงสุด: 40.6%
-- พิกัดทนแรงดันย้อนกลับไดโอด: PIV = Vm
+- แรงดันไฟตรงเฉลี่ย: $V_{\text{dc}} = V_m / \pi = 0.318\, V_m$
+- ความถี่ริปเปิล: $f_{\text{ripple}} = f_{\text{in}}$ (50 Hz)
+- ประสิทธิภาพสูงสุด: $40.6\%$
+- พิกัดทนแรงดันย้อนกลับไดโอด: $\text{PIV} = V_m$
 2. วงจรเต็มคลื่นแบบหม้อแปลงมีแท็ปกลาง (Center-Tapped - ใช้ไดโอด 2 ตัว):
-- แรงดันไฟตรงเฉลี่ย: Vdc = 2*Vm / pi = 0.637 Vm
-- ความถี่ริปเปิล: 2 เท่าของไฟเข้า = 2*fin (100 Hz กรองให้เรียบง่ายขึ้นมาก)
-- ประสิทธิภาพสูงสุด: 81.2%
-- พิกัดทนแรงดันย้อนกลับไดโอด: PIV = 2*Vm (ข้อเสียสำคัญ: ไดโอดต้องทนแรงดันย้อนกลับสูงถึง 2 เท่าของแรงดันพีก)
+- แรงดันไฟตรงเฉลี่ย: $V_{\text{dc}} = 2V_m / \pi = 0.637\, V_m$
+- ความถี่ริปเปิล: $f_{\text{ripple}} = 2f_{\text{in}}$ (100 Hz กรองให้เรียบง่ายขึ้นมาก)
+- ประสิทธิภาพสูงสุด: $81.2\%$
+- พิกัดทนแรงดันย้อนกลับไดโอด: $\text{PIV} = 2V_m$ (ข้อเสียสำคัญ: ไดโอดต้องทนแรงดันย้อนกลับสูงถึง 2 เท่าของแรงดันพีก)
 3. วงจรเต็มคลื่นแบบบริดจ์ (Bridge Rectifier - ใช้ไดโอด 4 ตัว):
-- แรงดันไฟตรงเฉลี่ย: Vdc = 2*Vm / pi = 0.637 Vm
-- ความถี่ริปเปิล: 2*fin (100 Hz)
-- ประสิทธิภาพสูงสุด: 81.2%
-- พิกัดทนแรงดันย้อนกลับไดโอด: PIV = Vm (ไดโอดรับแรงดันย้อนกลับเพียง 1 เท่า นิยมใช้มากที่สุดในอุตสาหกรรม)</t>
+- แรงดันไฟตรงเฉลี่ย: $V_{\text{dc}} = 2V_m / \pi = 0.637\, V_m$
+- ความถี่ริปเปิล: $f_{\text{ripple}} = 2f_{\text{in}}$ (100 Hz)
+- ประสิทธิภาพสูงสุด: $81.2\%$
+- พิกัดทนแรงดันย้อนกลับไดโอด: $\text{PIV} = V_m$ (ไดโอดรับแรงดันย้อนกลับเพียง 1 เท่า นิยมใช้มากที่สุดในอุตสาหกรรม)</t>
         </is>
       </c>
       <c r="L73" s="5" t="inlineStr">
@@ -7385,30 +7526,29 @@
       <c r="J74" s="3" t="inlineStr">
         <is>
           <t>1. Ideal Op-Amp Characteristics:
-- Input Impedance (Rin): Infinite (no current enters the input terminals: I+ = I- = 0).
-- Output Impedance (Rout): Zero (can supply any load current without internal voltage drop).
-- Open-Loop Voltage Gain (A_OL): Infinite.
-- Bandwidth (BW): Infinite (amplifies signals from DC to infinite frequency without attenuation).
-- Slew Rate: Infinite (output changes voltage instantaneously).
-- Common-Mode Rejection Ratio (CMRR): Infinite.
+- Input Impedance ($R_{\text{in}}$): Infinite ($I_+ = I_- = 0$).
+- Output Impedance ($R_{\text{out}}$): Zero (supplies load without drop).
+- Open-Loop Gain ($A_{OL}$): Infinite ($10^5 - 10^6$ in real chips).
+- Bandwidth ($BW$): Infinite (flat response from DC to $\infty$).
+- Slew Rate: Infinite (instantaneous output slew).
 2. Virtual Short &amp; Virtual Ground:
-Because open-loop gain A_OL is infinite, in any negative feedback configuration, the differential input voltage MUST be zero:
-(V+ - V-) = Vout / A_OL = Vout / infinity = 0  =&gt;  V+ = V-.
-This is called a 'Virtual Short'. If the non-inverting terminal V+ is tied to physical ground (0 V), then V- is held firmly at 0 V without being physically connected to ground, known as 'Virtual Ground'.</t>
+Because open-loop gain $A_{OL}$ is infinite, in any closed-loop negative feedback configuration, the differential input voltage must be zero:
+$$V_+ - V_- = \frac{V_{\text{out}}}{A_{OL}} = \frac{V_{\text{out}}}{\infty} = 0 \implies V_+ = V_-$$
+This condition is known as a Virtual Short. If the non-inverting terminal $V_+$ is connected to physical ground ($0\text{ V}$), then $V_-$ is held at zero volts without being physically grounded, known as Virtual Ground.</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
           <t>1. คุณสมบัติในอุดมคติของออปแอมป์ (Ideal Op-Amp):
-- ความต้านทานขาเข้า (Input Impedance: Rin) = อินฟินิตี้ (ไม่มีกระแสไหลเข้าขาอินพุต: I+ = I- = 0)
-- ความต้านทานขาออก (Output Impedance: Rout) = 0 โอห์ม (จ่ายกระแสโหลดได้ไม่จำกัดโดยแรงดันไม่ตก)
-- อัตราขยายแรงดันวงเปิด (Open-Loop Gain: A_OL) = อินฟินิตี้
-- แบนด์วิดท์ (Bandwidth: BW) = อินฟินิตี้ (ขยายสัญญาณได้ทุกความถี่ตั้งแต่ DC ถึงไม่สิ้นสุด)
-- สลูว์เรต (Slew Rate) = อินฟินิตี้ (แรงดันขาออกตอบสนองได้ทันทีโดยไม่มีความหน่วง)
+- ความต้านทานขาเข้า ($R_{\text{in}}$) = $\infty$ (ไม่มีกระแสไหลเข้าขาอินพุต: $I_+ = I_- = 0$)
+- ความต้านทานขาออก ($R_{\text{out}}$) = $0\;\Omega$ (จ่ายกระแสโหลดได้ไม่จำกัดโดยแรงดันไม่ตก)
+- อัตราขยายแรงดันวงเปิด ($A_{OL}$) = $\infty$
+- แบนด์วิดท์ ($BW$) = $\infty$ (ขยายสัญญาณได้ทุกความถี่ตั้งแต่ DC ถึงไม่สิ้นสุด)
+- สลูว์เรต (Slew Rate) = $\infty$ (แรงดันขาออกตอบสนองได้ทันทีโดยไม่มีความหน่วง)
 2. แนวคิดช็อตเสมือน (Virtual Short) และกราวด์เสมือน (Virtual Ground):
-เนื่องจากอัตราขยาย A_OL เป็นอนันต์ เมื่อมีการต่อป้อนกลับแบบลบ (Negative Feedback) ผลต่างแรงดันระหว่างขาอินพุตทั้งสองต้องมีค่าเป็นศูนย์:
-(V+ - V-) = Vout / A_OL = 0  =&gt;  V+ = V-
-สภาวะนี้เรียกว่า 'Virtual Short' และหากขา V+ ต่อลงกราวด์จริง (0 V) ขา V- ก็จะมีศักย์ไฟฟ้าเท่ากับ 0 V เสมือนต่อลงกราวด์ด้วย เรียกว่า 'Virtual Ground'</t>
+เนื่องจากอัตราขยาย $A_{OL}$ เป็นอนันต์ เมื่อมีการต่อป้อนกลับแบบลบ (Negative Feedback) ผลต่างแรงดันระหว่างขาอินพุตทั้งสองต้องมีค่าเป็นศูนย์:
+$$V_+ - V_- = \frac{V_{\text{out}}}{A_{OL}} = 0 \implies V_+ = V_-$$
+สภาวะนี้เรียกว่า 'Virtual Short' และหากขา $V_+$ ต่อลงกราวด์จริง ($0\text{ V}$) ขา $V_-$ ก็จะมีศักย์ไฟฟ้าเท่ากับ $0\text{ V}$ เสมือนต่อลงกราวด์ด้วย เรียกว่า 'Virtual Ground'</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix: resolve KaTeX square root radical stretching and refine 3-phase equations
</commit_message>
<xml_diff>
--- a/FunE_Master_Exam_Flashcards_Ch6_10_Master.xlsx
+++ b/FunE_Master_Exam_Flashcards_Ch6_10_Master.xlsx
@@ -616,28 +616,36 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Y: $V_L = \sqrt{3}V_p\angle +30^\circ,\ I_L = I_p$
-$\Delta$: $V_L = V_p,\ I_L = \sqrt{3}I_p\angle -30^\circ$</t>
+          <t>$$\text{Star (Y): } V_L = \sqrt{3}\, V_p \angle +30^\circ, \quad I_L = I_p$$
+$$\text{Delta (}\Delta\text{): } V_L = V_p, \quad I_L = \sqrt{3}\, I_p \angle -30^\circ$$</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1. Star (Y) Connection:
-- Line Voltage leads Phase Voltage by $30^\circ$: $V_{ab} = \sqrt{3}V_{an}\angle +30^\circ$
-- Line Current equals Phase Current: $I_L = I_p$
+- Line Voltage leads Phase Voltage by $30^\circ$:
+$$V_{ab} = \sqrt{3}\, V_{an} \angle +30^\circ$$
+- Line Current equals Phase Current:
+$$I_L = I_p$$
 2. Delta (Δ) Connection:
-- Line Voltage equals Phase Voltage: $V_L = V_p$
-- Line Current lags Phase Current by $30^\circ$: $I_a = \sqrt{3}I_{ab}\angle -30^\circ$</t>
+- Line Voltage equals Phase Voltage:
+$$V_L = V_p$$
+- Line Current lags Phase Current by $30^\circ$:
+$$I_a = \sqrt{3}\, I_{ab} \angle -30^\circ$$</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>1. การต่อแบบ Star (Y):
-- Line Voltage นำหน้า (leads) Phase Voltage อยู่ $30^\circ$: $V_{ab} = \sqrt{3}V_{an}\angle +30^\circ$
-- Line Current เท่ากับ Phase Current โดยตรง: $I_L = I_p$
+- Line Voltage นำหน้า (leads) Phase Voltage อยู่ $30^\circ$:
+$$V_{ab} = \sqrt{3}\, V_{an} \angle +30^\circ$$
+- Line Current เท่ากับ Phase Current โดยตรง:
+$$I_L = I_p$$
 2. การต่อแบบ Delta (Δ):
-- Line Voltage เท่ากับ Phase Voltage โดยตรง: $V_L = V_p$
-- Line Current ตามหลัง (lags) Phase Current อยู่ $30^\circ$: $I_a = \sqrt{3}I_{ab}\angle -30^\circ$</t>
+- Line Voltage เท่ากับ Phase Voltage โดยตรง:
+$$V_L = V_p$$
+- Line Current ตามหลัง (lags) Phase Current อยู่ $30^\circ$:
+$$I_a = \sqrt{3}\, I_{ab} \angle -30^\circ$$</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">

</xml_diff>